<commit_message>
Update for week of Aug 17 command board
</commit_message>
<xml_diff>
--- a/data/2026 Bowler Chart - OFS Training.xlsx
+++ b/data/2026 Bowler Chart - OFS Training.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\212668250\Box\OFS Global Technical Training @OFFICIAL NEW\Leadership Team\Bowler\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\212448292\AppData\Local\Box\Box Edit\Documents\yHKq1N8p9kanefDTz1B5ig==\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{D179DAEC-2DD2-40E5-A694-294F48291E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE4DF51E-D74C-4227-811D-516419DA60D5}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{A0FF72AF-E087-4B8F-939D-96A71C71115B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{099FC471-C0B4-45E1-B458-985519A21C3B}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="601" xr2:uid="{8476BB21-6D10-4BB9-B6CE-FEFD481D0662}"/>
+    <workbookView xWindow="-23148" yWindow="-48" windowWidth="23256" windowHeight="12456" tabRatio="601" xr2:uid="{8476BB21-6D10-4BB9-B6CE-FEFD481D0662}"/>
   </bookViews>
   <sheets>
     <sheet name="Bowler L1 Training" sheetId="16" r:id="rId1"/>
@@ -40,15 +40,28 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={06BE996C-F791-4A9F-AA6D-EE2A8EE2F4C3}</author>
     <author>Jen Wright</author>
+    <author>tc={17407CA0-19D6-410B-BD94-9BBC65BFCC7C}</author>
     <author>tc={160740E7-DFEB-4450-B5C5-A17286B215D6}</author>
     <author>Philip Ganssmann</author>
     <author>tc={50577B9E-D913-49BB-B91E-A5BD3E934319}</author>
     <author>tc={4A61949D-D058-4614-9CBE-136784BCC6E7}</author>
     <author>tc={40736F15-DF93-4810-BC49-A79E1FB56ED1}</author>
+    <author>tc={F644D89E-1836-4B19-B5E0-2664B9B5862D}</author>
   </authors>
   <commentList>
-    <comment ref="F7" authorId="0" shapeId="0" xr:uid="{6BB47BF6-B4F0-44A1-B661-DC1F618CF875}">
+    <comment ref="Q6" authorId="0" shapeId="0" xr:uid="{06BE996C-F791-4A9F-AA6D-EE2A8EE2F4C3}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    BLC: Lost Time Injury - Fall Event 7/21/2026. Recordable 
+Reply:
+    PSE Near Miss: HLC 7HA.03 Project Post Lift Operation Failure</t>
+      </text>
+    </comment>
+    <comment ref="F7" authorId="1" shapeId="0" xr:uid="{6BB47BF6-B4F0-44A1-B661-DC1F618CF875}">
       <text>
         <r>
           <rPr>
@@ -64,7 +77,17 @@
         </r>
       </text>
     </comment>
-    <comment ref="F13" authorId="1" shapeId="0" xr:uid="{160740E7-DFEB-4450-B5C5-A17286B215D6}">
+    <comment ref="Q9" authorId="2" shapeId="0" xr:uid="{17407CA0-19D6-410B-BD94-9BBC65BFCC7C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    1 X 200000/183589.43=1.089
+Reply:
+    I&amp;I FW 33 1.089</t>
+      </text>
+    </comment>
+    <comment ref="F13" authorId="3" shapeId="0" xr:uid="{160740E7-DFEB-4450-B5C5-A17286B215D6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -72,7 +95,7 @@
     90% RA ATS closure rate all sites by YE</t>
       </text>
     </comment>
-    <comment ref="I24" authorId="2" shapeId="0" xr:uid="{295EE1B2-A25B-412E-A639-7B1259576743}">
+    <comment ref="I24" authorId="4" shapeId="0" xr:uid="{295EE1B2-A25B-412E-A639-7B1259576743}">
       <text>
         <r>
           <rPr>
@@ -87,7 +110,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J24" authorId="2" shapeId="0" xr:uid="{DC09360C-6AE1-46FC-ABAD-4D81C3945042}">
+    <comment ref="J24" authorId="4" shapeId="0" xr:uid="{DC09360C-6AE1-46FC-ABAD-4D81C3945042}">
       <text>
         <r>
           <rPr>
@@ -106,7 +129,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K24" authorId="2" shapeId="0" xr:uid="{64E9CAD9-580E-40D0-B2F1-25AC4998B65A}">
+    <comment ref="K24" authorId="4" shapeId="0" xr:uid="{64E9CAD9-580E-40D0-B2F1-25AC4998B65A}">
       <text>
         <r>
           <rPr>
@@ -123,7 +146,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N24" authorId="2" shapeId="0" xr:uid="{7B5163D0-287F-484F-B9B7-4BE35DBAC943}">
+    <comment ref="N24" authorId="4" shapeId="0" xr:uid="{7B5163D0-287F-484F-B9B7-4BE35DBAC943}">
       <text>
         <r>
           <rPr>
@@ -140,7 +163,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I27" authorId="2" shapeId="0" xr:uid="{90DAD1A6-212D-45E4-8528-2D901E1C0C5A}">
+    <comment ref="I27" authorId="4" shapeId="0" xr:uid="{90DAD1A6-212D-45E4-8528-2D901E1C0C5A}">
       <text>
         <r>
           <rPr>
@@ -155,7 +178,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J27" authorId="2" shapeId="0" xr:uid="{7392AAE5-E54D-4232-B7DC-129B156C6F62}">
+    <comment ref="J27" authorId="4" shapeId="0" xr:uid="{7392AAE5-E54D-4232-B7DC-129B156C6F62}">
       <text>
         <r>
           <rPr>
@@ -182,7 +205,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K27" authorId="2" shapeId="0" xr:uid="{76FCDDC0-41DD-4A57-9E0C-979F0DC1595C}">
+    <comment ref="K27" authorId="4" shapeId="0" xr:uid="{76FCDDC0-41DD-4A57-9E0C-979F0DC1595C}">
       <text>
         <r>
           <rPr>
@@ -209,7 +232,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L27" authorId="2" shapeId="0" xr:uid="{C1388240-DDDB-4DD1-B7FE-11B7EF9BDF13}">
+    <comment ref="L27" authorId="4" shapeId="0" xr:uid="{C1388240-DDDB-4DD1-B7FE-11B7EF9BDF13}">
       <text>
         <r>
           <rPr>
@@ -236,7 +259,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C28" authorId="0" shapeId="0" xr:uid="{62BE848F-A00E-4544-8BD6-953D94ED5EF8}">
+    <comment ref="C28" authorId="1" shapeId="0" xr:uid="{62BE848F-A00E-4544-8BD6-953D94ED5EF8}">
       <text>
         <r>
           <rPr>
@@ -251,7 +274,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C34" authorId="0" shapeId="0" xr:uid="{508037C5-7575-470A-939A-71BD192D06EF}">
+    <comment ref="C34" authorId="1" shapeId="0" xr:uid="{508037C5-7575-470A-939A-71BD192D06EF}">
       <text>
         <r>
           <rPr>
@@ -266,7 +289,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C37" authorId="0" shapeId="0" xr:uid="{04C7CFAE-132D-4578-AA1A-A2AED2C7F976}">
+    <comment ref="C37" authorId="1" shapeId="0" xr:uid="{04C7CFAE-132D-4578-AA1A-A2AED2C7F976}">
       <text>
         <r>
           <rPr>
@@ -281,7 +304,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C40" authorId="0" shapeId="0" xr:uid="{81A96FEF-57F4-4F62-899B-7DDE3044B820}">
+    <comment ref="C40" authorId="1" shapeId="0" xr:uid="{81A96FEF-57F4-4F62-899B-7DDE3044B820}">
       <text>
         <r>
           <rPr>
@@ -296,7 +319,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I42" authorId="0" shapeId="0" xr:uid="{A05FB433-A643-4D7C-BFF5-71BFC3E8211F}">
+    <comment ref="I42" authorId="1" shapeId="0" xr:uid="{A05FB433-A643-4D7C-BFF5-71BFC3E8211F}">
       <text>
         <r>
           <rPr>
@@ -311,7 +334,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J42" authorId="0" shapeId="0" xr:uid="{DF2937F5-01F3-48AD-A59A-11E56D5B996A}">
+    <comment ref="J42" authorId="1" shapeId="0" xr:uid="{DF2937F5-01F3-48AD-A59A-11E56D5B996A}">
       <text>
         <r>
           <rPr>
@@ -326,7 +349,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N42" authorId="0" shapeId="0" xr:uid="{3EABDB6C-68E3-45A8-AD72-EE07047A2ABF}">
+    <comment ref="N42" authorId="1" shapeId="0" xr:uid="{3EABDB6C-68E3-45A8-AD72-EE07047A2ABF}">
       <text>
         <r>
           <rPr>
@@ -341,7 +364,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O42" authorId="3" shapeId="0" xr:uid="{50577B9E-D913-49BB-B91E-A5BD3E934319}">
+    <comment ref="O42" authorId="5" shapeId="0" xr:uid="{50577B9E-D913-49BB-B91E-A5BD3E934319}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -349,7 +372,7 @@
     Pre-arranged with Lead Instructor, the whole GT Mechanical class won't have Pre-OJT</t>
       </text>
     </comment>
-    <comment ref="C43" authorId="0" shapeId="0" xr:uid="{10FC5647-E364-4FB4-A6F5-83AB4EF2B64E}">
+    <comment ref="C43" authorId="1" shapeId="0" xr:uid="{10FC5647-E364-4FB4-A6F5-83AB4EF2B64E}">
       <text>
         <r>
           <rPr>
@@ -365,7 +388,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I45" authorId="0" shapeId="0" xr:uid="{92CB74F4-09AD-4D90-AC85-52E750F91E14}">
+    <comment ref="I45" authorId="1" shapeId="0" xr:uid="{92CB74F4-09AD-4D90-AC85-52E750F91E14}">
       <text>
         <r>
           <rPr>
@@ -380,7 +403,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J45" authorId="0" shapeId="0" xr:uid="{2FC2FC6F-F183-4A7F-9DBC-D4CAC96D4C64}">
+    <comment ref="J45" authorId="1" shapeId="0" xr:uid="{2FC2FC6F-F183-4A7F-9DBC-D4CAC96D4C64}">
       <text>
         <r>
           <rPr>
@@ -395,7 +418,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N45" authorId="0" shapeId="0" xr:uid="{48B8B58B-338A-4616-B616-2225EFDD218F}">
+    <comment ref="N45" authorId="1" shapeId="0" xr:uid="{48B8B58B-338A-4616-B616-2225EFDD218F}">
       <text>
         <r>
           <rPr>
@@ -410,7 +433,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F49" authorId="0" shapeId="0" xr:uid="{E891B715-76B2-41B3-BDA8-A3700F9F11CE}">
+    <comment ref="F49" authorId="1" shapeId="0" xr:uid="{E891B715-76B2-41B3-BDA8-A3700F9F11CE}">
       <text>
         <r>
           <rPr>
@@ -426,7 +449,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K51" authorId="4" shapeId="0" xr:uid="{4A61949D-D058-4614-9CBE-136784BCC6E7}">
+    <comment ref="K51" authorId="6" shapeId="0" xr:uid="{4A61949D-D058-4614-9CBE-136784BCC6E7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -436,7 +459,7 @@
 As tracking stabilizes and system issues are resolved, the data will more accurately reflect true performance and is expected to improve.</t>
       </text>
     </comment>
-    <comment ref="M51" authorId="5" shapeId="0" xr:uid="{40736F15-DF93-4810-BC49-A79E1FB56ED1}">
+    <comment ref="M51" authorId="7" shapeId="0" xr:uid="{40736F15-DF93-4810-BC49-A79E1FB56ED1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -444,7 +467,15 @@
     https://gevernova.box.com/s/17o8hpcpubfb6lm82c157gdcde9kcful</t>
       </text>
     </comment>
-    <comment ref="C52" authorId="0" shapeId="0" xr:uid="{1D261BA2-8304-49D6-B2B0-DECA97456338}">
+    <comment ref="Q51" authorId="8" shapeId="0" xr:uid="{F644D89E-1836-4B19-B5E0-2664B9B5862D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Ben Smith access issues</t>
+      </text>
+    </comment>
+    <comment ref="C52" authorId="1" shapeId="0" xr:uid="{1D261BA2-8304-49D6-B2B0-DECA97456338}">
       <text>
         <r>
           <rPr>
@@ -459,7 +490,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F55" authorId="0" shapeId="0" xr:uid="{B3DF712E-230B-4ACC-BC0C-C0EA167A269C}">
+    <comment ref="F55" authorId="1" shapeId="0" xr:uid="{B3DF712E-230B-4ACC-BC0C-C0EA167A269C}">
       <text>
         <r>
           <rPr>
@@ -475,7 +506,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C58" authorId="0" shapeId="0" xr:uid="{7B8C1B4B-4177-49F0-93C5-A2E4F5B08047}">
+    <comment ref="C58" authorId="1" shapeId="0" xr:uid="{7B8C1B4B-4177-49F0-93C5-A2E4F5B08047}">
       <text>
         <r>
           <rPr>
@@ -490,7 +521,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F58" authorId="0" shapeId="0" xr:uid="{DA09F69C-4C8F-41ED-BFBE-4EBADB371BF8}">
+    <comment ref="F58" authorId="1" shapeId="0" xr:uid="{DA09F69C-4C8F-41ED-BFBE-4EBADB371BF8}">
       <text>
         <r>
           <rPr>
@@ -511,7 +542,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="117">
   <si>
     <t>Level 2</t>
   </si>
@@ -632,6 +663,9 @@
   </si>
   <si>
     <t>Daxer</t>
+  </si>
+  <si>
+    <t>Jul: ENBW (2 courses)-customer mgmt w/ very positive feedback, participants complaints about Sim not site specific; Mill Creek: not recommended, because GT-Maint not needed (LTSA); GECOL: students expected cash or credit card - outside of OFS TRG scope</t>
   </si>
   <si>
     <t># Exams Migrated to Xyleme</t>
@@ -884,16 +918,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="8">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.0_);\(&quot;$&quot;#,##0.0\)"/>
-    <numFmt numFmtId="168" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;?_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0_);\(#,##0.0\)"/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0_);\(&quot;$&quot;#,##0.0\)"/>
+    <numFmt numFmtId="169" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;?_);_(@_)"/>
+    <numFmt numFmtId="170" formatCode="#,##0.0_);\(#,##0.0\)"/>
+    <numFmt numFmtId="171" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1056,11 +1090,6 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -1283,7 +1312,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="235">
@@ -1373,13 +1402,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1389,7 +1418,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1475,22 +1504,22 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="20" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1511,7 +1540,7 @@
     <xf numFmtId="1" fontId="11" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="27" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="27" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="7" fillId="5" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1532,22 +1561,22 @@
     <xf numFmtId="9" fontId="6" fillId="8" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="27" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="27" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="29" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="28" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="29" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="28" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="6" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1556,7 +1585,7 @@
     <xf numFmtId="1" fontId="6" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="29" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="28" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="37" fontId="6" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1569,9 +1598,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="6" fillId="5" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="27" fillId="8" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1598,64 +1624,328 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="29" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="29" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="29" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="29" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="29" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="1" fontId="28" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="28" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="28" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="9" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="7" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="27" fillId="8" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="7" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="3"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="29" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="30" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="21" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="37" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="168" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="37" fontId="9" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="37" fontId="29" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="28" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="165" fontId="26" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="14" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="21" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="29" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="37" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="170" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="22" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="21" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1670,15 +1960,9 @@
     <xf numFmtId="9" fontId="10" fillId="0" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="37" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="37" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1700,281 +1984,26 @@
     <xf numFmtId="1" fontId="14" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="10" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="3" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="22" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="37" fontId="21" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="30" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="31" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="30" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="2" builtinId="5"/>
+    <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2294,6 +2323,18 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="Q6" dT="2026-08-12T01:26:47.89" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{06BE996C-F791-4A9F-AA6D-EE2A8EE2F4C3}">
+    <text xml:space="preserve">BLC: Lost Time Injury - Fall Event 7/21/2026. Recordable </text>
+  </threadedComment>
+  <threadedComment ref="Q6" dT="2026-08-12T01:27:25.92" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{D6A2C5DA-DC04-4CDE-B78F-1BBC1E6623D5}" parentId="{06BE996C-F791-4A9F-AA6D-EE2A8EE2F4C3}">
+    <text>PSE Near Miss: HLC 7HA.03 Project Post Lift Operation Failure</text>
+  </threadedComment>
+  <threadedComment ref="Q9" dT="2026-08-12T12:52:30.70" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{17407CA0-19D6-410B-BD94-9BBC65BFCC7C}">
+    <text>1 X 200000/183589.43=1.089</text>
+  </threadedComment>
+  <threadedComment ref="Q9" dT="2026-08-12T12:52:46.71" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{CFF977E5-20AE-4211-A668-ADE79729D017}" parentId="{17407CA0-19D6-410B-BD94-9BBC65BFCC7C}">
+    <text>I&amp;I FW 33 1.089</text>
+  </threadedComment>
   <threadedComment ref="F13" dT="2024-05-21T17:14:25.01" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{160740E7-DFEB-4450-B5C5-A17286B215D6}">
     <text>90% RA ATS closure rate all sites by YE</text>
   </threadedComment>
@@ -2307,6 +2348,9 @@
   </threadedComment>
   <threadedComment ref="M51" dT="2026-05-08T18:34:11.14" personId="{5990F661-A3AB-41F4-AEAA-FE26C0B875A9}" id="{40736F15-DF93-4810-BC49-A79E1FB56ED1}">
     <text>https://gevernova.box.com/s/17o8hpcpubfb6lm82c157gdcde9kcful</text>
+  </threadedComment>
+  <threadedComment ref="Q51" dT="2026-08-10T18:51:22.55" personId="{5990F661-A3AB-41F4-AEAA-FE26C0B875A9}" id="{F644D89E-1836-4B19-B5E0-2664B9B5862D}">
+    <text>Ben Smith access issues</text>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -2365,31 +2409,31 @@
       <c r="W1" s="5"/>
       <c r="X1" s="6"/>
     </row>
-    <row r="2" spans="1:25" ht="18.600000000000001">
+    <row r="2" spans="1:25" ht="18">
       <c r="A2" s="5"/>
       <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="173">
+      <c r="I2" s="181">
         <v>2026</v>
       </c>
-      <c r="J2" s="174"/>
-      <c r="K2" s="174"/>
-      <c r="L2" s="174"/>
-      <c r="M2" s="174"/>
-      <c r="N2" s="174"/>
-      <c r="O2" s="174"/>
-      <c r="P2" s="174"/>
-      <c r="Q2" s="174"/>
-      <c r="R2" s="174"/>
-      <c r="S2" s="174"/>
-      <c r="T2" s="174"/>
-      <c r="U2" s="174"/>
-      <c r="V2" s="174"/>
-      <c r="W2" s="174"/>
-      <c r="X2" s="175"/>
-    </row>
-    <row r="3" spans="1:25" ht="30.95">
+      <c r="J2" s="182"/>
+      <c r="K2" s="182"/>
+      <c r="L2" s="182"/>
+      <c r="M2" s="182"/>
+      <c r="N2" s="182"/>
+      <c r="O2" s="182"/>
+      <c r="P2" s="182"/>
+      <c r="Q2" s="182"/>
+      <c r="R2" s="182"/>
+      <c r="S2" s="182"/>
+      <c r="T2" s="182"/>
+      <c r="U2" s="182"/>
+      <c r="V2" s="182"/>
+      <c r="W2" s="182"/>
+      <c r="X2" s="183"/>
+    </row>
+    <row r="3" spans="1:25" ht="31.15">
       <c r="A3" s="5"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2460,25 +2504,25 @@
       </c>
     </row>
     <row r="4" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B4" s="194" t="s">
+      <c r="B4" s="162" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="180" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="166" t="s">
+      <c r="D4" s="187" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="182">
+      <c r="E4" s="188">
         <f>SUM(L4,P4,T4,X4)</f>
         <v>0</v>
       </c>
-      <c r="F4" s="126">
-        <v>0</v>
-      </c>
-      <c r="G4" s="182">
+      <c r="F4" s="191">
+        <v>0</v>
+      </c>
+      <c r="G4" s="190">
         <f>SUM(L6,P6,T6,X6)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>26</v>
@@ -2537,12 +2581,12 @@
       </c>
     </row>
     <row r="5" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B5" s="194"/>
+      <c r="B5" s="162"/>
       <c r="C5" s="180"/>
-      <c r="D5" s="166"/>
-      <c r="E5" s="182"/>
-      <c r="F5" s="126"/>
-      <c r="G5" s="182"/>
+      <c r="D5" s="187"/>
+      <c r="E5" s="188"/>
+      <c r="F5" s="191"/>
+      <c r="G5" s="190"/>
       <c r="H5" s="11" t="s">
         <v>27</v>
       </c>
@@ -2600,12 +2644,12 @@
       </c>
     </row>
     <row r="6" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B6" s="194"/>
+      <c r="B6" s="162"/>
       <c r="C6" s="180"/>
-      <c r="D6" s="166"/>
-      <c r="E6" s="182"/>
-      <c r="F6" s="126"/>
-      <c r="G6" s="182"/>
+      <c r="D6" s="187"/>
+      <c r="E6" s="188"/>
+      <c r="F6" s="191"/>
+      <c r="G6" s="190"/>
       <c r="H6" s="11" t="s">
         <v>28</v>
       </c>
@@ -2628,19 +2672,21 @@
       <c r="N6" s="87">
         <v>0</v>
       </c>
-      <c r="O6" s="122">
+      <c r="O6" s="116">
         <v>0</v>
       </c>
       <c r="P6" s="98">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q6" s="14"/>
+      <c r="Q6" s="117">
+        <v>1</v>
+      </c>
       <c r="R6" s="14"/>
       <c r="S6" s="14"/>
       <c r="T6" s="13">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U6" s="14"/>
       <c r="V6" s="14"/>
@@ -2651,23 +2697,23 @@
       </c>
     </row>
     <row r="7" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B7" s="194"/>
-      <c r="C7" s="129" t="s">
+      <c r="B7" s="162"/>
+      <c r="C7" s="143" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="130" t="s">
+      <c r="D7" s="170" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="167">
-        <v>0</v>
-      </c>
-      <c r="F7" s="183">
-        <v>0</v>
-      </c>
-      <c r="G7" s="185">
-        <v>0</v>
-      </c>
-      <c r="H7" s="119" t="s">
+      <c r="E7" s="202">
+        <v>0</v>
+      </c>
+      <c r="F7" s="192">
+        <v>0</v>
+      </c>
+      <c r="G7" s="195">
+        <v>1.089</v>
+      </c>
+      <c r="H7" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I7" s="15">
@@ -2720,13 +2766,13 @@
       </c>
     </row>
     <row r="8" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B8" s="194"/>
-      <c r="C8" s="129"/>
-      <c r="D8" s="130"/>
-      <c r="E8" s="168"/>
-      <c r="F8" s="183"/>
-      <c r="G8" s="185"/>
-      <c r="H8" s="119" t="s">
+      <c r="B8" s="162"/>
+      <c r="C8" s="143"/>
+      <c r="D8" s="170"/>
+      <c r="E8" s="203"/>
+      <c r="F8" s="192"/>
+      <c r="G8" s="195"/>
+      <c r="H8" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I8" s="15">
@@ -2779,13 +2825,13 @@
       </c>
     </row>
     <row r="9" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B9" s="194"/>
-      <c r="C9" s="129"/>
-      <c r="D9" s="130"/>
-      <c r="E9" s="169"/>
-      <c r="F9" s="183"/>
-      <c r="G9" s="185"/>
-      <c r="H9" s="119" t="s">
+      <c r="B9" s="162"/>
+      <c r="C9" s="143"/>
+      <c r="D9" s="170"/>
+      <c r="E9" s="204"/>
+      <c r="F9" s="192"/>
+      <c r="G9" s="195"/>
+      <c r="H9" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I9" s="86">
@@ -2812,7 +2858,9 @@
       <c r="P9" s="98">
         <v>0</v>
       </c>
-      <c r="Q9" s="45"/>
+      <c r="Q9" s="124">
+        <v>1.089</v>
+      </c>
       <c r="R9" s="45"/>
       <c r="S9" s="45"/>
       <c r="T9" s="44"/>
@@ -2822,22 +2870,22 @@
       <c r="X9" s="16"/>
     </row>
     <row r="10" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B10" s="194"/>
+      <c r="B10" s="162"/>
       <c r="C10" s="180" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="166" t="s">
+      <c r="D10" s="187" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="137">
+      <c r="E10" s="201">
         <f>SUM(L10,P10,T10,X10)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="126">
+      <c r="F10" s="191">
         <f>SUM(L11,P11,T11,X11)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="182">
+      <c r="G10" s="188">
         <f>SUM(L12,P12,T12,X12)</f>
         <v>0</v>
       </c>
@@ -2898,12 +2946,12 @@
       </c>
     </row>
     <row r="11" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B11" s="194"/>
+      <c r="B11" s="162"/>
       <c r="C11" s="180"/>
-      <c r="D11" s="166"/>
-      <c r="E11" s="137"/>
-      <c r="F11" s="126"/>
-      <c r="G11" s="182"/>
+      <c r="D11" s="187"/>
+      <c r="E11" s="201"/>
+      <c r="F11" s="191"/>
+      <c r="G11" s="188"/>
       <c r="H11" s="11" t="s">
         <v>27</v>
       </c>
@@ -2961,12 +3009,12 @@
       </c>
     </row>
     <row r="12" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B12" s="194"/>
+      <c r="B12" s="162"/>
       <c r="C12" s="180"/>
-      <c r="D12" s="166"/>
-      <c r="E12" s="137"/>
-      <c r="F12" s="126"/>
-      <c r="G12" s="182"/>
+      <c r="D12" s="187"/>
+      <c r="E12" s="201"/>
+      <c r="F12" s="191"/>
+      <c r="G12" s="188"/>
       <c r="H12" s="11" t="s">
         <v>28</v>
       </c>
@@ -2996,7 +3044,9 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Q12" s="14"/>
+      <c r="Q12" s="87">
+        <v>0</v>
+      </c>
       <c r="R12" s="14"/>
       <c r="S12" s="14"/>
       <c r="T12" s="13">
@@ -3012,23 +3062,23 @@
       </c>
     </row>
     <row r="13" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B13" s="194"/>
-      <c r="C13" s="129" t="s">
+      <c r="B13" s="162"/>
+      <c r="C13" s="143" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="130" t="s">
+      <c r="D13" s="170" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="181">
+      <c r="E13" s="155">
         <v>1</v>
       </c>
-      <c r="F13" s="145">
-        <v>0.9</v>
-      </c>
-      <c r="G13" s="181">
-        <v>0.9</v>
-      </c>
-      <c r="H13" s="119" t="s">
+      <c r="F13" s="200">
+        <v>0.9</v>
+      </c>
+      <c r="G13" s="155">
+        <v>0.9</v>
+      </c>
+      <c r="H13" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I13" s="15" t="s">
@@ -3081,13 +3131,13 @@
       </c>
     </row>
     <row r="14" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B14" s="194"/>
-      <c r="C14" s="129"/>
-      <c r="D14" s="130"/>
-      <c r="E14" s="181"/>
-      <c r="F14" s="145"/>
-      <c r="G14" s="181"/>
-      <c r="H14" s="119" t="s">
+      <c r="B14" s="162"/>
+      <c r="C14" s="143"/>
+      <c r="D14" s="170"/>
+      <c r="E14" s="155"/>
+      <c r="F14" s="200"/>
+      <c r="G14" s="155"/>
+      <c r="H14" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I14" s="38">
@@ -3140,13 +3190,13 @@
       </c>
     </row>
     <row r="15" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B15" s="194"/>
-      <c r="C15" s="129"/>
-      <c r="D15" s="130"/>
-      <c r="E15" s="181"/>
-      <c r="F15" s="145"/>
-      <c r="G15" s="181"/>
-      <c r="H15" s="119" t="s">
+      <c r="B15" s="162"/>
+      <c r="C15" s="143"/>
+      <c r="D15" s="170"/>
+      <c r="E15" s="155"/>
+      <c r="F15" s="200"/>
+      <c r="G15" s="155"/>
+      <c r="H15" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I15" s="77">
@@ -3173,7 +3223,9 @@
       <c r="P15" s="88">
         <v>0.9</v>
       </c>
-      <c r="Q15" s="47"/>
+      <c r="Q15" s="77" t="s">
+        <v>32</v>
+      </c>
       <c r="R15" s="47"/>
       <c r="S15" s="47"/>
       <c r="T15" s="48"/>
@@ -3183,23 +3235,23 @@
       <c r="X15" s="16"/>
     </row>
     <row r="16" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B16" s="194"/>
-      <c r="C16" s="127" t="s">
+      <c r="B16" s="162"/>
+      <c r="C16" s="205" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="171" t="s">
+      <c r="D16" s="189" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="126" t="s">
+      <c r="E16" s="191" t="s">
         <v>35</v>
       </c>
-      <c r="F16" s="157">
-        <v>0.9</v>
-      </c>
-      <c r="G16" s="154">
+      <c r="F16" s="193">
+        <v>0.9</v>
+      </c>
+      <c r="G16" s="198">
         <v>0.95</v>
       </c>
-      <c r="H16" s="121" t="s">
+      <c r="H16" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I16" s="19" t="s">
@@ -3255,13 +3307,13 @@
       </c>
     </row>
     <row r="17" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B17" s="194"/>
-      <c r="C17" s="128"/>
-      <c r="D17" s="171"/>
-      <c r="E17" s="126"/>
-      <c r="F17" s="157"/>
-      <c r="G17" s="154"/>
-      <c r="H17" s="121" t="s">
+      <c r="B17" s="162"/>
+      <c r="C17" s="163"/>
+      <c r="D17" s="189"/>
+      <c r="E17" s="191"/>
+      <c r="F17" s="193"/>
+      <c r="G17" s="198"/>
+      <c r="H17" s="120" t="s">
         <v>27</v>
       </c>
       <c r="I17" s="21">
@@ -3314,13 +3366,13 @@
       </c>
     </row>
     <row r="18" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B18" s="194"/>
-      <c r="C18" s="128"/>
-      <c r="D18" s="171"/>
-      <c r="E18" s="126"/>
-      <c r="F18" s="184"/>
-      <c r="G18" s="155"/>
-      <c r="H18" s="121" t="s">
+      <c r="B18" s="162"/>
+      <c r="C18" s="163"/>
+      <c r="D18" s="189"/>
+      <c r="E18" s="191"/>
+      <c r="F18" s="194"/>
+      <c r="G18" s="199"/>
+      <c r="H18" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I18" s="85">
@@ -3335,19 +3387,21 @@
       <c r="L18" s="94">
         <v>0.92</v>
       </c>
-      <c r="M18" s="102">
-        <v>100</v>
-      </c>
-      <c r="N18" s="102">
-        <v>100</v>
-      </c>
-      <c r="O18" s="105">
+      <c r="M18" s="118">
+        <v>1</v>
+      </c>
+      <c r="N18" s="118">
+        <v>1</v>
+      </c>
+      <c r="O18" s="104">
         <v>84.6</v>
       </c>
-      <c r="P18" s="123">
-        <v>95</v>
-      </c>
-      <c r="Q18" s="52"/>
+      <c r="P18" s="94">
+        <v>0.95</v>
+      </c>
+      <c r="Q18" s="118">
+        <v>1</v>
+      </c>
       <c r="R18" s="53"/>
       <c r="S18" s="52"/>
       <c r="T18" s="43"/>
@@ -3357,25 +3411,25 @@
       <c r="X18" s="43"/>
     </row>
     <row r="19" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B19" s="194" t="s">
+      <c r="B19" s="162" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="129" t="s">
+      <c r="C19" s="143" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="130" t="s">
+      <c r="D19" s="170" t="s">
         <v>39</v>
       </c>
-      <c r="E19" s="131">
+      <c r="E19" s="218">
         <v>83</v>
       </c>
-      <c r="F19" s="143">
+      <c r="F19" s="228">
         <v>83</v>
       </c>
-      <c r="G19" s="124">
-        <v>84.9</v>
-      </c>
-      <c r="H19" s="119" t="s">
+      <c r="G19" s="218">
+        <v>83.8</v>
+      </c>
+      <c r="H19" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I19" s="56">
@@ -3428,13 +3482,13 @@
       </c>
     </row>
     <row r="20" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B20" s="194"/>
-      <c r="C20" s="129"/>
-      <c r="D20" s="130"/>
-      <c r="E20" s="132"/>
-      <c r="F20" s="144"/>
-      <c r="G20" s="125"/>
-      <c r="H20" s="119" t="s">
+      <c r="B20" s="162"/>
+      <c r="C20" s="143"/>
+      <c r="D20" s="170"/>
+      <c r="E20" s="219"/>
+      <c r="F20" s="229"/>
+      <c r="G20" s="219"/>
+      <c r="H20" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I20" s="56">
@@ -3487,13 +3541,13 @@
       </c>
     </row>
     <row r="21" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B21" s="194"/>
-      <c r="C21" s="129"/>
-      <c r="D21" s="130"/>
-      <c r="E21" s="132"/>
-      <c r="F21" s="144"/>
-      <c r="G21" s="125"/>
-      <c r="H21" s="119" t="s">
+      <c r="B21" s="162"/>
+      <c r="C21" s="143"/>
+      <c r="D21" s="170"/>
+      <c r="E21" s="219"/>
+      <c r="F21" s="229"/>
+      <c r="G21" s="219"/>
+      <c r="H21" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I21" s="76">
@@ -3511,16 +3565,18 @@
       <c r="M21" s="76">
         <v>79</v>
       </c>
-      <c r="N21" s="106">
+      <c r="N21" s="105">
         <v>91</v>
       </c>
       <c r="O21" s="76">
-        <v>80.599999999999994</v>
+        <v>78</v>
       </c>
       <c r="P21" s="90">
         <v>84.4</v>
       </c>
-      <c r="Q21" s="58"/>
+      <c r="Q21" s="76">
+        <v>82.5</v>
+      </c>
       <c r="R21" s="58"/>
       <c r="S21" s="58"/>
       <c r="T21" s="58"/>
@@ -3528,26 +3584,29 @@
       <c r="V21" s="58"/>
       <c r="W21" s="58"/>
       <c r="X21" s="44"/>
+      <c r="Y21" s="7" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="22" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B22" s="194"/>
-      <c r="C22" s="127" t="s">
-        <v>40</v>
-      </c>
-      <c r="D22" s="170" t="s">
+      <c r="B22" s="162"/>
+      <c r="C22" s="205" t="s">
         <v>41</v>
       </c>
-      <c r="E22" s="172" t="s">
+      <c r="D22" s="206" t="s">
+        <v>42</v>
+      </c>
+      <c r="E22" s="207" t="s">
         <v>35</v>
       </c>
-      <c r="F22" s="126">
+      <c r="F22" s="191">
         <v>55</v>
       </c>
-      <c r="G22" s="137">
+      <c r="G22" s="201">
         <f>SUM(L24,P24,T24,X24)</f>
-        <v>56</v>
-      </c>
-      <c r="H22" s="121" t="s">
+        <v>76</v>
+      </c>
+      <c r="H22" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I22" s="24" t="s">
@@ -3603,13 +3662,13 @@
       </c>
     </row>
     <row r="23" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B23" s="194"/>
-      <c r="C23" s="128"/>
-      <c r="D23" s="171"/>
-      <c r="E23" s="172"/>
-      <c r="F23" s="126"/>
-      <c r="G23" s="137"/>
-      <c r="H23" s="121" t="s">
+      <c r="B23" s="162"/>
+      <c r="C23" s="163"/>
+      <c r="D23" s="189"/>
+      <c r="E23" s="207"/>
+      <c r="F23" s="191"/>
+      <c r="G23" s="201"/>
+      <c r="H23" s="120" t="s">
         <v>27</v>
       </c>
       <c r="I23" s="12">
@@ -3662,13 +3721,13 @@
       </c>
     </row>
     <row r="24" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B24" s="194"/>
-      <c r="C24" s="128"/>
-      <c r="D24" s="171"/>
-      <c r="E24" s="172"/>
-      <c r="F24" s="126"/>
-      <c r="G24" s="137"/>
-      <c r="H24" s="121" t="s">
+      <c r="B24" s="162"/>
+      <c r="C24" s="163"/>
+      <c r="D24" s="189"/>
+      <c r="E24" s="207"/>
+      <c r="F24" s="191"/>
+      <c r="G24" s="201"/>
+      <c r="H24" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I24" s="86">
@@ -3696,12 +3755,14 @@
         <f>SUM(M24:O24)</f>
         <v>46</v>
       </c>
-      <c r="Q24" s="69"/>
+      <c r="Q24" s="84">
+        <v>20</v>
+      </c>
       <c r="R24" s="19"/>
       <c r="S24" s="69"/>
       <c r="T24" s="79">
         <f>SUM(Q24:S24)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="U24" s="69"/>
       <c r="V24" s="69"/>
@@ -3712,24 +3773,24 @@
       </c>
     </row>
     <row r="25" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B25" s="194"/>
-      <c r="C25" s="199" t="s">
+      <c r="B25" s="162"/>
+      <c r="C25" s="168" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="169" t="s">
         <v>42</v>
       </c>
-      <c r="D25" s="200" t="s">
-        <v>41</v>
-      </c>
-      <c r="E25" s="201" t="s">
+      <c r="E25" s="171" t="s">
         <v>35</v>
       </c>
-      <c r="F25" s="202">
+      <c r="F25" s="172">
         <v>120</v>
       </c>
-      <c r="G25" s="203">
+      <c r="G25" s="173">
         <f>SUM(L27,P27,T27,X27)</f>
-        <v>34</v>
-      </c>
-      <c r="H25" s="119" t="s">
+        <v>38</v>
+      </c>
+      <c r="H25" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I25" s="15" t="s">
@@ -3785,13 +3846,13 @@
       </c>
     </row>
     <row r="26" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B26" s="194"/>
-      <c r="C26" s="129"/>
-      <c r="D26" s="130"/>
-      <c r="E26" s="201"/>
-      <c r="F26" s="202"/>
-      <c r="G26" s="204"/>
-      <c r="H26" s="119" t="s">
+      <c r="B26" s="162"/>
+      <c r="C26" s="143"/>
+      <c r="D26" s="170"/>
+      <c r="E26" s="171"/>
+      <c r="F26" s="172"/>
+      <c r="G26" s="174"/>
+      <c r="H26" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I26" s="15">
@@ -3843,17 +3904,17 @@
         <v>30</v>
       </c>
       <c r="Y26" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B27" s="194"/>
-      <c r="C27" s="129"/>
-      <c r="D27" s="130"/>
-      <c r="E27" s="201"/>
-      <c r="F27" s="202"/>
-      <c r="G27" s="204"/>
-      <c r="H27" s="119" t="s">
+      <c r="B27" s="162"/>
+      <c r="C27" s="143"/>
+      <c r="D27" s="170"/>
+      <c r="E27" s="171"/>
+      <c r="F27" s="172"/>
+      <c r="G27" s="174"/>
+      <c r="H27" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I27" s="80">
@@ -3882,40 +3943,42 @@
         <f>SUM(M27:O27)</f>
         <v>31</v>
       </c>
-      <c r="Q27" s="103"/>
-      <c r="R27" s="103"/>
-      <c r="S27" s="103"/>
+      <c r="Q27" s="80">
+        <v>4</v>
+      </c>
+      <c r="R27" s="102"/>
+      <c r="S27" s="102"/>
       <c r="T27" s="57">
         <f>SUM(Q27:S27)</f>
-        <v>0</v>
-      </c>
-      <c r="U27" s="103"/>
-      <c r="V27" s="103"/>
-      <c r="W27" s="103"/>
+        <v>4</v>
+      </c>
+      <c r="U27" s="102"/>
+      <c r="V27" s="102"/>
+      <c r="W27" s="102"/>
       <c r="X27" s="57">
         <f>SUM(U27:W27)</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B28" s="194"/>
-      <c r="C28" s="127" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" s="170" t="s">
-        <v>41</v>
-      </c>
-      <c r="E28" s="172" t="s">
+      <c r="B28" s="162"/>
+      <c r="C28" s="205" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28" s="206" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28" s="207" t="s">
         <v>35</v>
       </c>
-      <c r="F28" s="148">
-        <v>0.85</v>
-      </c>
-      <c r="G28" s="149">
+      <c r="F28" s="209">
+        <v>0.82</v>
+      </c>
+      <c r="G28" s="232">
         <f>O30</f>
         <v>0.73</v>
       </c>
-      <c r="H28" s="121" t="s">
+      <c r="H28" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I28" s="24" t="s">
@@ -3971,13 +4034,13 @@
       </c>
     </row>
     <row r="29" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B29" s="194"/>
-      <c r="C29" s="128"/>
-      <c r="D29" s="171"/>
-      <c r="E29" s="172"/>
-      <c r="F29" s="148"/>
-      <c r="G29" s="149"/>
-      <c r="H29" s="121" t="s">
+      <c r="B29" s="162"/>
+      <c r="C29" s="163"/>
+      <c r="D29" s="189"/>
+      <c r="E29" s="207"/>
+      <c r="F29" s="209"/>
+      <c r="G29" s="232"/>
+      <c r="H29" s="120" t="s">
         <v>27</v>
       </c>
       <c r="I29" s="24">
@@ -4029,17 +4092,17 @@
         <v>0.85</v>
       </c>
       <c r="Y29" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B30" s="194"/>
-      <c r="C30" s="128"/>
-      <c r="D30" s="171"/>
-      <c r="E30" s="172"/>
-      <c r="F30" s="148"/>
-      <c r="G30" s="149"/>
-      <c r="H30" s="121" t="s">
+      <c r="B30" s="162"/>
+      <c r="C30" s="163"/>
+      <c r="D30" s="189"/>
+      <c r="E30" s="207"/>
+      <c r="F30" s="209"/>
+      <c r="G30" s="232"/>
+      <c r="H30" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I30" s="78">
@@ -4068,12 +4131,14 @@
         <f>AVERAGE(M30:O30)</f>
         <v>0.77333333333333332</v>
       </c>
-      <c r="Q30" s="65"/>
+      <c r="Q30" s="77">
+        <v>0.82</v>
+      </c>
       <c r="R30" s="19"/>
       <c r="S30" s="65"/>
-      <c r="T30" s="66" t="e">
+      <c r="T30" s="66">
         <f>AVERAGE(Q30:S30)</f>
-        <v>#DIV/0!</v>
+        <v>0.82</v>
       </c>
       <c r="U30" s="65"/>
       <c r="V30" s="65"/>
@@ -4084,23 +4149,23 @@
       </c>
     </row>
     <row r="31" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B31" s="194"/>
-      <c r="C31" s="129" t="s">
-        <v>46</v>
-      </c>
-      <c r="D31" s="130" t="s">
+      <c r="B31" s="162"/>
+      <c r="C31" s="143" t="s">
         <v>47</v>
       </c>
-      <c r="E31" s="181">
+      <c r="D31" s="170" t="s">
+        <v>48</v>
+      </c>
+      <c r="E31" s="155">
         <v>0.82</v>
       </c>
-      <c r="F31" s="145">
+      <c r="F31" s="200">
         <v>0.7</v>
       </c>
-      <c r="G31" s="181">
+      <c r="G31" s="155">
         <v>0.83</v>
       </c>
-      <c r="H31" s="119" t="s">
+      <c r="H31" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I31" s="26" t="s">
@@ -4153,13 +4218,13 @@
       </c>
     </row>
     <row r="32" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B32" s="194"/>
-      <c r="C32" s="129"/>
-      <c r="D32" s="130"/>
-      <c r="E32" s="181"/>
-      <c r="F32" s="145"/>
-      <c r="G32" s="181"/>
-      <c r="H32" s="119" t="s">
+      <c r="B32" s="162"/>
+      <c r="C32" s="143"/>
+      <c r="D32" s="170"/>
+      <c r="E32" s="155"/>
+      <c r="F32" s="200"/>
+      <c r="G32" s="155"/>
+      <c r="H32" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I32" s="26">
@@ -4211,24 +4276,24 @@
         <v>0.7</v>
       </c>
       <c r="Y32" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B33" s="194"/>
-      <c r="C33" s="129"/>
-      <c r="D33" s="130"/>
-      <c r="E33" s="181"/>
-      <c r="F33" s="145"/>
-      <c r="G33" s="181"/>
-      <c r="H33" s="119" t="s">
+      <c r="B33" s="162"/>
+      <c r="C33" s="143"/>
+      <c r="D33" s="170"/>
+      <c r="E33" s="155"/>
+      <c r="F33" s="200"/>
+      <c r="G33" s="155"/>
+      <c r="H33" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I33" s="26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J33" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K33" s="77">
         <v>0.83</v>
@@ -4237,10 +4302,10 @@
         <v>0.83</v>
       </c>
       <c r="M33" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N33" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O33" s="77">
         <v>0.81</v>
@@ -4248,7 +4313,9 @@
       <c r="P33" s="88">
         <v>0.81</v>
       </c>
-      <c r="Q33" s="49"/>
+      <c r="Q33" s="15" t="s">
+        <v>50</v>
+      </c>
       <c r="R33" s="15"/>
       <c r="S33" s="49"/>
       <c r="T33" s="63"/>
@@ -4258,25 +4325,25 @@
       <c r="X33" s="33"/>
     </row>
     <row r="34" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B34" s="186" t="s">
-        <v>50</v>
-      </c>
-      <c r="C34" s="128" t="s">
+      <c r="B34" s="147" t="s">
         <v>51</v>
       </c>
-      <c r="D34" s="150" t="s">
+      <c r="C34" s="163" t="s">
         <v>52</v>
       </c>
-      <c r="E34" s="154">
+      <c r="D34" s="153" t="s">
+        <v>53</v>
+      </c>
+      <c r="E34" s="198">
         <v>0.77</v>
       </c>
-      <c r="F34" s="148">
+      <c r="F34" s="209">
         <v>0.85</v>
       </c>
-      <c r="G34" s="158">
+      <c r="G34" s="196">
         <v>0.79</v>
       </c>
-      <c r="H34" s="121" t="s">
+      <c r="H34" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I34" s="21">
@@ -4329,13 +4396,13 @@
       </c>
     </row>
     <row r="35" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B35" s="187"/>
-      <c r="C35" s="128"/>
-      <c r="D35" s="150"/>
-      <c r="E35" s="154"/>
-      <c r="F35" s="148"/>
-      <c r="G35" s="158"/>
-      <c r="H35" s="121" t="s">
+      <c r="B35" s="148"/>
+      <c r="C35" s="163"/>
+      <c r="D35" s="153"/>
+      <c r="E35" s="198"/>
+      <c r="F35" s="209"/>
+      <c r="G35" s="196"/>
+      <c r="H35" s="120" t="s">
         <v>27</v>
       </c>
       <c r="I35" s="21">
@@ -4388,13 +4455,13 @@
       </c>
     </row>
     <row r="36" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B36" s="187"/>
-      <c r="C36" s="195"/>
-      <c r="D36" s="191"/>
-      <c r="E36" s="155"/>
-      <c r="F36" s="148"/>
-      <c r="G36" s="234"/>
-      <c r="H36" s="121" t="s">
+      <c r="B36" s="148"/>
+      <c r="C36" s="164"/>
+      <c r="D36" s="159"/>
+      <c r="E36" s="199"/>
+      <c r="F36" s="209"/>
+      <c r="G36" s="197"/>
+      <c r="H36" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I36" s="77">
@@ -4421,7 +4488,9 @@
       <c r="P36" s="95">
         <v>0.8</v>
       </c>
-      <c r="Q36" s="50"/>
+      <c r="Q36" s="78">
+        <v>0.79</v>
+      </c>
       <c r="R36" s="50"/>
       <c r="S36" s="50"/>
       <c r="T36" s="67"/>
@@ -4431,20 +4500,20 @@
       <c r="X36" s="67"/>
     </row>
     <row r="37" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B37" s="187"/>
-      <c r="C37" s="138" t="s">
-        <v>53</v>
-      </c>
-      <c r="D37" s="141" t="s">
+      <c r="B37" s="148"/>
+      <c r="C37" s="223" t="s">
         <v>54</v>
       </c>
-      <c r="E37" s="161" t="s">
+      <c r="D37" s="226" t="s">
+        <v>55</v>
+      </c>
+      <c r="E37" s="213" t="s">
         <v>35</v>
       </c>
-      <c r="F37" s="162">
-        <v>0.9</v>
-      </c>
-      <c r="G37" s="165">
+      <c r="F37" s="214">
+        <v>0.9</v>
+      </c>
+      <c r="G37" s="217">
         <v>0.6</v>
       </c>
       <c r="H37" s="39" t="s">
@@ -4503,12 +4572,12 @@
       </c>
     </row>
     <row r="38" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B38" s="187"/>
-      <c r="C38" s="139"/>
-      <c r="D38" s="142"/>
-      <c r="E38" s="161"/>
-      <c r="F38" s="162"/>
-      <c r="G38" s="165"/>
+      <c r="B38" s="148"/>
+      <c r="C38" s="224"/>
+      <c r="D38" s="227"/>
+      <c r="E38" s="213"/>
+      <c r="F38" s="214"/>
+      <c r="G38" s="217"/>
       <c r="H38" s="39" t="s">
         <v>27</v>
       </c>
@@ -4562,12 +4631,12 @@
       </c>
     </row>
     <row r="39" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B39" s="187"/>
-      <c r="C39" s="140"/>
-      <c r="D39" s="142"/>
-      <c r="E39" s="161"/>
-      <c r="F39" s="163"/>
-      <c r="G39" s="165"/>
+      <c r="B39" s="148"/>
+      <c r="C39" s="225"/>
+      <c r="D39" s="227"/>
+      <c r="E39" s="213"/>
+      <c r="F39" s="215"/>
+      <c r="G39" s="217"/>
       <c r="H39" s="39" t="s">
         <v>28</v>
       </c>
@@ -4595,7 +4664,9 @@
       <c r="P39" s="95">
         <v>0.4</v>
       </c>
-      <c r="Q39" s="60"/>
+      <c r="Q39" s="78">
+        <v>0.2</v>
+      </c>
       <c r="R39" s="60"/>
       <c r="S39" s="60"/>
       <c r="T39" s="60"/>
@@ -4605,20 +4676,20 @@
       <c r="X39" s="18"/>
     </row>
     <row r="40" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B40" s="187"/>
-      <c r="C40" s="205" t="s">
+      <c r="B40" s="148"/>
+      <c r="C40" s="175" t="s">
+        <v>56</v>
+      </c>
+      <c r="D40" s="178" t="s">
         <v>55</v>
       </c>
-      <c r="D40" s="208" t="s">
-        <v>54</v>
-      </c>
-      <c r="E40" s="209" t="s">
+      <c r="E40" s="179" t="s">
         <v>35</v>
       </c>
-      <c r="F40" s="148">
-        <v>0.9</v>
-      </c>
-      <c r="G40" s="159">
+      <c r="F40" s="209">
+        <v>0.9</v>
+      </c>
+      <c r="G40" s="211">
         <v>0.85</v>
       </c>
       <c r="H40" s="59" t="s">
@@ -4677,12 +4748,12 @@
       </c>
     </row>
     <row r="41" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B41" s="187"/>
-      <c r="C41" s="206"/>
-      <c r="D41" s="150"/>
-      <c r="E41" s="209"/>
-      <c r="F41" s="148"/>
-      <c r="G41" s="160"/>
+      <c r="B41" s="148"/>
+      <c r="C41" s="176"/>
+      <c r="D41" s="153"/>
+      <c r="E41" s="179"/>
+      <c r="F41" s="209"/>
+      <c r="G41" s="212"/>
       <c r="H41" s="59" t="s">
         <v>27</v>
       </c>
@@ -4736,12 +4807,12 @@
       </c>
     </row>
     <row r="42" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B42" s="187"/>
-      <c r="C42" s="207"/>
-      <c r="D42" s="150"/>
-      <c r="E42" s="209"/>
-      <c r="F42" s="148"/>
-      <c r="G42" s="160"/>
+      <c r="B42" s="148"/>
+      <c r="C42" s="177"/>
+      <c r="D42" s="153"/>
+      <c r="E42" s="179"/>
+      <c r="F42" s="209"/>
+      <c r="G42" s="212"/>
       <c r="H42" s="59" t="s">
         <v>28</v>
       </c>
@@ -4769,7 +4840,9 @@
       <c r="P42" s="101">
         <v>0.57999999999999996</v>
       </c>
-      <c r="Q42" s="51"/>
+      <c r="Q42" s="83">
+        <v>0.7</v>
+      </c>
       <c r="R42" s="51"/>
       <c r="S42" s="51"/>
       <c r="T42" s="51"/>
@@ -4779,20 +4852,20 @@
       <c r="X42" s="13"/>
     </row>
     <row r="43" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B43" s="187"/>
-      <c r="C43" s="146" t="s">
-        <v>56</v>
-      </c>
-      <c r="D43" s="141" t="s">
-        <v>54</v>
-      </c>
-      <c r="E43" s="161" t="s">
+      <c r="B43" s="148"/>
+      <c r="C43" s="230" t="s">
+        <v>57</v>
+      </c>
+      <c r="D43" s="226" t="s">
+        <v>55</v>
+      </c>
+      <c r="E43" s="213" t="s">
         <v>35</v>
       </c>
-      <c r="F43" s="162">
+      <c r="F43" s="214">
         <v>1</v>
       </c>
-      <c r="G43" s="164">
+      <c r="G43" s="216">
         <v>0.93</v>
       </c>
       <c r="H43" s="39" t="s">
@@ -4851,12 +4924,12 @@
       </c>
     </row>
     <row r="44" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B44" s="187"/>
-      <c r="C44" s="147"/>
-      <c r="D44" s="142"/>
-      <c r="E44" s="161"/>
-      <c r="F44" s="162"/>
-      <c r="G44" s="164"/>
+      <c r="B44" s="148"/>
+      <c r="C44" s="231"/>
+      <c r="D44" s="227"/>
+      <c r="E44" s="213"/>
+      <c r="F44" s="214"/>
+      <c r="G44" s="216"/>
       <c r="H44" s="39" t="s">
         <v>27</v>
       </c>
@@ -4909,16 +4982,16 @@
         <v>1</v>
       </c>
       <c r="Y44" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="45" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B45" s="187"/>
-      <c r="C45" s="147"/>
-      <c r="D45" s="142"/>
-      <c r="E45" s="161"/>
-      <c r="F45" s="163"/>
-      <c r="G45" s="164"/>
+      <c r="B45" s="148"/>
+      <c r="C45" s="231"/>
+      <c r="D45" s="227"/>
+      <c r="E45" s="213"/>
+      <c r="F45" s="215"/>
+      <c r="G45" s="216"/>
       <c r="H45" s="39" t="s">
         <v>28</v>
       </c>
@@ -4946,7 +5019,9 @@
       <c r="P45" s="101">
         <v>0.99</v>
       </c>
-      <c r="Q45" s="60"/>
+      <c r="Q45" s="83">
+        <v>0.95</v>
+      </c>
       <c r="R45" s="60"/>
       <c r="S45" s="60"/>
       <c r="T45" s="60"/>
@@ -4956,144 +5031,144 @@
       <c r="X45" s="18"/>
     </row>
     <row r="46" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B46" s="187"/>
-      <c r="C46" s="128" t="s">
-        <v>58</v>
-      </c>
-      <c r="D46" s="150" t="s">
-        <v>54</v>
-      </c>
-      <c r="E46" s="151">
+      <c r="B46" s="148"/>
+      <c r="C46" s="163" t="s">
+        <v>59</v>
+      </c>
+      <c r="D46" s="153" t="s">
+        <v>55</v>
+      </c>
+      <c r="E46" s="233">
         <v>372</v>
       </c>
-      <c r="F46" s="152">
+      <c r="F46" s="234">
         <v>366</v>
       </c>
-      <c r="G46" s="137">
+      <c r="G46" s="201">
         <v>365</v>
       </c>
-      <c r="H46" s="121" t="s">
+      <c r="H46" s="120" t="s">
         <v>26</v>
       </c>
-      <c r="I46" s="107">
+      <c r="I46" s="106">
         <v>383</v>
       </c>
-      <c r="J46" s="107">
+      <c r="J46" s="106">
         <v>381</v>
       </c>
-      <c r="K46" s="107">
+      <c r="K46" s="106">
         <v>380</v>
       </c>
-      <c r="L46" s="108">
+      <c r="L46" s="107">
         <v>381</v>
       </c>
-      <c r="M46" s="107">
+      <c r="M46" s="106">
         <v>378</v>
       </c>
-      <c r="N46" s="107">
+      <c r="N46" s="106">
         <v>376</v>
       </c>
-      <c r="O46" s="107">
+      <c r="O46" s="106">
         <v>374</v>
       </c>
-      <c r="P46" s="108">
+      <c r="P46" s="107">
         <v>376</v>
       </c>
-      <c r="Q46" s="107">
+      <c r="Q46" s="106">
         <v>372</v>
       </c>
-      <c r="R46" s="107">
+      <c r="R46" s="106">
         <v>370</v>
       </c>
-      <c r="S46" s="107">
+      <c r="S46" s="106">
         <v>371</v>
       </c>
-      <c r="T46" s="108">
+      <c r="T46" s="107">
         <v>371</v>
       </c>
-      <c r="U46" s="107">
+      <c r="U46" s="106">
         <v>372</v>
       </c>
-      <c r="V46" s="107">
+      <c r="V46" s="106">
         <v>371</v>
       </c>
-      <c r="W46" s="107">
+      <c r="W46" s="106">
         <v>371</v>
       </c>
-      <c r="X46" s="108">
+      <c r="X46" s="107">
         <v>371</v>
       </c>
     </row>
     <row r="47" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B47" s="187"/>
-      <c r="C47" s="128"/>
-      <c r="D47" s="150"/>
-      <c r="E47" s="151"/>
-      <c r="F47" s="152"/>
-      <c r="G47" s="137"/>
-      <c r="H47" s="121" t="s">
+      <c r="B47" s="148"/>
+      <c r="C47" s="163"/>
+      <c r="D47" s="153"/>
+      <c r="E47" s="233"/>
+      <c r="F47" s="234"/>
+      <c r="G47" s="201"/>
+      <c r="H47" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="I47" s="107">
+      <c r="I47" s="106">
         <v>366</v>
       </c>
-      <c r="J47" s="107">
+      <c r="J47" s="106">
         <v>366</v>
       </c>
-      <c r="K47" s="107">
+      <c r="K47" s="106">
         <v>366</v>
       </c>
-      <c r="L47" s="108">
+      <c r="L47" s="107">
         <v>366</v>
       </c>
-      <c r="M47" s="107">
+      <c r="M47" s="106">
         <v>366</v>
       </c>
-      <c r="N47" s="107">
+      <c r="N47" s="106">
         <v>366</v>
       </c>
-      <c r="O47" s="107">
+      <c r="O47" s="106">
         <v>366</v>
       </c>
-      <c r="P47" s="108">
+      <c r="P47" s="107">
         <v>366</v>
       </c>
-      <c r="Q47" s="107">
+      <c r="Q47" s="106">
         <v>366</v>
       </c>
-      <c r="R47" s="107">
+      <c r="R47" s="106">
         <v>366</v>
       </c>
-      <c r="S47" s="107">
+      <c r="S47" s="106">
         <v>366</v>
       </c>
-      <c r="T47" s="108">
+      <c r="T47" s="107">
         <v>366</v>
       </c>
-      <c r="U47" s="107">
+      <c r="U47" s="106">
         <v>366</v>
       </c>
-      <c r="V47" s="107">
+      <c r="V47" s="106">
         <v>366</v>
       </c>
-      <c r="W47" s="107">
+      <c r="W47" s="106">
         <v>366</v>
       </c>
-      <c r="X47" s="108">
+      <c r="X47" s="107">
         <v>366</v>
       </c>
       <c r="Y47" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="48" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B48" s="187"/>
-      <c r="C48" s="128"/>
-      <c r="D48" s="150"/>
-      <c r="E48" s="151"/>
-      <c r="F48" s="152"/>
-      <c r="G48" s="137"/>
-      <c r="H48" s="121" t="s">
+      <c r="B48" s="148"/>
+      <c r="C48" s="163"/>
+      <c r="D48" s="153"/>
+      <c r="E48" s="233"/>
+      <c r="F48" s="234"/>
+      <c r="G48" s="201"/>
+      <c r="H48" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I48" s="76">
@@ -5120,33 +5195,35 @@
       <c r="P48" s="96">
         <v>369</v>
       </c>
-      <c r="Q48" s="107"/>
-      <c r="R48" s="107"/>
-      <c r="S48" s="107"/>
-      <c r="T48" s="108"/>
-      <c r="U48" s="107"/>
-      <c r="V48" s="107"/>
-      <c r="W48" s="107"/>
-      <c r="X48" s="108"/>
+      <c r="Q48" s="87">
+        <v>363</v>
+      </c>
+      <c r="R48" s="106"/>
+      <c r="S48" s="106"/>
+      <c r="T48" s="107"/>
+      <c r="U48" s="106"/>
+      <c r="V48" s="106"/>
+      <c r="W48" s="106"/>
+      <c r="X48" s="107"/>
     </row>
     <row r="49" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B49" s="187"/>
-      <c r="C49" s="176" t="s">
-        <v>60</v>
-      </c>
-      <c r="D49" s="177" t="s">
-        <v>47</v>
-      </c>
-      <c r="E49" s="179">
+      <c r="B49" s="148"/>
+      <c r="C49" s="184" t="s">
+        <v>61</v>
+      </c>
+      <c r="D49" s="185" t="s">
+        <v>48</v>
+      </c>
+      <c r="E49" s="186">
         <v>0.71</v>
       </c>
-      <c r="F49" s="197">
+      <c r="F49" s="166">
         <v>0.92</v>
       </c>
-      <c r="G49" s="133">
+      <c r="G49" s="220">
         <v>0.72</v>
       </c>
-      <c r="H49" s="119" t="s">
+      <c r="H49" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I49" s="26">
@@ -5199,13 +5276,13 @@
       </c>
     </row>
     <row r="50" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B50" s="187"/>
-      <c r="C50" s="129"/>
-      <c r="D50" s="178"/>
-      <c r="E50" s="179"/>
-      <c r="F50" s="197"/>
-      <c r="G50" s="134"/>
-      <c r="H50" s="119" t="s">
+      <c r="B50" s="148"/>
+      <c r="C50" s="143"/>
+      <c r="D50" s="144"/>
+      <c r="E50" s="186"/>
+      <c r="F50" s="166"/>
+      <c r="G50" s="221"/>
+      <c r="H50" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I50" s="26">
@@ -5258,13 +5335,13 @@
       </c>
     </row>
     <row r="51" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B51" s="187"/>
-      <c r="C51" s="129"/>
-      <c r="D51" s="178"/>
-      <c r="E51" s="179"/>
-      <c r="F51" s="197"/>
-      <c r="G51" s="134"/>
-      <c r="H51" s="119" t="s">
+      <c r="B51" s="148"/>
+      <c r="C51" s="143"/>
+      <c r="D51" s="144"/>
+      <c r="E51" s="186"/>
+      <c r="F51" s="166"/>
+      <c r="G51" s="221"/>
+      <c r="H51" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I51" s="78">
@@ -5274,7 +5351,7 @@
         <v>0.6</v>
       </c>
       <c r="K51" s="78" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L51" s="95">
         <v>0.72</v>
@@ -5291,7 +5368,9 @@
       <c r="P51" s="95">
         <v>0.82</v>
       </c>
-      <c r="Q51" s="49"/>
+      <c r="Q51" s="78">
+        <v>0.89</v>
+      </c>
       <c r="R51" s="49"/>
       <c r="S51" s="49"/>
       <c r="T51" s="48"/>
@@ -5301,23 +5380,23 @@
       <c r="X51" s="27"/>
     </row>
     <row r="52" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B52" s="187"/>
-      <c r="C52" s="128" t="s">
-        <v>62</v>
-      </c>
-      <c r="D52" s="150" t="s">
-        <v>47</v>
-      </c>
-      <c r="E52" s="198" t="s">
+      <c r="B52" s="148"/>
+      <c r="C52" s="163" t="s">
+        <v>63</v>
+      </c>
+      <c r="D52" s="153" t="s">
+        <v>48</v>
+      </c>
+      <c r="E52" s="167" t="s">
         <v>35</v>
       </c>
-      <c r="F52" s="156" t="s">
-        <v>63</v>
-      </c>
-      <c r="G52" s="158">
+      <c r="F52" s="210" t="s">
+        <v>64</v>
+      </c>
+      <c r="G52" s="196">
         <v>0.28999999999999998</v>
       </c>
-      <c r="H52" s="121" t="s">
+      <c r="H52" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I52" s="24" t="s">
@@ -5373,58 +5452,58 @@
       </c>
     </row>
     <row r="53" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B53" s="187"/>
-      <c r="C53" s="128"/>
-      <c r="D53" s="150"/>
-      <c r="E53" s="198"/>
-      <c r="F53" s="157"/>
-      <c r="G53" s="158"/>
-      <c r="H53" s="121" t="s">
+      <c r="B53" s="148"/>
+      <c r="C53" s="163"/>
+      <c r="D53" s="153"/>
+      <c r="E53" s="167"/>
+      <c r="F53" s="193"/>
+      <c r="G53" s="196"/>
+      <c r="H53" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="I53" s="135"/>
-      <c r="J53" s="135"/>
-      <c r="K53" s="135"/>
-      <c r="L53" s="109" t="s">
-        <v>63</v>
-      </c>
-      <c r="M53" s="135"/>
-      <c r="N53" s="135"/>
-      <c r="O53" s="135"/>
-      <c r="P53" s="109" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q53" s="135"/>
-      <c r="R53" s="135"/>
-      <c r="S53" s="135"/>
-      <c r="T53" s="109" t="s">
-        <v>63</v>
-      </c>
-      <c r="U53" s="135"/>
-      <c r="V53" s="135"/>
-      <c r="W53" s="135"/>
-      <c r="X53" s="109" t="s">
-        <v>63</v>
+      <c r="I53" s="130"/>
+      <c r="J53" s="130"/>
+      <c r="K53" s="130"/>
+      <c r="L53" s="108" t="s">
+        <v>64</v>
+      </c>
+      <c r="M53" s="130"/>
+      <c r="N53" s="130"/>
+      <c r="O53" s="130"/>
+      <c r="P53" s="108" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q53" s="130"/>
+      <c r="R53" s="130"/>
+      <c r="S53" s="130"/>
+      <c r="T53" s="108" t="s">
+        <v>64</v>
+      </c>
+      <c r="U53" s="130"/>
+      <c r="V53" s="130"/>
+      <c r="W53" s="130"/>
+      <c r="X53" s="108" t="s">
+        <v>64</v>
       </c>
       <c r="Y53" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="54" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B54" s="187"/>
-      <c r="C54" s="128"/>
-      <c r="D54" s="150"/>
-      <c r="E54" s="198"/>
-      <c r="F54" s="157"/>
-      <c r="G54" s="158"/>
-      <c r="H54" s="121" t="s">
+      <c r="B54" s="148"/>
+      <c r="C54" s="163"/>
+      <c r="D54" s="153"/>
+      <c r="E54" s="167"/>
+      <c r="F54" s="193"/>
+      <c r="G54" s="196"/>
+      <c r="H54" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I54" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J54" s="24" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K54" s="24">
         <v>0.28799999999999998</v>
@@ -5444,7 +5523,9 @@
       <c r="P54" s="95">
         <v>0.16</v>
       </c>
-      <c r="Q54" s="24"/>
+      <c r="Q54" s="24">
+        <v>0.214</v>
+      </c>
       <c r="R54" s="24"/>
       <c r="S54" s="24"/>
       <c r="T54" s="25"/>
@@ -5454,25 +5535,25 @@
       <c r="X54" s="25"/>
     </row>
     <row r="55" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B55" s="187"/>
-      <c r="C55" s="129" t="s">
-        <v>67</v>
-      </c>
-      <c r="D55" s="178" t="s">
+      <c r="B55" s="148"/>
+      <c r="C55" s="143" t="s">
         <v>68</v>
       </c>
-      <c r="E55" s="213">
+      <c r="D55" s="144" t="s">
+        <v>69</v>
+      </c>
+      <c r="E55" s="145">
         <f>X55</f>
         <v>40</v>
       </c>
-      <c r="F55" s="196">
+      <c r="F55" s="165">
         <v>55</v>
       </c>
-      <c r="G55" s="136">
+      <c r="G55" s="222">
         <f>X57</f>
-        <v>42</v>
-      </c>
-      <c r="H55" s="119" t="s">
+        <v>44</v>
+      </c>
+      <c r="H55" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I55" s="15">
@@ -5525,117 +5606,119 @@
       </c>
     </row>
     <row r="56" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B56" s="187"/>
-      <c r="C56" s="129"/>
-      <c r="D56" s="178"/>
-      <c r="E56" s="213"/>
-      <c r="F56" s="196"/>
-      <c r="G56" s="136"/>
-      <c r="H56" s="119" t="s">
+      <c r="B56" s="148"/>
+      <c r="C56" s="143"/>
+      <c r="D56" s="144"/>
+      <c r="E56" s="145"/>
+      <c r="F56" s="165"/>
+      <c r="G56" s="222"/>
+      <c r="H56" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I56" s="153" t="s">
-        <v>32</v>
-      </c>
-      <c r="J56" s="153"/>
-      <c r="K56" s="153"/>
+      <c r="I56" s="208" t="s">
+        <v>32</v>
+      </c>
+      <c r="J56" s="208"/>
+      <c r="K56" s="208"/>
       <c r="L56" s="18">
         <v>13</v>
       </c>
-      <c r="M56" s="153" t="s">
-        <v>32</v>
-      </c>
-      <c r="N56" s="153"/>
-      <c r="O56" s="153"/>
+      <c r="M56" s="208" t="s">
+        <v>32</v>
+      </c>
+      <c r="N56" s="208"/>
+      <c r="O56" s="208"/>
       <c r="P56" s="18">
         <v>27</v>
       </c>
-      <c r="Q56" s="153" t="s">
-        <v>32</v>
-      </c>
-      <c r="R56" s="153"/>
-      <c r="S56" s="153"/>
+      <c r="Q56" s="208" t="s">
+        <v>32</v>
+      </c>
+      <c r="R56" s="208"/>
+      <c r="S56" s="208"/>
       <c r="T56" s="18">
         <v>41</v>
       </c>
-      <c r="U56" s="153" t="s">
-        <v>32</v>
-      </c>
-      <c r="V56" s="153"/>
-      <c r="W56" s="153"/>
+      <c r="U56" s="208" t="s">
+        <v>32</v>
+      </c>
+      <c r="V56" s="208"/>
+      <c r="W56" s="208"/>
       <c r="X56" s="18">
         <v>55</v>
       </c>
     </row>
     <row r="57" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B57" s="187"/>
-      <c r="C57" s="129"/>
-      <c r="D57" s="178"/>
-      <c r="E57" s="213"/>
-      <c r="F57" s="196"/>
-      <c r="G57" s="136"/>
-      <c r="H57" s="119" t="s">
+      <c r="B57" s="148"/>
+      <c r="C57" s="143"/>
+      <c r="D57" s="144"/>
+      <c r="E57" s="145"/>
+      <c r="F57" s="165"/>
+      <c r="G57" s="222"/>
+      <c r="H57" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="I57" s="110">
-        <v>0</v>
-      </c>
-      <c r="J57" s="110">
-        <v>0</v>
-      </c>
-      <c r="K57" s="110">
+      <c r="I57" s="109">
+        <v>0</v>
+      </c>
+      <c r="J57" s="109">
+        <v>0</v>
+      </c>
+      <c r="K57" s="109">
         <v>17</v>
       </c>
       <c r="L57" s="90">
         <v>17</v>
       </c>
-      <c r="M57" s="110">
+      <c r="M57" s="109">
         <v>25</v>
       </c>
-      <c r="N57" s="110">
-        <v>0</v>
-      </c>
-      <c r="O57" s="110">
-        <v>0</v>
-      </c>
-      <c r="P57" s="115">
+      <c r="N57" s="109">
+        <v>0</v>
+      </c>
+      <c r="O57" s="109">
+        <v>0</v>
+      </c>
+      <c r="P57" s="114">
         <v>42</v>
       </c>
-      <c r="Q57" s="110"/>
-      <c r="R57" s="110"/>
-      <c r="S57" s="110"/>
-      <c r="T57" s="111">
+      <c r="Q57" s="109">
+        <v>2</v>
+      </c>
+      <c r="R57" s="109"/>
+      <c r="S57" s="109"/>
+      <c r="T57" s="110">
         <f>SUM(P57:S57)</f>
-        <v>42</v>
-      </c>
-      <c r="U57" s="110"/>
-      <c r="V57" s="110"/>
-      <c r="W57" s="110"/>
-      <c r="X57" s="111">
+        <v>44</v>
+      </c>
+      <c r="U57" s="109"/>
+      <c r="V57" s="109"/>
+      <c r="W57" s="109"/>
+      <c r="X57" s="110">
         <f>SUM(T57:W57)</f>
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="58" spans="2:25" ht="15" hidden="1" customHeight="1">
-      <c r="B58" s="186" t="s">
-        <v>69</v>
-      </c>
-      <c r="C58" s="188" t="s">
+      <c r="B58" s="147" t="s">
         <v>70</v>
       </c>
-      <c r="D58" s="191" t="s">
+      <c r="C58" s="156" t="s">
         <v>71</v>
       </c>
-      <c r="E58" s="220">
+      <c r="D58" s="159" t="s">
+        <v>72</v>
+      </c>
+      <c r="E58" s="135">
         <v>92.5</v>
       </c>
-      <c r="F58" s="229">
+      <c r="F58" s="132">
         <v>93</v>
       </c>
-      <c r="G58" s="220">
+      <c r="G58" s="135">
         <v>92.5</v>
       </c>
-      <c r="H58" s="121" t="s">
+      <c r="H58" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I58" s="34">
@@ -5687,17 +5770,17 @@
         <v>92.5</v>
       </c>
       <c r="Y58" s="37" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="59" spans="2:25" ht="15" hidden="1" customHeight="1">
-      <c r="B59" s="187"/>
-      <c r="C59" s="189"/>
-      <c r="D59" s="192"/>
-      <c r="E59" s="221"/>
-      <c r="F59" s="230"/>
-      <c r="G59" s="221"/>
-      <c r="H59" s="121" t="s">
+      <c r="B59" s="148"/>
+      <c r="C59" s="157"/>
+      <c r="D59" s="160"/>
+      <c r="E59" s="136"/>
+      <c r="F59" s="133"/>
+      <c r="G59" s="136"/>
+      <c r="H59" s="120" t="s">
         <v>27</v>
       </c>
       <c r="I59" s="19">
@@ -5749,17 +5832,17 @@
         <v>93</v>
       </c>
       <c r="Y59" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="60" spans="2:25" ht="15" hidden="1" customHeight="1">
-      <c r="B60" s="187"/>
-      <c r="C60" s="190"/>
-      <c r="D60" s="193"/>
-      <c r="E60" s="222"/>
-      <c r="F60" s="231"/>
-      <c r="G60" s="222"/>
-      <c r="H60" s="121" t="s">
+      <c r="B60" s="148"/>
+      <c r="C60" s="158"/>
+      <c r="D60" s="161"/>
+      <c r="E60" s="137"/>
+      <c r="F60" s="134"/>
+      <c r="G60" s="137"/>
+      <c r="H60" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I60" s="36">
@@ -5777,33 +5860,33 @@
       <c r="S60" s="22"/>
       <c r="T60" s="20"/>
       <c r="U60" s="22"/>
-      <c r="V60" s="104"/>
-      <c r="W60" s="104"/>
+      <c r="V60" s="103"/>
+      <c r="W60" s="103"/>
       <c r="X60" s="20"/>
     </row>
     <row r="61" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B61" s="186" t="s">
-        <v>74</v>
-      </c>
-      <c r="C61" s="214" t="s">
+      <c r="B61" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="D61" s="150" t="s">
+      <c r="C61" s="146" t="s">
+        <v>76</v>
+      </c>
+      <c r="D61" s="153" t="s">
         <v>39</v>
       </c>
-      <c r="E61" s="219">
+      <c r="E61" s="154">
         <f>L61+P61+T61+X61</f>
         <v>30.187825999999998</v>
       </c>
-      <c r="F61" s="233">
+      <c r="F61" s="139">
         <f>SUM(L62,P62,T62,X62)</f>
         <v>28</v>
       </c>
-      <c r="G61" s="228">
+      <c r="G61" s="131">
         <f>L63+P63+T63+X63</f>
-        <v>11.850283999999998</v>
-      </c>
-      <c r="H61" s="121" t="s">
+        <v>14.112583999999998</v>
+      </c>
+      <c r="H61" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I61" s="70">
@@ -5859,123 +5942,125 @@
       </c>
     </row>
     <row r="62" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B62" s="187"/>
-      <c r="C62" s="214"/>
-      <c r="D62" s="150"/>
-      <c r="E62" s="219"/>
-      <c r="F62" s="233"/>
-      <c r="G62" s="228"/>
-      <c r="H62" s="121" t="s">
+      <c r="B62" s="148"/>
+      <c r="C62" s="146"/>
+      <c r="D62" s="153"/>
+      <c r="E62" s="154"/>
+      <c r="F62" s="139"/>
+      <c r="G62" s="131"/>
+      <c r="H62" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="I62" s="135" t="s">
-        <v>32</v>
-      </c>
-      <c r="J62" s="135"/>
-      <c r="K62" s="135"/>
+      <c r="I62" s="130" t="s">
+        <v>32</v>
+      </c>
+      <c r="J62" s="130"/>
+      <c r="K62" s="130"/>
       <c r="L62" s="71">
         <v>5</v>
       </c>
-      <c r="M62" s="135" t="s">
-        <v>32</v>
-      </c>
-      <c r="N62" s="135"/>
-      <c r="O62" s="135"/>
+      <c r="M62" s="130" t="s">
+        <v>32</v>
+      </c>
+      <c r="N62" s="130"/>
+      <c r="O62" s="130"/>
       <c r="P62" s="71">
         <v>7</v>
       </c>
-      <c r="Q62" s="135" t="s">
-        <v>32</v>
-      </c>
-      <c r="R62" s="135"/>
-      <c r="S62" s="135"/>
+      <c r="Q62" s="130" t="s">
+        <v>32</v>
+      </c>
+      <c r="R62" s="130"/>
+      <c r="S62" s="130"/>
       <c r="T62" s="71">
         <v>7</v>
       </c>
       <c r="U62" s="71" t="s">
         <v>32</v>
       </c>
-      <c r="V62" s="117"/>
-      <c r="W62" s="117"/>
+      <c r="V62" s="119"/>
+      <c r="W62" s="119"/>
       <c r="X62" s="71">
         <v>9</v>
       </c>
     </row>
     <row r="63" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B63" s="187"/>
-      <c r="C63" s="214"/>
-      <c r="D63" s="150"/>
-      <c r="E63" s="219"/>
-      <c r="F63" s="233"/>
-      <c r="G63" s="228"/>
-      <c r="H63" s="121" t="s">
+      <c r="B63" s="148"/>
+      <c r="C63" s="146"/>
+      <c r="D63" s="153"/>
+      <c r="E63" s="154"/>
+      <c r="F63" s="139"/>
+      <c r="G63" s="131"/>
+      <c r="H63" s="120" t="s">
         <v>28</v>
       </c>
-      <c r="I63" s="117">
+      <c r="I63" s="119">
         <v>1.333</v>
       </c>
-      <c r="J63" s="117">
+      <c r="J63" s="119">
         <v>1.4</v>
       </c>
-      <c r="K63" s="117">
+      <c r="K63" s="119">
         <v>2.5</v>
       </c>
       <c r="L63" s="91">
         <f>K63+J63+I63</f>
         <v>5.2329999999999997</v>
       </c>
-      <c r="M63" s="117">
+      <c r="M63" s="119">
         <v>1.5</v>
       </c>
-      <c r="N63" s="117">
+      <c r="N63" s="119">
         <v>3.2572839999999998</v>
       </c>
-      <c r="O63" s="117">
+      <c r="O63" s="119">
         <v>1.86</v>
       </c>
-      <c r="P63" s="114">
+      <c r="P63" s="113">
         <f>O63+N63+M63</f>
         <v>6.6172839999999997</v>
       </c>
-      <c r="Q63" s="117"/>
-      <c r="R63" s="117"/>
-      <c r="S63" s="117"/>
+      <c r="Q63" s="119">
+        <v>2.2623000000000002</v>
+      </c>
+      <c r="R63" s="119"/>
+      <c r="S63" s="119"/>
       <c r="T63" s="92">
         <f>S63+R63+Q63</f>
-        <v>0</v>
-      </c>
-      <c r="U63" s="117"/>
-      <c r="V63" s="117"/>
-      <c r="W63" s="117"/>
+        <v>2.2623000000000002</v>
+      </c>
+      <c r="U63" s="119"/>
+      <c r="V63" s="119"/>
+      <c r="W63" s="119"/>
       <c r="X63" s="92">
         <f>W63+V63+U63</f>
         <v>0</v>
       </c>
       <c r="Y63" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="64" spans="2:25" ht="15.6">
-      <c r="B64" s="187"/>
-      <c r="C64" s="210" t="s">
-        <v>77</v>
-      </c>
-      <c r="D64" s="211" t="s">
+      <c r="B64" s="148"/>
+      <c r="C64" s="140" t="s">
         <v>78</v>
       </c>
-      <c r="E64" s="212">
+      <c r="D64" s="141" t="s">
+        <v>79</v>
+      </c>
+      <c r="E64" s="142">
         <f>L64+P64+T64+X64</f>
         <v>-8.4644727175232077</v>
       </c>
-      <c r="F64" s="232">
+      <c r="F64" s="138">
         <f>SUM(L65,P65,T65,X65)</f>
         <v>-7.0189285867816498</v>
       </c>
-      <c r="G64" s="227">
-        <f>SUM(L66,P66,T66,X66)</f>
-        <v>-3.8762228984112506</v>
-      </c>
-      <c r="H64" s="118" t="s">
+      <c r="G64" s="129">
+        <f>SUM(L66,P66,T66,Q66,X66)</f>
+        <v>-5.8522190000397307</v>
+      </c>
+      <c r="H64" s="122" t="s">
         <v>26</v>
       </c>
       <c r="I64" s="72">
@@ -6032,13 +6117,13 @@
       </c>
     </row>
     <row r="65" spans="2:24" ht="15.6">
-      <c r="B65" s="187"/>
-      <c r="C65" s="210"/>
-      <c r="D65" s="211"/>
-      <c r="E65" s="212"/>
-      <c r="F65" s="232"/>
-      <c r="G65" s="227"/>
-      <c r="H65" s="118" t="s">
+      <c r="B65" s="148"/>
+      <c r="C65" s="140"/>
+      <c r="D65" s="141"/>
+      <c r="E65" s="142"/>
+      <c r="F65" s="138"/>
+      <c r="G65" s="129"/>
+      <c r="H65" s="122" t="s">
         <v>27</v>
       </c>
       <c r="I65" s="72">
@@ -6095,13 +6180,13 @@
       </c>
     </row>
     <row r="66" spans="2:24" ht="15.6">
-      <c r="B66" s="187"/>
-      <c r="C66" s="210"/>
-      <c r="D66" s="211"/>
-      <c r="E66" s="212"/>
-      <c r="F66" s="232"/>
-      <c r="G66" s="227"/>
-      <c r="H66" s="118" t="s">
+      <c r="B66" s="148"/>
+      <c r="C66" s="140"/>
+      <c r="D66" s="141"/>
+      <c r="E66" s="142"/>
+      <c r="F66" s="138"/>
+      <c r="G66" s="129"/>
+      <c r="H66" s="122" t="s">
         <v>28</v>
       </c>
       <c r="I66" s="82">
@@ -6130,42 +6215,44 @@
         <f>SUM(M66:O66)</f>
         <v>-1.7762228984112503</v>
       </c>
-      <c r="Q66" s="72"/>
+      <c r="Q66" s="82">
+        <v>-0.98799805081423986</v>
+      </c>
       <c r="R66" s="72"/>
       <c r="S66" s="72"/>
-      <c r="T66" s="112">
+      <c r="T66" s="111">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-0.98799805081423986</v>
       </c>
       <c r="U66" s="72"/>
       <c r="V66" s="72"/>
       <c r="W66" s="72"/>
-      <c r="X66" s="112">
+      <c r="X66" s="111">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
     <row r="67" spans="2:24" ht="15" customHeight="1">
-      <c r="B67" s="187"/>
-      <c r="C67" s="216" t="s">
+      <c r="B67" s="148"/>
+      <c r="C67" s="150" t="s">
+        <v>80</v>
+      </c>
+      <c r="D67" s="151" t="s">
         <v>79</v>
       </c>
-      <c r="D67" s="217" t="s">
-        <v>78</v>
-      </c>
-      <c r="E67" s="218">
+      <c r="E67" s="152">
         <f>L67+P67+T67+X67</f>
         <v>-20.34262829557931</v>
       </c>
-      <c r="F67" s="223">
+      <c r="F67" s="125">
         <f>SUM(L68,P68,T68,X68)</f>
         <v>-24.141371751369434</v>
       </c>
-      <c r="G67" s="226">
+      <c r="G67" s="128">
         <f>SUM(L69,P69,T69,X69)</f>
-        <v>-11.6</v>
-      </c>
-      <c r="H67" s="120" t="s">
+        <v>-14.40318635548517</v>
+      </c>
+      <c r="H67" s="123" t="s">
         <v>26</v>
       </c>
       <c r="I67" s="74">
@@ -6222,13 +6309,13 @@
       </c>
     </row>
     <row r="68" spans="2:24" ht="15" customHeight="1">
-      <c r="B68" s="187"/>
-      <c r="C68" s="216"/>
-      <c r="D68" s="217"/>
-      <c r="E68" s="218"/>
-      <c r="F68" s="224"/>
-      <c r="G68" s="226"/>
-      <c r="H68" s="120" t="s">
+      <c r="B68" s="148"/>
+      <c r="C68" s="150"/>
+      <c r="D68" s="151"/>
+      <c r="E68" s="152"/>
+      <c r="F68" s="126"/>
+      <c r="G68" s="128"/>
+      <c r="H68" s="123" t="s">
         <v>27</v>
       </c>
       <c r="I68" s="74">
@@ -6285,13 +6372,13 @@
       </c>
     </row>
     <row r="69" spans="2:24" ht="15" customHeight="1">
-      <c r="B69" s="215"/>
-      <c r="C69" s="216"/>
-      <c r="D69" s="217"/>
-      <c r="E69" s="218"/>
-      <c r="F69" s="225"/>
-      <c r="G69" s="226"/>
-      <c r="H69" s="120" t="s">
+      <c r="B69" s="149"/>
+      <c r="C69" s="150"/>
+      <c r="D69" s="151"/>
+      <c r="E69" s="152"/>
+      <c r="F69" s="127"/>
+      <c r="G69" s="128"/>
+      <c r="H69" s="123" t="s">
         <v>28</v>
       </c>
       <c r="I69" s="89">
@@ -6316,21 +6403,23 @@
       <c r="O69" s="89">
         <v>-1.4</v>
       </c>
-      <c r="P69" s="116">
+      <c r="P69" s="115">
         <f t="shared" si="9"/>
         <v>-6.6</v>
       </c>
-      <c r="Q69" s="74"/>
+      <c r="Q69" s="82">
+        <v>-2.8031863554851699</v>
+      </c>
       <c r="R69" s="74"/>
       <c r="S69" s="74"/>
-      <c r="T69" s="113">
+      <c r="T69" s="112">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-2.8031863554851699</v>
       </c>
       <c r="U69" s="74"/>
       <c r="V69" s="74"/>
       <c r="W69" s="74"/>
-      <c r="X69" s="113">
+      <c r="X69" s="112">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -6349,31 +6438,84 @@
     </row>
   </sheetData>
   <mergeCells count="127">
-    <mergeCell ref="F67:F69"/>
-    <mergeCell ref="G67:G69"/>
-    <mergeCell ref="G64:G66"/>
-    <mergeCell ref="M62:O62"/>
-    <mergeCell ref="Q62:S62"/>
-    <mergeCell ref="G61:G63"/>
-    <mergeCell ref="F58:F60"/>
-    <mergeCell ref="G58:G60"/>
-    <mergeCell ref="I62:K62"/>
-    <mergeCell ref="F64:F66"/>
-    <mergeCell ref="F61:F63"/>
-    <mergeCell ref="C64:C66"/>
-    <mergeCell ref="D64:D66"/>
-    <mergeCell ref="E64:E66"/>
-    <mergeCell ref="C55:C57"/>
-    <mergeCell ref="D55:D57"/>
-    <mergeCell ref="E55:E57"/>
-    <mergeCell ref="C61:C63"/>
-    <mergeCell ref="B61:B69"/>
-    <mergeCell ref="C67:C69"/>
-    <mergeCell ref="D67:D69"/>
-    <mergeCell ref="E67:E69"/>
-    <mergeCell ref="D61:D63"/>
-    <mergeCell ref="E61:E63"/>
-    <mergeCell ref="E58:E60"/>
+    <mergeCell ref="G19:G21"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="D19:D21"/>
+    <mergeCell ref="E19:E21"/>
+    <mergeCell ref="G49:G51"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="G55:G57"/>
+    <mergeCell ref="G22:G24"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="D37:D39"/>
+    <mergeCell ref="F19:F21"/>
+    <mergeCell ref="F22:F24"/>
+    <mergeCell ref="F31:F33"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="D43:D45"/>
+    <mergeCell ref="F28:F30"/>
+    <mergeCell ref="G28:G30"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="F46:F48"/>
+    <mergeCell ref="G46:G48"/>
+    <mergeCell ref="M56:O56"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="Q56:S56"/>
+    <mergeCell ref="U56:W56"/>
+    <mergeCell ref="M53:O53"/>
+    <mergeCell ref="Q53:S53"/>
+    <mergeCell ref="U53:W53"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="F34:F36"/>
+    <mergeCell ref="F52:F54"/>
+    <mergeCell ref="G52:G54"/>
+    <mergeCell ref="F40:F42"/>
+    <mergeCell ref="G40:G42"/>
+    <mergeCell ref="E43:E45"/>
+    <mergeCell ref="F43:F45"/>
+    <mergeCell ref="G43:G45"/>
+    <mergeCell ref="E37:E39"/>
+    <mergeCell ref="F37:F39"/>
+    <mergeCell ref="G37:G39"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="D22:D24"/>
+    <mergeCell ref="E22:E24"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="D28:D30"/>
+    <mergeCell ref="E28:E30"/>
+    <mergeCell ref="I2:X2"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="D49:D51"/>
+    <mergeCell ref="E49:E51"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="E31:E33"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="G4:G6"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="F10:F12"/>
+    <mergeCell ref="G10:G12"/>
+    <mergeCell ref="F7:F9"/>
+    <mergeCell ref="G31:G33"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="G7:G9"/>
+    <mergeCell ref="G34:G36"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="F13:F15"/>
     <mergeCell ref="G13:G15"/>
     <mergeCell ref="B58:B60"/>
     <mergeCell ref="C58:C60"/>
@@ -6398,84 +6540,31 @@
     <mergeCell ref="B4:B18"/>
     <mergeCell ref="C31:C33"/>
     <mergeCell ref="C10:C12"/>
-    <mergeCell ref="I2:X2"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="D49:D51"/>
-    <mergeCell ref="E49:E51"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="D31:D33"/>
-    <mergeCell ref="E31:E33"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="D16:D18"/>
-    <mergeCell ref="G4:G6"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="F10:F12"/>
-    <mergeCell ref="G10:G12"/>
-    <mergeCell ref="F7:F9"/>
-    <mergeCell ref="G31:G33"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="F16:F18"/>
-    <mergeCell ref="G7:G9"/>
-    <mergeCell ref="G34:G36"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="F13:F15"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="E10:E12"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="D22:D24"/>
-    <mergeCell ref="E22:E24"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="D28:D30"/>
-    <mergeCell ref="E28:E30"/>
-    <mergeCell ref="M56:O56"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="Q56:S56"/>
-    <mergeCell ref="U56:W56"/>
-    <mergeCell ref="M53:O53"/>
-    <mergeCell ref="Q53:S53"/>
-    <mergeCell ref="U53:W53"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="F34:F36"/>
-    <mergeCell ref="F52:F54"/>
-    <mergeCell ref="G52:G54"/>
-    <mergeCell ref="F40:F42"/>
-    <mergeCell ref="G40:G42"/>
-    <mergeCell ref="E43:E45"/>
-    <mergeCell ref="F43:F45"/>
-    <mergeCell ref="G43:G45"/>
-    <mergeCell ref="E37:E39"/>
-    <mergeCell ref="F37:F39"/>
-    <mergeCell ref="G37:G39"/>
-    <mergeCell ref="G19:G21"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="C19:C21"/>
-    <mergeCell ref="D19:D21"/>
-    <mergeCell ref="E19:E21"/>
-    <mergeCell ref="G49:G51"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="G55:G57"/>
-    <mergeCell ref="G22:G24"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="D37:D39"/>
-    <mergeCell ref="F19:F21"/>
-    <mergeCell ref="F22:F24"/>
-    <mergeCell ref="F31:F33"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="D43:D45"/>
-    <mergeCell ref="F28:F30"/>
-    <mergeCell ref="G28:G30"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="F46:F48"/>
-    <mergeCell ref="G46:G48"/>
+    <mergeCell ref="C64:C66"/>
+    <mergeCell ref="D64:D66"/>
+    <mergeCell ref="E64:E66"/>
+    <mergeCell ref="C55:C57"/>
+    <mergeCell ref="D55:D57"/>
+    <mergeCell ref="E55:E57"/>
+    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="B61:B69"/>
+    <mergeCell ref="C67:C69"/>
+    <mergeCell ref="D67:D69"/>
+    <mergeCell ref="E67:E69"/>
+    <mergeCell ref="D61:D63"/>
+    <mergeCell ref="E61:E63"/>
+    <mergeCell ref="E58:E60"/>
+    <mergeCell ref="F67:F69"/>
+    <mergeCell ref="G67:G69"/>
+    <mergeCell ref="G64:G66"/>
+    <mergeCell ref="M62:O62"/>
+    <mergeCell ref="Q62:S62"/>
+    <mergeCell ref="G61:G63"/>
+    <mergeCell ref="F58:F60"/>
+    <mergeCell ref="G58:G60"/>
+    <mergeCell ref="I62:K62"/>
+    <mergeCell ref="F64:F66"/>
+    <mergeCell ref="F61:F63"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6496,55 +6585,55 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="29.1">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="28.9">
       <c r="A3" s="31" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="41" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B4" s="41" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="29.1">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="28.9">
       <c r="A5" s="41" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B5" s="41" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="62" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B6" s="62" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="31" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.6">
       <c r="A8" s="64" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B8" s="64"/>
       <c r="C8" s="30"/>
@@ -6554,7 +6643,7 @@
     </row>
     <row r="9" spans="1:6" ht="15.6">
       <c r="A9" s="64" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B9" s="64"/>
       <c r="C9" s="30"/>
@@ -6562,24 +6651,24 @@
       <c r="E9" s="30"/>
       <c r="F9" s="30"/>
     </row>
-    <row r="10" spans="1:6" ht="77.45">
+    <row r="10" spans="1:6" ht="78">
       <c r="A10" s="42" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B10" s="42" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C10" s="30"/>
       <c r="D10" s="30"/>
       <c r="E10" s="30"/>
       <c r="F10" s="30"/>
     </row>
-    <row r="11" spans="1:6" ht="46.5">
+    <row r="11" spans="1:6" ht="46.9">
       <c r="A11" s="42" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B11" s="42" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C11" s="30"/>
       <c r="D11" s="30"/>
@@ -6588,25 +6677,25 @@
     </row>
     <row r="12" spans="1:6" ht="15.6">
       <c r="A12" s="62" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C12" s="30"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="62" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.6">
       <c r="A14" s="31" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C14" s="30"/>
       <c r="D14" s="30"/>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="31" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -6626,26 +6715,26 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="F1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="B2" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="B3" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:6" outlineLevel="1">
@@ -6653,35 +6742,35 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:6" outlineLevel="1">
       <c r="B5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:6" outlineLevel="1">
       <c r="B6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:6" outlineLevel="1">
       <c r="B7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -6808,10 +6897,10 @@
     </row>
     <row r="26" spans="1:4">
       <c r="B26" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D26" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -6901,15 +6990,15 @@
     </row>
     <row r="44" spans="1:3">
       <c r="B44" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C44" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Preview: Week of 2026-08-17 — built 2026-08-14T11:45:50Z
</commit_message>
<xml_diff>
--- a/data/2026 Bowler Chart - OFS Training.xlsx
+++ b/data/2026 Bowler Chart - OFS Training.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\212668250\Box\OFS Global Technical Training @OFFICIAL NEW\Leadership Team\Bowler\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\212448292\AppData\Local\Box\Box Edit\Documents\yHKq1N8p9kanefDTz1B5ig==\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{D179DAEC-2DD2-40E5-A694-294F48291E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE4DF51E-D74C-4227-811D-516419DA60D5}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{A0FF72AF-E087-4B8F-939D-96A71C71115B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{099FC471-C0B4-45E1-B458-985519A21C3B}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="601" xr2:uid="{8476BB21-6D10-4BB9-B6CE-FEFD481D0662}"/>
+    <workbookView xWindow="-23148" yWindow="-48" windowWidth="23256" windowHeight="12456" tabRatio="601" xr2:uid="{8476BB21-6D10-4BB9-B6CE-FEFD481D0662}"/>
   </bookViews>
   <sheets>
     <sheet name="Bowler L1 Training" sheetId="16" r:id="rId1"/>
@@ -40,15 +40,28 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={06BE996C-F791-4A9F-AA6D-EE2A8EE2F4C3}</author>
     <author>Jen Wright</author>
+    <author>tc={17407CA0-19D6-410B-BD94-9BBC65BFCC7C}</author>
     <author>tc={160740E7-DFEB-4450-B5C5-A17286B215D6}</author>
     <author>Philip Ganssmann</author>
     <author>tc={50577B9E-D913-49BB-B91E-A5BD3E934319}</author>
     <author>tc={4A61949D-D058-4614-9CBE-136784BCC6E7}</author>
     <author>tc={40736F15-DF93-4810-BC49-A79E1FB56ED1}</author>
+    <author>tc={F644D89E-1836-4B19-B5E0-2664B9B5862D}</author>
   </authors>
   <commentList>
-    <comment ref="F7" authorId="0" shapeId="0" xr:uid="{6BB47BF6-B4F0-44A1-B661-DC1F618CF875}">
+    <comment ref="Q6" authorId="0" shapeId="0" xr:uid="{06BE996C-F791-4A9F-AA6D-EE2A8EE2F4C3}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    BLC: Lost Time Injury - Fall Event 7/21/2026. Recordable 
+Reply:
+    PSE Near Miss: HLC 7HA.03 Project Post Lift Operation Failure</t>
+      </text>
+    </comment>
+    <comment ref="F7" authorId="1" shapeId="0" xr:uid="{6BB47BF6-B4F0-44A1-B661-DC1F618CF875}">
       <text>
         <r>
           <rPr>
@@ -64,7 +77,17 @@
         </r>
       </text>
     </comment>
-    <comment ref="F13" authorId="1" shapeId="0" xr:uid="{160740E7-DFEB-4450-B5C5-A17286B215D6}">
+    <comment ref="Q9" authorId="2" shapeId="0" xr:uid="{17407CA0-19D6-410B-BD94-9BBC65BFCC7C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    1 X 200000/183589.43=1.089
+Reply:
+    I&amp;I FW 33 1.089</t>
+      </text>
+    </comment>
+    <comment ref="F13" authorId="3" shapeId="0" xr:uid="{160740E7-DFEB-4450-B5C5-A17286B215D6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -72,7 +95,7 @@
     90% RA ATS closure rate all sites by YE</t>
       </text>
     </comment>
-    <comment ref="I24" authorId="2" shapeId="0" xr:uid="{295EE1B2-A25B-412E-A639-7B1259576743}">
+    <comment ref="I24" authorId="4" shapeId="0" xr:uid="{295EE1B2-A25B-412E-A639-7B1259576743}">
       <text>
         <r>
           <rPr>
@@ -87,7 +110,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J24" authorId="2" shapeId="0" xr:uid="{DC09360C-6AE1-46FC-ABAD-4D81C3945042}">
+    <comment ref="J24" authorId="4" shapeId="0" xr:uid="{DC09360C-6AE1-46FC-ABAD-4D81C3945042}">
       <text>
         <r>
           <rPr>
@@ -106,7 +129,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K24" authorId="2" shapeId="0" xr:uid="{64E9CAD9-580E-40D0-B2F1-25AC4998B65A}">
+    <comment ref="K24" authorId="4" shapeId="0" xr:uid="{64E9CAD9-580E-40D0-B2F1-25AC4998B65A}">
       <text>
         <r>
           <rPr>
@@ -123,7 +146,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N24" authorId="2" shapeId="0" xr:uid="{7B5163D0-287F-484F-B9B7-4BE35DBAC943}">
+    <comment ref="N24" authorId="4" shapeId="0" xr:uid="{7B5163D0-287F-484F-B9B7-4BE35DBAC943}">
       <text>
         <r>
           <rPr>
@@ -140,7 +163,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I27" authorId="2" shapeId="0" xr:uid="{90DAD1A6-212D-45E4-8528-2D901E1C0C5A}">
+    <comment ref="I27" authorId="4" shapeId="0" xr:uid="{90DAD1A6-212D-45E4-8528-2D901E1C0C5A}">
       <text>
         <r>
           <rPr>
@@ -155,7 +178,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J27" authorId="2" shapeId="0" xr:uid="{7392AAE5-E54D-4232-B7DC-129B156C6F62}">
+    <comment ref="J27" authorId="4" shapeId="0" xr:uid="{7392AAE5-E54D-4232-B7DC-129B156C6F62}">
       <text>
         <r>
           <rPr>
@@ -182,7 +205,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K27" authorId="2" shapeId="0" xr:uid="{76FCDDC0-41DD-4A57-9E0C-979F0DC1595C}">
+    <comment ref="K27" authorId="4" shapeId="0" xr:uid="{76FCDDC0-41DD-4A57-9E0C-979F0DC1595C}">
       <text>
         <r>
           <rPr>
@@ -209,7 +232,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L27" authorId="2" shapeId="0" xr:uid="{C1388240-DDDB-4DD1-B7FE-11B7EF9BDF13}">
+    <comment ref="L27" authorId="4" shapeId="0" xr:uid="{C1388240-DDDB-4DD1-B7FE-11B7EF9BDF13}">
       <text>
         <r>
           <rPr>
@@ -236,7 +259,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C28" authorId="0" shapeId="0" xr:uid="{62BE848F-A00E-4544-8BD6-953D94ED5EF8}">
+    <comment ref="C28" authorId="1" shapeId="0" xr:uid="{62BE848F-A00E-4544-8BD6-953D94ED5EF8}">
       <text>
         <r>
           <rPr>
@@ -251,7 +274,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C34" authorId="0" shapeId="0" xr:uid="{508037C5-7575-470A-939A-71BD192D06EF}">
+    <comment ref="C34" authorId="1" shapeId="0" xr:uid="{508037C5-7575-470A-939A-71BD192D06EF}">
       <text>
         <r>
           <rPr>
@@ -266,7 +289,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C37" authorId="0" shapeId="0" xr:uid="{04C7CFAE-132D-4578-AA1A-A2AED2C7F976}">
+    <comment ref="C37" authorId="1" shapeId="0" xr:uid="{04C7CFAE-132D-4578-AA1A-A2AED2C7F976}">
       <text>
         <r>
           <rPr>
@@ -281,7 +304,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C40" authorId="0" shapeId="0" xr:uid="{81A96FEF-57F4-4F62-899B-7DDE3044B820}">
+    <comment ref="C40" authorId="1" shapeId="0" xr:uid="{81A96FEF-57F4-4F62-899B-7DDE3044B820}">
       <text>
         <r>
           <rPr>
@@ -296,7 +319,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I42" authorId="0" shapeId="0" xr:uid="{A05FB433-A643-4D7C-BFF5-71BFC3E8211F}">
+    <comment ref="I42" authorId="1" shapeId="0" xr:uid="{A05FB433-A643-4D7C-BFF5-71BFC3E8211F}">
       <text>
         <r>
           <rPr>
@@ -311,7 +334,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J42" authorId="0" shapeId="0" xr:uid="{DF2937F5-01F3-48AD-A59A-11E56D5B996A}">
+    <comment ref="J42" authorId="1" shapeId="0" xr:uid="{DF2937F5-01F3-48AD-A59A-11E56D5B996A}">
       <text>
         <r>
           <rPr>
@@ -326,7 +349,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N42" authorId="0" shapeId="0" xr:uid="{3EABDB6C-68E3-45A8-AD72-EE07047A2ABF}">
+    <comment ref="N42" authorId="1" shapeId="0" xr:uid="{3EABDB6C-68E3-45A8-AD72-EE07047A2ABF}">
       <text>
         <r>
           <rPr>
@@ -341,7 +364,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O42" authorId="3" shapeId="0" xr:uid="{50577B9E-D913-49BB-B91E-A5BD3E934319}">
+    <comment ref="O42" authorId="5" shapeId="0" xr:uid="{50577B9E-D913-49BB-B91E-A5BD3E934319}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -349,7 +372,7 @@
     Pre-arranged with Lead Instructor, the whole GT Mechanical class won't have Pre-OJT</t>
       </text>
     </comment>
-    <comment ref="C43" authorId="0" shapeId="0" xr:uid="{10FC5647-E364-4FB4-A6F5-83AB4EF2B64E}">
+    <comment ref="C43" authorId="1" shapeId="0" xr:uid="{10FC5647-E364-4FB4-A6F5-83AB4EF2B64E}">
       <text>
         <r>
           <rPr>
@@ -365,7 +388,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I45" authorId="0" shapeId="0" xr:uid="{92CB74F4-09AD-4D90-AC85-52E750F91E14}">
+    <comment ref="I45" authorId="1" shapeId="0" xr:uid="{92CB74F4-09AD-4D90-AC85-52E750F91E14}">
       <text>
         <r>
           <rPr>
@@ -380,7 +403,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J45" authorId="0" shapeId="0" xr:uid="{2FC2FC6F-F183-4A7F-9DBC-D4CAC96D4C64}">
+    <comment ref="J45" authorId="1" shapeId="0" xr:uid="{2FC2FC6F-F183-4A7F-9DBC-D4CAC96D4C64}">
       <text>
         <r>
           <rPr>
@@ -395,7 +418,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N45" authorId="0" shapeId="0" xr:uid="{48B8B58B-338A-4616-B616-2225EFDD218F}">
+    <comment ref="N45" authorId="1" shapeId="0" xr:uid="{48B8B58B-338A-4616-B616-2225EFDD218F}">
       <text>
         <r>
           <rPr>
@@ -410,7 +433,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F49" authorId="0" shapeId="0" xr:uid="{E891B715-76B2-41B3-BDA8-A3700F9F11CE}">
+    <comment ref="F49" authorId="1" shapeId="0" xr:uid="{E891B715-76B2-41B3-BDA8-A3700F9F11CE}">
       <text>
         <r>
           <rPr>
@@ -426,7 +449,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K51" authorId="4" shapeId="0" xr:uid="{4A61949D-D058-4614-9CBE-136784BCC6E7}">
+    <comment ref="K51" authorId="6" shapeId="0" xr:uid="{4A61949D-D058-4614-9CBE-136784BCC6E7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -436,7 +459,7 @@
 As tracking stabilizes and system issues are resolved, the data will more accurately reflect true performance and is expected to improve.</t>
       </text>
     </comment>
-    <comment ref="M51" authorId="5" shapeId="0" xr:uid="{40736F15-DF93-4810-BC49-A79E1FB56ED1}">
+    <comment ref="M51" authorId="7" shapeId="0" xr:uid="{40736F15-DF93-4810-BC49-A79E1FB56ED1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -444,7 +467,15 @@
     https://gevernova.box.com/s/17o8hpcpubfb6lm82c157gdcde9kcful</t>
       </text>
     </comment>
-    <comment ref="C52" authorId="0" shapeId="0" xr:uid="{1D261BA2-8304-49D6-B2B0-DECA97456338}">
+    <comment ref="Q51" authorId="8" shapeId="0" xr:uid="{F644D89E-1836-4B19-B5E0-2664B9B5862D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Ben Smith access issues</t>
+      </text>
+    </comment>
+    <comment ref="C52" authorId="1" shapeId="0" xr:uid="{1D261BA2-8304-49D6-B2B0-DECA97456338}">
       <text>
         <r>
           <rPr>
@@ -459,7 +490,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F55" authorId="0" shapeId="0" xr:uid="{B3DF712E-230B-4ACC-BC0C-C0EA167A269C}">
+    <comment ref="F55" authorId="1" shapeId="0" xr:uid="{B3DF712E-230B-4ACC-BC0C-C0EA167A269C}">
       <text>
         <r>
           <rPr>
@@ -475,7 +506,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C58" authorId="0" shapeId="0" xr:uid="{7B8C1B4B-4177-49F0-93C5-A2E4F5B08047}">
+    <comment ref="C58" authorId="1" shapeId="0" xr:uid="{7B8C1B4B-4177-49F0-93C5-A2E4F5B08047}">
       <text>
         <r>
           <rPr>
@@ -490,7 +521,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F58" authorId="0" shapeId="0" xr:uid="{DA09F69C-4C8F-41ED-BFBE-4EBADB371BF8}">
+    <comment ref="F58" authorId="1" shapeId="0" xr:uid="{DA09F69C-4C8F-41ED-BFBE-4EBADB371BF8}">
       <text>
         <r>
           <rPr>
@@ -511,7 +542,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="117">
   <si>
     <t>Level 2</t>
   </si>
@@ -632,6 +663,9 @@
   </si>
   <si>
     <t>Daxer</t>
+  </si>
+  <si>
+    <t>Jul: ENBW (2 courses)-customer mgmt w/ very positive feedback, participants complaints about Sim not site specific; Mill Creek: not recommended, because GT-Maint not needed (LTSA); GECOL: students expected cash or credit card - outside of OFS TRG scope</t>
   </si>
   <si>
     <t># Exams Migrated to Xyleme</t>
@@ -884,16 +918,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="8">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.0_);\(&quot;$&quot;#,##0.0\)"/>
-    <numFmt numFmtId="168" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;?_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0_);\(#,##0.0\)"/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0_);\(&quot;$&quot;#,##0.0\)"/>
+    <numFmt numFmtId="169" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;?_);_(@_)"/>
+    <numFmt numFmtId="170" formatCode="#,##0.0_);\(#,##0.0\)"/>
+    <numFmt numFmtId="171" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1056,11 +1090,6 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -1283,7 +1312,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="235">
@@ -1373,13 +1402,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1389,7 +1418,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1475,22 +1504,22 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="20" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1511,7 +1540,7 @@
     <xf numFmtId="1" fontId="11" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="27" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="27" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="7" fillId="5" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1532,22 +1561,22 @@
     <xf numFmtId="9" fontId="6" fillId="8" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="27" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="27" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="29" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="28" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="29" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="28" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="6" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1556,7 +1585,7 @@
     <xf numFmtId="1" fontId="6" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="29" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="28" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="37" fontId="6" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1569,9 +1598,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="6" fillId="5" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="27" fillId="8" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1598,64 +1624,328 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="29" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="29" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="29" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="29" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="29" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="1" fontId="28" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="28" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="28" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="9" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="7" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="27" fillId="8" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="7" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="3"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="29" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="30" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="21" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="37" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="168" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="37" fontId="9" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="37" fontId="29" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="28" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="165" fontId="26" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="14" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="21" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="29" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="37" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="170" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="22" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="21" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1670,15 +1960,9 @@
     <xf numFmtId="9" fontId="10" fillId="0" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="37" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="37" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1700,281 +1984,26 @@
     <xf numFmtId="1" fontId="14" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="10" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="3" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="22" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="37" fontId="21" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="30" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="31" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="30" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="2" builtinId="5"/>
+    <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2294,6 +2323,18 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="Q6" dT="2026-08-12T01:26:47.89" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{06BE996C-F791-4A9F-AA6D-EE2A8EE2F4C3}">
+    <text xml:space="preserve">BLC: Lost Time Injury - Fall Event 7/21/2026. Recordable </text>
+  </threadedComment>
+  <threadedComment ref="Q6" dT="2026-08-12T01:27:25.92" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{D6A2C5DA-DC04-4CDE-B78F-1BBC1E6623D5}" parentId="{06BE996C-F791-4A9F-AA6D-EE2A8EE2F4C3}">
+    <text>PSE Near Miss: HLC 7HA.03 Project Post Lift Operation Failure</text>
+  </threadedComment>
+  <threadedComment ref="Q9" dT="2026-08-12T12:52:30.70" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{17407CA0-19D6-410B-BD94-9BBC65BFCC7C}">
+    <text>1 X 200000/183589.43=1.089</text>
+  </threadedComment>
+  <threadedComment ref="Q9" dT="2026-08-12T12:52:46.71" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{CFF977E5-20AE-4211-A668-ADE79729D017}" parentId="{17407CA0-19D6-410B-BD94-9BBC65BFCC7C}">
+    <text>I&amp;I FW 33 1.089</text>
+  </threadedComment>
   <threadedComment ref="F13" dT="2024-05-21T17:14:25.01" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{160740E7-DFEB-4450-B5C5-A17286B215D6}">
     <text>90% RA ATS closure rate all sites by YE</text>
   </threadedComment>
@@ -2307,6 +2348,9 @@
   </threadedComment>
   <threadedComment ref="M51" dT="2026-05-08T18:34:11.14" personId="{5990F661-A3AB-41F4-AEAA-FE26C0B875A9}" id="{40736F15-DF93-4810-BC49-A79E1FB56ED1}">
     <text>https://gevernova.box.com/s/17o8hpcpubfb6lm82c157gdcde9kcful</text>
+  </threadedComment>
+  <threadedComment ref="Q51" dT="2026-08-10T18:51:22.55" personId="{5990F661-A3AB-41F4-AEAA-FE26C0B875A9}" id="{F644D89E-1836-4B19-B5E0-2664B9B5862D}">
+    <text>Ben Smith access issues</text>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -2365,31 +2409,31 @@
       <c r="W1" s="5"/>
       <c r="X1" s="6"/>
     </row>
-    <row r="2" spans="1:25" ht="18.600000000000001">
+    <row r="2" spans="1:25" ht="18">
       <c r="A2" s="5"/>
       <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="173">
+      <c r="I2" s="181">
         <v>2026</v>
       </c>
-      <c r="J2" s="174"/>
-      <c r="K2" s="174"/>
-      <c r="L2" s="174"/>
-      <c r="M2" s="174"/>
-      <c r="N2" s="174"/>
-      <c r="O2" s="174"/>
-      <c r="P2" s="174"/>
-      <c r="Q2" s="174"/>
-      <c r="R2" s="174"/>
-      <c r="S2" s="174"/>
-      <c r="T2" s="174"/>
-      <c r="U2" s="174"/>
-      <c r="V2" s="174"/>
-      <c r="W2" s="174"/>
-      <c r="X2" s="175"/>
-    </row>
-    <row r="3" spans="1:25" ht="30.95">
+      <c r="J2" s="182"/>
+      <c r="K2" s="182"/>
+      <c r="L2" s="182"/>
+      <c r="M2" s="182"/>
+      <c r="N2" s="182"/>
+      <c r="O2" s="182"/>
+      <c r="P2" s="182"/>
+      <c r="Q2" s="182"/>
+      <c r="R2" s="182"/>
+      <c r="S2" s="182"/>
+      <c r="T2" s="182"/>
+      <c r="U2" s="182"/>
+      <c r="V2" s="182"/>
+      <c r="W2" s="182"/>
+      <c r="X2" s="183"/>
+    </row>
+    <row r="3" spans="1:25" ht="31.15">
       <c r="A3" s="5"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2460,25 +2504,25 @@
       </c>
     </row>
     <row r="4" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B4" s="194" t="s">
+      <c r="B4" s="162" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="180" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="166" t="s">
+      <c r="D4" s="187" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="182">
+      <c r="E4" s="188">
         <f>SUM(L4,P4,T4,X4)</f>
         <v>0</v>
       </c>
-      <c r="F4" s="126">
-        <v>0</v>
-      </c>
-      <c r="G4" s="182">
+      <c r="F4" s="191">
+        <v>0</v>
+      </c>
+      <c r="G4" s="190">
         <f>SUM(L6,P6,T6,X6)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>26</v>
@@ -2537,12 +2581,12 @@
       </c>
     </row>
     <row r="5" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B5" s="194"/>
+      <c r="B5" s="162"/>
       <c r="C5" s="180"/>
-      <c r="D5" s="166"/>
-      <c r="E5" s="182"/>
-      <c r="F5" s="126"/>
-      <c r="G5" s="182"/>
+      <c r="D5" s="187"/>
+      <c r="E5" s="188"/>
+      <c r="F5" s="191"/>
+      <c r="G5" s="190"/>
       <c r="H5" s="11" t="s">
         <v>27</v>
       </c>
@@ -2600,12 +2644,12 @@
       </c>
     </row>
     <row r="6" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B6" s="194"/>
+      <c r="B6" s="162"/>
       <c r="C6" s="180"/>
-      <c r="D6" s="166"/>
-      <c r="E6" s="182"/>
-      <c r="F6" s="126"/>
-      <c r="G6" s="182"/>
+      <c r="D6" s="187"/>
+      <c r="E6" s="188"/>
+      <c r="F6" s="191"/>
+      <c r="G6" s="190"/>
       <c r="H6" s="11" t="s">
         <v>28</v>
       </c>
@@ -2628,19 +2672,21 @@
       <c r="N6" s="87">
         <v>0</v>
       </c>
-      <c r="O6" s="122">
+      <c r="O6" s="116">
         <v>0</v>
       </c>
       <c r="P6" s="98">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q6" s="14"/>
+      <c r="Q6" s="117">
+        <v>1</v>
+      </c>
       <c r="R6" s="14"/>
       <c r="S6" s="14"/>
       <c r="T6" s="13">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U6" s="14"/>
       <c r="V6" s="14"/>
@@ -2651,23 +2697,23 @@
       </c>
     </row>
     <row r="7" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B7" s="194"/>
-      <c r="C7" s="129" t="s">
+      <c r="B7" s="162"/>
+      <c r="C7" s="143" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="130" t="s">
+      <c r="D7" s="170" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="167">
-        <v>0</v>
-      </c>
-      <c r="F7" s="183">
-        <v>0</v>
-      </c>
-      <c r="G7" s="185">
-        <v>0</v>
-      </c>
-      <c r="H7" s="119" t="s">
+      <c r="E7" s="202">
+        <v>0</v>
+      </c>
+      <c r="F7" s="192">
+        <v>0</v>
+      </c>
+      <c r="G7" s="195">
+        <v>1.089</v>
+      </c>
+      <c r="H7" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I7" s="15">
@@ -2720,13 +2766,13 @@
       </c>
     </row>
     <row r="8" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B8" s="194"/>
-      <c r="C8" s="129"/>
-      <c r="D8" s="130"/>
-      <c r="E8" s="168"/>
-      <c r="F8" s="183"/>
-      <c r="G8" s="185"/>
-      <c r="H8" s="119" t="s">
+      <c r="B8" s="162"/>
+      <c r="C8" s="143"/>
+      <c r="D8" s="170"/>
+      <c r="E8" s="203"/>
+      <c r="F8" s="192"/>
+      <c r="G8" s="195"/>
+      <c r="H8" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I8" s="15">
@@ -2779,13 +2825,13 @@
       </c>
     </row>
     <row r="9" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B9" s="194"/>
-      <c r="C9" s="129"/>
-      <c r="D9" s="130"/>
-      <c r="E9" s="169"/>
-      <c r="F9" s="183"/>
-      <c r="G9" s="185"/>
-      <c r="H9" s="119" t="s">
+      <c r="B9" s="162"/>
+      <c r="C9" s="143"/>
+      <c r="D9" s="170"/>
+      <c r="E9" s="204"/>
+      <c r="F9" s="192"/>
+      <c r="G9" s="195"/>
+      <c r="H9" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I9" s="86">
@@ -2812,7 +2858,9 @@
       <c r="P9" s="98">
         <v>0</v>
       </c>
-      <c r="Q9" s="45"/>
+      <c r="Q9" s="124">
+        <v>1.089</v>
+      </c>
       <c r="R9" s="45"/>
       <c r="S9" s="45"/>
       <c r="T9" s="44"/>
@@ -2822,22 +2870,22 @@
       <c r="X9" s="16"/>
     </row>
     <row r="10" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B10" s="194"/>
+      <c r="B10" s="162"/>
       <c r="C10" s="180" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="166" t="s">
+      <c r="D10" s="187" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="137">
+      <c r="E10" s="201">
         <f>SUM(L10,P10,T10,X10)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="126">
+      <c r="F10" s="191">
         <f>SUM(L11,P11,T11,X11)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="182">
+      <c r="G10" s="188">
         <f>SUM(L12,P12,T12,X12)</f>
         <v>0</v>
       </c>
@@ -2898,12 +2946,12 @@
       </c>
     </row>
     <row r="11" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B11" s="194"/>
+      <c r="B11" s="162"/>
       <c r="C11" s="180"/>
-      <c r="D11" s="166"/>
-      <c r="E11" s="137"/>
-      <c r="F11" s="126"/>
-      <c r="G11" s="182"/>
+      <c r="D11" s="187"/>
+      <c r="E11" s="201"/>
+      <c r="F11" s="191"/>
+      <c r="G11" s="188"/>
       <c r="H11" s="11" t="s">
         <v>27</v>
       </c>
@@ -2961,12 +3009,12 @@
       </c>
     </row>
     <row r="12" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B12" s="194"/>
+      <c r="B12" s="162"/>
       <c r="C12" s="180"/>
-      <c r="D12" s="166"/>
-      <c r="E12" s="137"/>
-      <c r="F12" s="126"/>
-      <c r="G12" s="182"/>
+      <c r="D12" s="187"/>
+      <c r="E12" s="201"/>
+      <c r="F12" s="191"/>
+      <c r="G12" s="188"/>
       <c r="H12" s="11" t="s">
         <v>28</v>
       </c>
@@ -2996,7 +3044,9 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Q12" s="14"/>
+      <c r="Q12" s="87">
+        <v>0</v>
+      </c>
       <c r="R12" s="14"/>
       <c r="S12" s="14"/>
       <c r="T12" s="13">
@@ -3012,23 +3062,23 @@
       </c>
     </row>
     <row r="13" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B13" s="194"/>
-      <c r="C13" s="129" t="s">
+      <c r="B13" s="162"/>
+      <c r="C13" s="143" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="130" t="s">
+      <c r="D13" s="170" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="181">
+      <c r="E13" s="155">
         <v>1</v>
       </c>
-      <c r="F13" s="145">
-        <v>0.9</v>
-      </c>
-      <c r="G13" s="181">
-        <v>0.9</v>
-      </c>
-      <c r="H13" s="119" t="s">
+      <c r="F13" s="200">
+        <v>0.9</v>
+      </c>
+      <c r="G13" s="155">
+        <v>0.9</v>
+      </c>
+      <c r="H13" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I13" s="15" t="s">
@@ -3081,13 +3131,13 @@
       </c>
     </row>
     <row r="14" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B14" s="194"/>
-      <c r="C14" s="129"/>
-      <c r="D14" s="130"/>
-      <c r="E14" s="181"/>
-      <c r="F14" s="145"/>
-      <c r="G14" s="181"/>
-      <c r="H14" s="119" t="s">
+      <c r="B14" s="162"/>
+      <c r="C14" s="143"/>
+      <c r="D14" s="170"/>
+      <c r="E14" s="155"/>
+      <c r="F14" s="200"/>
+      <c r="G14" s="155"/>
+      <c r="H14" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I14" s="38">
@@ -3140,13 +3190,13 @@
       </c>
     </row>
     <row r="15" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B15" s="194"/>
-      <c r="C15" s="129"/>
-      <c r="D15" s="130"/>
-      <c r="E15" s="181"/>
-      <c r="F15" s="145"/>
-      <c r="G15" s="181"/>
-      <c r="H15" s="119" t="s">
+      <c r="B15" s="162"/>
+      <c r="C15" s="143"/>
+      <c r="D15" s="170"/>
+      <c r="E15" s="155"/>
+      <c r="F15" s="200"/>
+      <c r="G15" s="155"/>
+      <c r="H15" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I15" s="77">
@@ -3173,7 +3223,9 @@
       <c r="P15" s="88">
         <v>0.9</v>
       </c>
-      <c r="Q15" s="47"/>
+      <c r="Q15" s="77" t="s">
+        <v>32</v>
+      </c>
       <c r="R15" s="47"/>
       <c r="S15" s="47"/>
       <c r="T15" s="48"/>
@@ -3183,23 +3235,23 @@
       <c r="X15" s="16"/>
     </row>
     <row r="16" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B16" s="194"/>
-      <c r="C16" s="127" t="s">
+      <c r="B16" s="162"/>
+      <c r="C16" s="205" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="171" t="s">
+      <c r="D16" s="189" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="126" t="s">
+      <c r="E16" s="191" t="s">
         <v>35</v>
       </c>
-      <c r="F16" s="157">
-        <v>0.9</v>
-      </c>
-      <c r="G16" s="154">
+      <c r="F16" s="193">
+        <v>0.9</v>
+      </c>
+      <c r="G16" s="198">
         <v>0.95</v>
       </c>
-      <c r="H16" s="121" t="s">
+      <c r="H16" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I16" s="19" t="s">
@@ -3255,13 +3307,13 @@
       </c>
     </row>
     <row r="17" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B17" s="194"/>
-      <c r="C17" s="128"/>
-      <c r="D17" s="171"/>
-      <c r="E17" s="126"/>
-      <c r="F17" s="157"/>
-      <c r="G17" s="154"/>
-      <c r="H17" s="121" t="s">
+      <c r="B17" s="162"/>
+      <c r="C17" s="163"/>
+      <c r="D17" s="189"/>
+      <c r="E17" s="191"/>
+      <c r="F17" s="193"/>
+      <c r="G17" s="198"/>
+      <c r="H17" s="120" t="s">
         <v>27</v>
       </c>
       <c r="I17" s="21">
@@ -3314,13 +3366,13 @@
       </c>
     </row>
     <row r="18" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B18" s="194"/>
-      <c r="C18" s="128"/>
-      <c r="D18" s="171"/>
-      <c r="E18" s="126"/>
-      <c r="F18" s="184"/>
-      <c r="G18" s="155"/>
-      <c r="H18" s="121" t="s">
+      <c r="B18" s="162"/>
+      <c r="C18" s="163"/>
+      <c r="D18" s="189"/>
+      <c r="E18" s="191"/>
+      <c r="F18" s="194"/>
+      <c r="G18" s="199"/>
+      <c r="H18" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I18" s="85">
@@ -3335,19 +3387,21 @@
       <c r="L18" s="94">
         <v>0.92</v>
       </c>
-      <c r="M18" s="102">
-        <v>100</v>
-      </c>
-      <c r="N18" s="102">
-        <v>100</v>
-      </c>
-      <c r="O18" s="105">
+      <c r="M18" s="118">
+        <v>1</v>
+      </c>
+      <c r="N18" s="118">
+        <v>1</v>
+      </c>
+      <c r="O18" s="104">
         <v>84.6</v>
       </c>
-      <c r="P18" s="123">
-        <v>95</v>
-      </c>
-      <c r="Q18" s="52"/>
+      <c r="P18" s="94">
+        <v>0.95</v>
+      </c>
+      <c r="Q18" s="118">
+        <v>1</v>
+      </c>
       <c r="R18" s="53"/>
       <c r="S18" s="52"/>
       <c r="T18" s="43"/>
@@ -3357,25 +3411,25 @@
       <c r="X18" s="43"/>
     </row>
     <row r="19" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B19" s="194" t="s">
+      <c r="B19" s="162" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="129" t="s">
+      <c r="C19" s="143" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="130" t="s">
+      <c r="D19" s="170" t="s">
         <v>39</v>
       </c>
-      <c r="E19" s="131">
+      <c r="E19" s="218">
         <v>83</v>
       </c>
-      <c r="F19" s="143">
+      <c r="F19" s="228">
         <v>83</v>
       </c>
-      <c r="G19" s="124">
-        <v>84.9</v>
-      </c>
-      <c r="H19" s="119" t="s">
+      <c r="G19" s="218">
+        <v>83.8</v>
+      </c>
+      <c r="H19" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I19" s="56">
@@ -3428,13 +3482,13 @@
       </c>
     </row>
     <row r="20" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B20" s="194"/>
-      <c r="C20" s="129"/>
-      <c r="D20" s="130"/>
-      <c r="E20" s="132"/>
-      <c r="F20" s="144"/>
-      <c r="G20" s="125"/>
-      <c r="H20" s="119" t="s">
+      <c r="B20" s="162"/>
+      <c r="C20" s="143"/>
+      <c r="D20" s="170"/>
+      <c r="E20" s="219"/>
+      <c r="F20" s="229"/>
+      <c r="G20" s="219"/>
+      <c r="H20" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I20" s="56">
@@ -3487,13 +3541,13 @@
       </c>
     </row>
     <row r="21" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B21" s="194"/>
-      <c r="C21" s="129"/>
-      <c r="D21" s="130"/>
-      <c r="E21" s="132"/>
-      <c r="F21" s="144"/>
-      <c r="G21" s="125"/>
-      <c r="H21" s="119" t="s">
+      <c r="B21" s="162"/>
+      <c r="C21" s="143"/>
+      <c r="D21" s="170"/>
+      <c r="E21" s="219"/>
+      <c r="F21" s="229"/>
+      <c r="G21" s="219"/>
+      <c r="H21" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I21" s="76">
@@ -3511,16 +3565,18 @@
       <c r="M21" s="76">
         <v>79</v>
       </c>
-      <c r="N21" s="106">
+      <c r="N21" s="105">
         <v>91</v>
       </c>
       <c r="O21" s="76">
-        <v>80.599999999999994</v>
+        <v>78</v>
       </c>
       <c r="P21" s="90">
         <v>84.4</v>
       </c>
-      <c r="Q21" s="58"/>
+      <c r="Q21" s="76">
+        <v>82.5</v>
+      </c>
       <c r="R21" s="58"/>
       <c r="S21" s="58"/>
       <c r="T21" s="58"/>
@@ -3528,26 +3584,29 @@
       <c r="V21" s="58"/>
       <c r="W21" s="58"/>
       <c r="X21" s="44"/>
+      <c r="Y21" s="7" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="22" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B22" s="194"/>
-      <c r="C22" s="127" t="s">
-        <v>40</v>
-      </c>
-      <c r="D22" s="170" t="s">
+      <c r="B22" s="162"/>
+      <c r="C22" s="205" t="s">
         <v>41</v>
       </c>
-      <c r="E22" s="172" t="s">
+      <c r="D22" s="206" t="s">
+        <v>42</v>
+      </c>
+      <c r="E22" s="207" t="s">
         <v>35</v>
       </c>
-      <c r="F22" s="126">
+      <c r="F22" s="191">
         <v>55</v>
       </c>
-      <c r="G22" s="137">
+      <c r="G22" s="201">
         <f>SUM(L24,P24,T24,X24)</f>
-        <v>56</v>
-      </c>
-      <c r="H22" s="121" t="s">
+        <v>76</v>
+      </c>
+      <c r="H22" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I22" s="24" t="s">
@@ -3603,13 +3662,13 @@
       </c>
     </row>
     <row r="23" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B23" s="194"/>
-      <c r="C23" s="128"/>
-      <c r="D23" s="171"/>
-      <c r="E23" s="172"/>
-      <c r="F23" s="126"/>
-      <c r="G23" s="137"/>
-      <c r="H23" s="121" t="s">
+      <c r="B23" s="162"/>
+      <c r="C23" s="163"/>
+      <c r="D23" s="189"/>
+      <c r="E23" s="207"/>
+      <c r="F23" s="191"/>
+      <c r="G23" s="201"/>
+      <c r="H23" s="120" t="s">
         <v>27</v>
       </c>
       <c r="I23" s="12">
@@ -3662,13 +3721,13 @@
       </c>
     </row>
     <row r="24" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B24" s="194"/>
-      <c r="C24" s="128"/>
-      <c r="D24" s="171"/>
-      <c r="E24" s="172"/>
-      <c r="F24" s="126"/>
-      <c r="G24" s="137"/>
-      <c r="H24" s="121" t="s">
+      <c r="B24" s="162"/>
+      <c r="C24" s="163"/>
+      <c r="D24" s="189"/>
+      <c r="E24" s="207"/>
+      <c r="F24" s="191"/>
+      <c r="G24" s="201"/>
+      <c r="H24" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I24" s="86">
@@ -3696,12 +3755,14 @@
         <f>SUM(M24:O24)</f>
         <v>46</v>
       </c>
-      <c r="Q24" s="69"/>
+      <c r="Q24" s="84">
+        <v>20</v>
+      </c>
       <c r="R24" s="19"/>
       <c r="S24" s="69"/>
       <c r="T24" s="79">
         <f>SUM(Q24:S24)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="U24" s="69"/>
       <c r="V24" s="69"/>
@@ -3712,24 +3773,24 @@
       </c>
     </row>
     <row r="25" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B25" s="194"/>
-      <c r="C25" s="199" t="s">
+      <c r="B25" s="162"/>
+      <c r="C25" s="168" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="169" t="s">
         <v>42</v>
       </c>
-      <c r="D25" s="200" t="s">
-        <v>41</v>
-      </c>
-      <c r="E25" s="201" t="s">
+      <c r="E25" s="171" t="s">
         <v>35</v>
       </c>
-      <c r="F25" s="202">
+      <c r="F25" s="172">
         <v>120</v>
       </c>
-      <c r="G25" s="203">
+      <c r="G25" s="173">
         <f>SUM(L27,P27,T27,X27)</f>
-        <v>34</v>
-      </c>
-      <c r="H25" s="119" t="s">
+        <v>38</v>
+      </c>
+      <c r="H25" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I25" s="15" t="s">
@@ -3785,13 +3846,13 @@
       </c>
     </row>
     <row r="26" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B26" s="194"/>
-      <c r="C26" s="129"/>
-      <c r="D26" s="130"/>
-      <c r="E26" s="201"/>
-      <c r="F26" s="202"/>
-      <c r="G26" s="204"/>
-      <c r="H26" s="119" t="s">
+      <c r="B26" s="162"/>
+      <c r="C26" s="143"/>
+      <c r="D26" s="170"/>
+      <c r="E26" s="171"/>
+      <c r="F26" s="172"/>
+      <c r="G26" s="174"/>
+      <c r="H26" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I26" s="15">
@@ -3843,17 +3904,17 @@
         <v>30</v>
       </c>
       <c r="Y26" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B27" s="194"/>
-      <c r="C27" s="129"/>
-      <c r="D27" s="130"/>
-      <c r="E27" s="201"/>
-      <c r="F27" s="202"/>
-      <c r="G27" s="204"/>
-      <c r="H27" s="119" t="s">
+      <c r="B27" s="162"/>
+      <c r="C27" s="143"/>
+      <c r="D27" s="170"/>
+      <c r="E27" s="171"/>
+      <c r="F27" s="172"/>
+      <c r="G27" s="174"/>
+      <c r="H27" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I27" s="80">
@@ -3882,40 +3943,42 @@
         <f>SUM(M27:O27)</f>
         <v>31</v>
       </c>
-      <c r="Q27" s="103"/>
-      <c r="R27" s="103"/>
-      <c r="S27" s="103"/>
+      <c r="Q27" s="80">
+        <v>4</v>
+      </c>
+      <c r="R27" s="102"/>
+      <c r="S27" s="102"/>
       <c r="T27" s="57">
         <f>SUM(Q27:S27)</f>
-        <v>0</v>
-      </c>
-      <c r="U27" s="103"/>
-      <c r="V27" s="103"/>
-      <c r="W27" s="103"/>
+        <v>4</v>
+      </c>
+      <c r="U27" s="102"/>
+      <c r="V27" s="102"/>
+      <c r="W27" s="102"/>
       <c r="X27" s="57">
         <f>SUM(U27:W27)</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B28" s="194"/>
-      <c r="C28" s="127" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" s="170" t="s">
-        <v>41</v>
-      </c>
-      <c r="E28" s="172" t="s">
+      <c r="B28" s="162"/>
+      <c r="C28" s="205" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28" s="206" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28" s="207" t="s">
         <v>35</v>
       </c>
-      <c r="F28" s="148">
-        <v>0.85</v>
-      </c>
-      <c r="G28" s="149">
+      <c r="F28" s="209">
+        <v>0.82</v>
+      </c>
+      <c r="G28" s="232">
         <f>O30</f>
         <v>0.73</v>
       </c>
-      <c r="H28" s="121" t="s">
+      <c r="H28" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I28" s="24" t="s">
@@ -3971,13 +4034,13 @@
       </c>
     </row>
     <row r="29" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B29" s="194"/>
-      <c r="C29" s="128"/>
-      <c r="D29" s="171"/>
-      <c r="E29" s="172"/>
-      <c r="F29" s="148"/>
-      <c r="G29" s="149"/>
-      <c r="H29" s="121" t="s">
+      <c r="B29" s="162"/>
+      <c r="C29" s="163"/>
+      <c r="D29" s="189"/>
+      <c r="E29" s="207"/>
+      <c r="F29" s="209"/>
+      <c r="G29" s="232"/>
+      <c r="H29" s="120" t="s">
         <v>27</v>
       </c>
       <c r="I29" s="24">
@@ -4029,17 +4092,17 @@
         <v>0.85</v>
       </c>
       <c r="Y29" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B30" s="194"/>
-      <c r="C30" s="128"/>
-      <c r="D30" s="171"/>
-      <c r="E30" s="172"/>
-      <c r="F30" s="148"/>
-      <c r="G30" s="149"/>
-      <c r="H30" s="121" t="s">
+      <c r="B30" s="162"/>
+      <c r="C30" s="163"/>
+      <c r="D30" s="189"/>
+      <c r="E30" s="207"/>
+      <c r="F30" s="209"/>
+      <c r="G30" s="232"/>
+      <c r="H30" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I30" s="78">
@@ -4068,12 +4131,14 @@
         <f>AVERAGE(M30:O30)</f>
         <v>0.77333333333333332</v>
       </c>
-      <c r="Q30" s="65"/>
+      <c r="Q30" s="77">
+        <v>0.82</v>
+      </c>
       <c r="R30" s="19"/>
       <c r="S30" s="65"/>
-      <c r="T30" s="66" t="e">
+      <c r="T30" s="66">
         <f>AVERAGE(Q30:S30)</f>
-        <v>#DIV/0!</v>
+        <v>0.82</v>
       </c>
       <c r="U30" s="65"/>
       <c r="V30" s="65"/>
@@ -4084,23 +4149,23 @@
       </c>
     </row>
     <row r="31" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B31" s="194"/>
-      <c r="C31" s="129" t="s">
-        <v>46</v>
-      </c>
-      <c r="D31" s="130" t="s">
+      <c r="B31" s="162"/>
+      <c r="C31" s="143" t="s">
         <v>47</v>
       </c>
-      <c r="E31" s="181">
+      <c r="D31" s="170" t="s">
+        <v>48</v>
+      </c>
+      <c r="E31" s="155">
         <v>0.82</v>
       </c>
-      <c r="F31" s="145">
+      <c r="F31" s="200">
         <v>0.7</v>
       </c>
-      <c r="G31" s="181">
+      <c r="G31" s="155">
         <v>0.83</v>
       </c>
-      <c r="H31" s="119" t="s">
+      <c r="H31" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I31" s="26" t="s">
@@ -4153,13 +4218,13 @@
       </c>
     </row>
     <row r="32" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B32" s="194"/>
-      <c r="C32" s="129"/>
-      <c r="D32" s="130"/>
-      <c r="E32" s="181"/>
-      <c r="F32" s="145"/>
-      <c r="G32" s="181"/>
-      <c r="H32" s="119" t="s">
+      <c r="B32" s="162"/>
+      <c r="C32" s="143"/>
+      <c r="D32" s="170"/>
+      <c r="E32" s="155"/>
+      <c r="F32" s="200"/>
+      <c r="G32" s="155"/>
+      <c r="H32" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I32" s="26">
@@ -4211,24 +4276,24 @@
         <v>0.7</v>
       </c>
       <c r="Y32" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B33" s="194"/>
-      <c r="C33" s="129"/>
-      <c r="D33" s="130"/>
-      <c r="E33" s="181"/>
-      <c r="F33" s="145"/>
-      <c r="G33" s="181"/>
-      <c r="H33" s="119" t="s">
+      <c r="B33" s="162"/>
+      <c r="C33" s="143"/>
+      <c r="D33" s="170"/>
+      <c r="E33" s="155"/>
+      <c r="F33" s="200"/>
+      <c r="G33" s="155"/>
+      <c r="H33" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I33" s="26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J33" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K33" s="77">
         <v>0.83</v>
@@ -4237,10 +4302,10 @@
         <v>0.83</v>
       </c>
       <c r="M33" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N33" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O33" s="77">
         <v>0.81</v>
@@ -4248,7 +4313,9 @@
       <c r="P33" s="88">
         <v>0.81</v>
       </c>
-      <c r="Q33" s="49"/>
+      <c r="Q33" s="15" t="s">
+        <v>50</v>
+      </c>
       <c r="R33" s="15"/>
       <c r="S33" s="49"/>
       <c r="T33" s="63"/>
@@ -4258,25 +4325,25 @@
       <c r="X33" s="33"/>
     </row>
     <row r="34" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B34" s="186" t="s">
-        <v>50</v>
-      </c>
-      <c r="C34" s="128" t="s">
+      <c r="B34" s="147" t="s">
         <v>51</v>
       </c>
-      <c r="D34" s="150" t="s">
+      <c r="C34" s="163" t="s">
         <v>52</v>
       </c>
-      <c r="E34" s="154">
+      <c r="D34" s="153" t="s">
+        <v>53</v>
+      </c>
+      <c r="E34" s="198">
         <v>0.77</v>
       </c>
-      <c r="F34" s="148">
+      <c r="F34" s="209">
         <v>0.85</v>
       </c>
-      <c r="G34" s="158">
+      <c r="G34" s="196">
         <v>0.79</v>
       </c>
-      <c r="H34" s="121" t="s">
+      <c r="H34" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I34" s="21">
@@ -4329,13 +4396,13 @@
       </c>
     </row>
     <row r="35" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B35" s="187"/>
-      <c r="C35" s="128"/>
-      <c r="D35" s="150"/>
-      <c r="E35" s="154"/>
-      <c r="F35" s="148"/>
-      <c r="G35" s="158"/>
-      <c r="H35" s="121" t="s">
+      <c r="B35" s="148"/>
+      <c r="C35" s="163"/>
+      <c r="D35" s="153"/>
+      <c r="E35" s="198"/>
+      <c r="F35" s="209"/>
+      <c r="G35" s="196"/>
+      <c r="H35" s="120" t="s">
         <v>27</v>
       </c>
       <c r="I35" s="21">
@@ -4388,13 +4455,13 @@
       </c>
     </row>
     <row r="36" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B36" s="187"/>
-      <c r="C36" s="195"/>
-      <c r="D36" s="191"/>
-      <c r="E36" s="155"/>
-      <c r="F36" s="148"/>
-      <c r="G36" s="234"/>
-      <c r="H36" s="121" t="s">
+      <c r="B36" s="148"/>
+      <c r="C36" s="164"/>
+      <c r="D36" s="159"/>
+      <c r="E36" s="199"/>
+      <c r="F36" s="209"/>
+      <c r="G36" s="197"/>
+      <c r="H36" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I36" s="77">
@@ -4421,7 +4488,9 @@
       <c r="P36" s="95">
         <v>0.8</v>
       </c>
-      <c r="Q36" s="50"/>
+      <c r="Q36" s="78">
+        <v>0.79</v>
+      </c>
       <c r="R36" s="50"/>
       <c r="S36" s="50"/>
       <c r="T36" s="67"/>
@@ -4431,20 +4500,20 @@
       <c r="X36" s="67"/>
     </row>
     <row r="37" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B37" s="187"/>
-      <c r="C37" s="138" t="s">
-        <v>53</v>
-      </c>
-      <c r="D37" s="141" t="s">
+      <c r="B37" s="148"/>
+      <c r="C37" s="223" t="s">
         <v>54</v>
       </c>
-      <c r="E37" s="161" t="s">
+      <c r="D37" s="226" t="s">
+        <v>55</v>
+      </c>
+      <c r="E37" s="213" t="s">
         <v>35</v>
       </c>
-      <c r="F37" s="162">
-        <v>0.9</v>
-      </c>
-      <c r="G37" s="165">
+      <c r="F37" s="214">
+        <v>0.9</v>
+      </c>
+      <c r="G37" s="217">
         <v>0.6</v>
       </c>
       <c r="H37" s="39" t="s">
@@ -4503,12 +4572,12 @@
       </c>
     </row>
     <row r="38" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B38" s="187"/>
-      <c r="C38" s="139"/>
-      <c r="D38" s="142"/>
-      <c r="E38" s="161"/>
-      <c r="F38" s="162"/>
-      <c r="G38" s="165"/>
+      <c r="B38" s="148"/>
+      <c r="C38" s="224"/>
+      <c r="D38" s="227"/>
+      <c r="E38" s="213"/>
+      <c r="F38" s="214"/>
+      <c r="G38" s="217"/>
       <c r="H38" s="39" t="s">
         <v>27</v>
       </c>
@@ -4562,12 +4631,12 @@
       </c>
     </row>
     <row r="39" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B39" s="187"/>
-      <c r="C39" s="140"/>
-      <c r="D39" s="142"/>
-      <c r="E39" s="161"/>
-      <c r="F39" s="163"/>
-      <c r="G39" s="165"/>
+      <c r="B39" s="148"/>
+      <c r="C39" s="225"/>
+      <c r="D39" s="227"/>
+      <c r="E39" s="213"/>
+      <c r="F39" s="215"/>
+      <c r="G39" s="217"/>
       <c r="H39" s="39" t="s">
         <v>28</v>
       </c>
@@ -4595,7 +4664,9 @@
       <c r="P39" s="95">
         <v>0.4</v>
       </c>
-      <c r="Q39" s="60"/>
+      <c r="Q39" s="78">
+        <v>0.2</v>
+      </c>
       <c r="R39" s="60"/>
       <c r="S39" s="60"/>
       <c r="T39" s="60"/>
@@ -4605,20 +4676,20 @@
       <c r="X39" s="18"/>
     </row>
     <row r="40" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B40" s="187"/>
-      <c r="C40" s="205" t="s">
+      <c r="B40" s="148"/>
+      <c r="C40" s="175" t="s">
+        <v>56</v>
+      </c>
+      <c r="D40" s="178" t="s">
         <v>55</v>
       </c>
-      <c r="D40" s="208" t="s">
-        <v>54</v>
-      </c>
-      <c r="E40" s="209" t="s">
+      <c r="E40" s="179" t="s">
         <v>35</v>
       </c>
-      <c r="F40" s="148">
-        <v>0.9</v>
-      </c>
-      <c r="G40" s="159">
+      <c r="F40" s="209">
+        <v>0.9</v>
+      </c>
+      <c r="G40" s="211">
         <v>0.85</v>
       </c>
       <c r="H40" s="59" t="s">
@@ -4677,12 +4748,12 @@
       </c>
     </row>
     <row r="41" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B41" s="187"/>
-      <c r="C41" s="206"/>
-      <c r="D41" s="150"/>
-      <c r="E41" s="209"/>
-      <c r="F41" s="148"/>
-      <c r="G41" s="160"/>
+      <c r="B41" s="148"/>
+      <c r="C41" s="176"/>
+      <c r="D41" s="153"/>
+      <c r="E41" s="179"/>
+      <c r="F41" s="209"/>
+      <c r="G41" s="212"/>
       <c r="H41" s="59" t="s">
         <v>27</v>
       </c>
@@ -4736,12 +4807,12 @@
       </c>
     </row>
     <row r="42" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B42" s="187"/>
-      <c r="C42" s="207"/>
-      <c r="D42" s="150"/>
-      <c r="E42" s="209"/>
-      <c r="F42" s="148"/>
-      <c r="G42" s="160"/>
+      <c r="B42" s="148"/>
+      <c r="C42" s="177"/>
+      <c r="D42" s="153"/>
+      <c r="E42" s="179"/>
+      <c r="F42" s="209"/>
+      <c r="G42" s="212"/>
       <c r="H42" s="59" t="s">
         <v>28</v>
       </c>
@@ -4769,7 +4840,9 @@
       <c r="P42" s="101">
         <v>0.57999999999999996</v>
       </c>
-      <c r="Q42" s="51"/>
+      <c r="Q42" s="83">
+        <v>0.7</v>
+      </c>
       <c r="R42" s="51"/>
       <c r="S42" s="51"/>
       <c r="T42" s="51"/>
@@ -4779,20 +4852,20 @@
       <c r="X42" s="13"/>
     </row>
     <row r="43" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B43" s="187"/>
-      <c r="C43" s="146" t="s">
-        <v>56</v>
-      </c>
-      <c r="D43" s="141" t="s">
-        <v>54</v>
-      </c>
-      <c r="E43" s="161" t="s">
+      <c r="B43" s="148"/>
+      <c r="C43" s="230" t="s">
+        <v>57</v>
+      </c>
+      <c r="D43" s="226" t="s">
+        <v>55</v>
+      </c>
+      <c r="E43" s="213" t="s">
         <v>35</v>
       </c>
-      <c r="F43" s="162">
+      <c r="F43" s="214">
         <v>1</v>
       </c>
-      <c r="G43" s="164">
+      <c r="G43" s="216">
         <v>0.93</v>
       </c>
       <c r="H43" s="39" t="s">
@@ -4851,12 +4924,12 @@
       </c>
     </row>
     <row r="44" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B44" s="187"/>
-      <c r="C44" s="147"/>
-      <c r="D44" s="142"/>
-      <c r="E44" s="161"/>
-      <c r="F44" s="162"/>
-      <c r="G44" s="164"/>
+      <c r="B44" s="148"/>
+      <c r="C44" s="231"/>
+      <c r="D44" s="227"/>
+      <c r="E44" s="213"/>
+      <c r="F44" s="214"/>
+      <c r="G44" s="216"/>
       <c r="H44" s="39" t="s">
         <v>27</v>
       </c>
@@ -4909,16 +4982,16 @@
         <v>1</v>
       </c>
       <c r="Y44" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="45" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B45" s="187"/>
-      <c r="C45" s="147"/>
-      <c r="D45" s="142"/>
-      <c r="E45" s="161"/>
-      <c r="F45" s="163"/>
-      <c r="G45" s="164"/>
+      <c r="B45" s="148"/>
+      <c r="C45" s="231"/>
+      <c r="D45" s="227"/>
+      <c r="E45" s="213"/>
+      <c r="F45" s="215"/>
+      <c r="G45" s="216"/>
       <c r="H45" s="39" t="s">
         <v>28</v>
       </c>
@@ -4946,7 +5019,9 @@
       <c r="P45" s="101">
         <v>0.99</v>
       </c>
-      <c r="Q45" s="60"/>
+      <c r="Q45" s="83">
+        <v>0.95</v>
+      </c>
       <c r="R45" s="60"/>
       <c r="S45" s="60"/>
       <c r="T45" s="60"/>
@@ -4956,144 +5031,144 @@
       <c r="X45" s="18"/>
     </row>
     <row r="46" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B46" s="187"/>
-      <c r="C46" s="128" t="s">
-        <v>58</v>
-      </c>
-      <c r="D46" s="150" t="s">
-        <v>54</v>
-      </c>
-      <c r="E46" s="151">
+      <c r="B46" s="148"/>
+      <c r="C46" s="163" t="s">
+        <v>59</v>
+      </c>
+      <c r="D46" s="153" t="s">
+        <v>55</v>
+      </c>
+      <c r="E46" s="233">
         <v>372</v>
       </c>
-      <c r="F46" s="152">
+      <c r="F46" s="234">
         <v>366</v>
       </c>
-      <c r="G46" s="137">
+      <c r="G46" s="201">
         <v>365</v>
       </c>
-      <c r="H46" s="121" t="s">
+      <c r="H46" s="120" t="s">
         <v>26</v>
       </c>
-      <c r="I46" s="107">
+      <c r="I46" s="106">
         <v>383</v>
       </c>
-      <c r="J46" s="107">
+      <c r="J46" s="106">
         <v>381</v>
       </c>
-      <c r="K46" s="107">
+      <c r="K46" s="106">
         <v>380</v>
       </c>
-      <c r="L46" s="108">
+      <c r="L46" s="107">
         <v>381</v>
       </c>
-      <c r="M46" s="107">
+      <c r="M46" s="106">
         <v>378</v>
       </c>
-      <c r="N46" s="107">
+      <c r="N46" s="106">
         <v>376</v>
       </c>
-      <c r="O46" s="107">
+      <c r="O46" s="106">
         <v>374</v>
       </c>
-      <c r="P46" s="108">
+      <c r="P46" s="107">
         <v>376</v>
       </c>
-      <c r="Q46" s="107">
+      <c r="Q46" s="106">
         <v>372</v>
       </c>
-      <c r="R46" s="107">
+      <c r="R46" s="106">
         <v>370</v>
       </c>
-      <c r="S46" s="107">
+      <c r="S46" s="106">
         <v>371</v>
       </c>
-      <c r="T46" s="108">
+      <c r="T46" s="107">
         <v>371</v>
       </c>
-      <c r="U46" s="107">
+      <c r="U46" s="106">
         <v>372</v>
       </c>
-      <c r="V46" s="107">
+      <c r="V46" s="106">
         <v>371</v>
       </c>
-      <c r="W46" s="107">
+      <c r="W46" s="106">
         <v>371</v>
       </c>
-      <c r="X46" s="108">
+      <c r="X46" s="107">
         <v>371</v>
       </c>
     </row>
     <row r="47" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B47" s="187"/>
-      <c r="C47" s="128"/>
-      <c r="D47" s="150"/>
-      <c r="E47" s="151"/>
-      <c r="F47" s="152"/>
-      <c r="G47" s="137"/>
-      <c r="H47" s="121" t="s">
+      <c r="B47" s="148"/>
+      <c r="C47" s="163"/>
+      <c r="D47" s="153"/>
+      <c r="E47" s="233"/>
+      <c r="F47" s="234"/>
+      <c r="G47" s="201"/>
+      <c r="H47" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="I47" s="107">
+      <c r="I47" s="106">
         <v>366</v>
       </c>
-      <c r="J47" s="107">
+      <c r="J47" s="106">
         <v>366</v>
       </c>
-      <c r="K47" s="107">
+      <c r="K47" s="106">
         <v>366</v>
       </c>
-      <c r="L47" s="108">
+      <c r="L47" s="107">
         <v>366</v>
       </c>
-      <c r="M47" s="107">
+      <c r="M47" s="106">
         <v>366</v>
       </c>
-      <c r="N47" s="107">
+      <c r="N47" s="106">
         <v>366</v>
       </c>
-      <c r="O47" s="107">
+      <c r="O47" s="106">
         <v>366</v>
       </c>
-      <c r="P47" s="108">
+      <c r="P47" s="107">
         <v>366</v>
       </c>
-      <c r="Q47" s="107">
+      <c r="Q47" s="106">
         <v>366</v>
       </c>
-      <c r="R47" s="107">
+      <c r="R47" s="106">
         <v>366</v>
       </c>
-      <c r="S47" s="107">
+      <c r="S47" s="106">
         <v>366</v>
       </c>
-      <c r="T47" s="108">
+      <c r="T47" s="107">
         <v>366</v>
       </c>
-      <c r="U47" s="107">
+      <c r="U47" s="106">
         <v>366</v>
       </c>
-      <c r="V47" s="107">
+      <c r="V47" s="106">
         <v>366</v>
       </c>
-      <c r="W47" s="107">
+      <c r="W47" s="106">
         <v>366</v>
       </c>
-      <c r="X47" s="108">
+      <c r="X47" s="107">
         <v>366</v>
       </c>
       <c r="Y47" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="48" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B48" s="187"/>
-      <c r="C48" s="128"/>
-      <c r="D48" s="150"/>
-      <c r="E48" s="151"/>
-      <c r="F48" s="152"/>
-      <c r="G48" s="137"/>
-      <c r="H48" s="121" t="s">
+      <c r="B48" s="148"/>
+      <c r="C48" s="163"/>
+      <c r="D48" s="153"/>
+      <c r="E48" s="233"/>
+      <c r="F48" s="234"/>
+      <c r="G48" s="201"/>
+      <c r="H48" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I48" s="76">
@@ -5120,33 +5195,35 @@
       <c r="P48" s="96">
         <v>369</v>
       </c>
-      <c r="Q48" s="107"/>
-      <c r="R48" s="107"/>
-      <c r="S48" s="107"/>
-      <c r="T48" s="108"/>
-      <c r="U48" s="107"/>
-      <c r="V48" s="107"/>
-      <c r="W48" s="107"/>
-      <c r="X48" s="108"/>
+      <c r="Q48" s="87">
+        <v>363</v>
+      </c>
+      <c r="R48" s="106"/>
+      <c r="S48" s="106"/>
+      <c r="T48" s="107"/>
+      <c r="U48" s="106"/>
+      <c r="V48" s="106"/>
+      <c r="W48" s="106"/>
+      <c r="X48" s="107"/>
     </row>
     <row r="49" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B49" s="187"/>
-      <c r="C49" s="176" t="s">
-        <v>60</v>
-      </c>
-      <c r="D49" s="177" t="s">
-        <v>47</v>
-      </c>
-      <c r="E49" s="179">
+      <c r="B49" s="148"/>
+      <c r="C49" s="184" t="s">
+        <v>61</v>
+      </c>
+      <c r="D49" s="185" t="s">
+        <v>48</v>
+      </c>
+      <c r="E49" s="186">
         <v>0.71</v>
       </c>
-      <c r="F49" s="197">
+      <c r="F49" s="166">
         <v>0.92</v>
       </c>
-      <c r="G49" s="133">
+      <c r="G49" s="220">
         <v>0.72</v>
       </c>
-      <c r="H49" s="119" t="s">
+      <c r="H49" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I49" s="26">
@@ -5199,13 +5276,13 @@
       </c>
     </row>
     <row r="50" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B50" s="187"/>
-      <c r="C50" s="129"/>
-      <c r="D50" s="178"/>
-      <c r="E50" s="179"/>
-      <c r="F50" s="197"/>
-      <c r="G50" s="134"/>
-      <c r="H50" s="119" t="s">
+      <c r="B50" s="148"/>
+      <c r="C50" s="143"/>
+      <c r="D50" s="144"/>
+      <c r="E50" s="186"/>
+      <c r="F50" s="166"/>
+      <c r="G50" s="221"/>
+      <c r="H50" s="121" t="s">
         <v>27</v>
       </c>
       <c r="I50" s="26">
@@ -5258,13 +5335,13 @@
       </c>
     </row>
     <row r="51" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B51" s="187"/>
-      <c r="C51" s="129"/>
-      <c r="D51" s="178"/>
-      <c r="E51" s="179"/>
-      <c r="F51" s="197"/>
-      <c r="G51" s="134"/>
-      <c r="H51" s="119" t="s">
+      <c r="B51" s="148"/>
+      <c r="C51" s="143"/>
+      <c r="D51" s="144"/>
+      <c r="E51" s="186"/>
+      <c r="F51" s="166"/>
+      <c r="G51" s="221"/>
+      <c r="H51" s="121" t="s">
         <v>28</v>
       </c>
       <c r="I51" s="78">
@@ -5274,7 +5351,7 @@
         <v>0.6</v>
       </c>
       <c r="K51" s="78" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L51" s="95">
         <v>0.72</v>
@@ -5291,7 +5368,9 @@
       <c r="P51" s="95">
         <v>0.82</v>
       </c>
-      <c r="Q51" s="49"/>
+      <c r="Q51" s="78">
+        <v>0.89</v>
+      </c>
       <c r="R51" s="49"/>
       <c r="S51" s="49"/>
       <c r="T51" s="48"/>
@@ -5301,23 +5380,23 @@
       <c r="X51" s="27"/>
     </row>
     <row r="52" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B52" s="187"/>
-      <c r="C52" s="128" t="s">
-        <v>62</v>
-      </c>
-      <c r="D52" s="150" t="s">
-        <v>47</v>
-      </c>
-      <c r="E52" s="198" t="s">
+      <c r="B52" s="148"/>
+      <c r="C52" s="163" t="s">
+        <v>63</v>
+      </c>
+      <c r="D52" s="153" t="s">
+        <v>48</v>
+      </c>
+      <c r="E52" s="167" t="s">
         <v>35</v>
       </c>
-      <c r="F52" s="156" t="s">
-        <v>63</v>
-      </c>
-      <c r="G52" s="158">
+      <c r="F52" s="210" t="s">
+        <v>64</v>
+      </c>
+      <c r="G52" s="196">
         <v>0.28999999999999998</v>
       </c>
-      <c r="H52" s="121" t="s">
+      <c r="H52" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I52" s="24" t="s">
@@ -5373,58 +5452,58 @@
       </c>
     </row>
     <row r="53" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B53" s="187"/>
-      <c r="C53" s="128"/>
-      <c r="D53" s="150"/>
-      <c r="E53" s="198"/>
-      <c r="F53" s="157"/>
-      <c r="G53" s="158"/>
-      <c r="H53" s="121" t="s">
+      <c r="B53" s="148"/>
+      <c r="C53" s="163"/>
+      <c r="D53" s="153"/>
+      <c r="E53" s="167"/>
+      <c r="F53" s="193"/>
+      <c r="G53" s="196"/>
+      <c r="H53" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="I53" s="135"/>
-      <c r="J53" s="135"/>
-      <c r="K53" s="135"/>
-      <c r="L53" s="109" t="s">
-        <v>63</v>
-      </c>
-      <c r="M53" s="135"/>
-      <c r="N53" s="135"/>
-      <c r="O53" s="135"/>
-      <c r="P53" s="109" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q53" s="135"/>
-      <c r="R53" s="135"/>
-      <c r="S53" s="135"/>
-      <c r="T53" s="109" t="s">
-        <v>63</v>
-      </c>
-      <c r="U53" s="135"/>
-      <c r="V53" s="135"/>
-      <c r="W53" s="135"/>
-      <c r="X53" s="109" t="s">
-        <v>63</v>
+      <c r="I53" s="130"/>
+      <c r="J53" s="130"/>
+      <c r="K53" s="130"/>
+      <c r="L53" s="108" t="s">
+        <v>64</v>
+      </c>
+      <c r="M53" s="130"/>
+      <c r="N53" s="130"/>
+      <c r="O53" s="130"/>
+      <c r="P53" s="108" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q53" s="130"/>
+      <c r="R53" s="130"/>
+      <c r="S53" s="130"/>
+      <c r="T53" s="108" t="s">
+        <v>64</v>
+      </c>
+      <c r="U53" s="130"/>
+      <c r="V53" s="130"/>
+      <c r="W53" s="130"/>
+      <c r="X53" s="108" t="s">
+        <v>64</v>
       </c>
       <c r="Y53" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="54" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B54" s="187"/>
-      <c r="C54" s="128"/>
-      <c r="D54" s="150"/>
-      <c r="E54" s="198"/>
-      <c r="F54" s="157"/>
-      <c r="G54" s="158"/>
-      <c r="H54" s="121" t="s">
+      <c r="B54" s="148"/>
+      <c r="C54" s="163"/>
+      <c r="D54" s="153"/>
+      <c r="E54" s="167"/>
+      <c r="F54" s="193"/>
+      <c r="G54" s="196"/>
+      <c r="H54" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I54" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J54" s="24" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K54" s="24">
         <v>0.28799999999999998</v>
@@ -5444,7 +5523,9 @@
       <c r="P54" s="95">
         <v>0.16</v>
       </c>
-      <c r="Q54" s="24"/>
+      <c r="Q54" s="24">
+        <v>0.214</v>
+      </c>
       <c r="R54" s="24"/>
       <c r="S54" s="24"/>
       <c r="T54" s="25"/>
@@ -5454,25 +5535,25 @@
       <c r="X54" s="25"/>
     </row>
     <row r="55" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B55" s="187"/>
-      <c r="C55" s="129" t="s">
-        <v>67</v>
-      </c>
-      <c r="D55" s="178" t="s">
+      <c r="B55" s="148"/>
+      <c r="C55" s="143" t="s">
         <v>68</v>
       </c>
-      <c r="E55" s="213">
+      <c r="D55" s="144" t="s">
+        <v>69</v>
+      </c>
+      <c r="E55" s="145">
         <f>X55</f>
         <v>40</v>
       </c>
-      <c r="F55" s="196">
+      <c r="F55" s="165">
         <v>55</v>
       </c>
-      <c r="G55" s="136">
+      <c r="G55" s="222">
         <f>X57</f>
-        <v>42</v>
-      </c>
-      <c r="H55" s="119" t="s">
+        <v>44</v>
+      </c>
+      <c r="H55" s="121" t="s">
         <v>26</v>
       </c>
       <c r="I55" s="15">
@@ -5525,117 +5606,119 @@
       </c>
     </row>
     <row r="56" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B56" s="187"/>
-      <c r="C56" s="129"/>
-      <c r="D56" s="178"/>
-      <c r="E56" s="213"/>
-      <c r="F56" s="196"/>
-      <c r="G56" s="136"/>
-      <c r="H56" s="119" t="s">
+      <c r="B56" s="148"/>
+      <c r="C56" s="143"/>
+      <c r="D56" s="144"/>
+      <c r="E56" s="145"/>
+      <c r="F56" s="165"/>
+      <c r="G56" s="222"/>
+      <c r="H56" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I56" s="153" t="s">
-        <v>32</v>
-      </c>
-      <c r="J56" s="153"/>
-      <c r="K56" s="153"/>
+      <c r="I56" s="208" t="s">
+        <v>32</v>
+      </c>
+      <c r="J56" s="208"/>
+      <c r="K56" s="208"/>
       <c r="L56" s="18">
         <v>13</v>
       </c>
-      <c r="M56" s="153" t="s">
-        <v>32</v>
-      </c>
-      <c r="N56" s="153"/>
-      <c r="O56" s="153"/>
+      <c r="M56" s="208" t="s">
+        <v>32</v>
+      </c>
+      <c r="N56" s="208"/>
+      <c r="O56" s="208"/>
       <c r="P56" s="18">
         <v>27</v>
       </c>
-      <c r="Q56" s="153" t="s">
-        <v>32</v>
-      </c>
-      <c r="R56" s="153"/>
-      <c r="S56" s="153"/>
+      <c r="Q56" s="208" t="s">
+        <v>32</v>
+      </c>
+      <c r="R56" s="208"/>
+      <c r="S56" s="208"/>
       <c r="T56" s="18">
         <v>41</v>
       </c>
-      <c r="U56" s="153" t="s">
-        <v>32</v>
-      </c>
-      <c r="V56" s="153"/>
-      <c r="W56" s="153"/>
+      <c r="U56" s="208" t="s">
+        <v>32</v>
+      </c>
+      <c r="V56" s="208"/>
+      <c r="W56" s="208"/>
       <c r="X56" s="18">
         <v>55</v>
       </c>
     </row>
     <row r="57" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B57" s="187"/>
-      <c r="C57" s="129"/>
-      <c r="D57" s="178"/>
-      <c r="E57" s="213"/>
-      <c r="F57" s="196"/>
-      <c r="G57" s="136"/>
-      <c r="H57" s="119" t="s">
+      <c r="B57" s="148"/>
+      <c r="C57" s="143"/>
+      <c r="D57" s="144"/>
+      <c r="E57" s="145"/>
+      <c r="F57" s="165"/>
+      <c r="G57" s="222"/>
+      <c r="H57" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="I57" s="110">
-        <v>0</v>
-      </c>
-      <c r="J57" s="110">
-        <v>0</v>
-      </c>
-      <c r="K57" s="110">
+      <c r="I57" s="109">
+        <v>0</v>
+      </c>
+      <c r="J57" s="109">
+        <v>0</v>
+      </c>
+      <c r="K57" s="109">
         <v>17</v>
       </c>
       <c r="L57" s="90">
         <v>17</v>
       </c>
-      <c r="M57" s="110">
+      <c r="M57" s="109">
         <v>25</v>
       </c>
-      <c r="N57" s="110">
-        <v>0</v>
-      </c>
-      <c r="O57" s="110">
-        <v>0</v>
-      </c>
-      <c r="P57" s="115">
+      <c r="N57" s="109">
+        <v>0</v>
+      </c>
+      <c r="O57" s="109">
+        <v>0</v>
+      </c>
+      <c r="P57" s="114">
         <v>42</v>
       </c>
-      <c r="Q57" s="110"/>
-      <c r="R57" s="110"/>
-      <c r="S57" s="110"/>
-      <c r="T57" s="111">
+      <c r="Q57" s="109">
+        <v>2</v>
+      </c>
+      <c r="R57" s="109"/>
+      <c r="S57" s="109"/>
+      <c r="T57" s="110">
         <f>SUM(P57:S57)</f>
-        <v>42</v>
-      </c>
-      <c r="U57" s="110"/>
-      <c r="V57" s="110"/>
-      <c r="W57" s="110"/>
-      <c r="X57" s="111">
+        <v>44</v>
+      </c>
+      <c r="U57" s="109"/>
+      <c r="V57" s="109"/>
+      <c r="W57" s="109"/>
+      <c r="X57" s="110">
         <f>SUM(T57:W57)</f>
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="58" spans="2:25" ht="15" hidden="1" customHeight="1">
-      <c r="B58" s="186" t="s">
-        <v>69</v>
-      </c>
-      <c r="C58" s="188" t="s">
+      <c r="B58" s="147" t="s">
         <v>70</v>
       </c>
-      <c r="D58" s="191" t="s">
+      <c r="C58" s="156" t="s">
         <v>71</v>
       </c>
-      <c r="E58" s="220">
+      <c r="D58" s="159" t="s">
+        <v>72</v>
+      </c>
+      <c r="E58" s="135">
         <v>92.5</v>
       </c>
-      <c r="F58" s="229">
+      <c r="F58" s="132">
         <v>93</v>
       </c>
-      <c r="G58" s="220">
+      <c r="G58" s="135">
         <v>92.5</v>
       </c>
-      <c r="H58" s="121" t="s">
+      <c r="H58" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I58" s="34">
@@ -5687,17 +5770,17 @@
         <v>92.5</v>
       </c>
       <c r="Y58" s="37" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="59" spans="2:25" ht="15" hidden="1" customHeight="1">
-      <c r="B59" s="187"/>
-      <c r="C59" s="189"/>
-      <c r="D59" s="192"/>
-      <c r="E59" s="221"/>
-      <c r="F59" s="230"/>
-      <c r="G59" s="221"/>
-      <c r="H59" s="121" t="s">
+      <c r="B59" s="148"/>
+      <c r="C59" s="157"/>
+      <c r="D59" s="160"/>
+      <c r="E59" s="136"/>
+      <c r="F59" s="133"/>
+      <c r="G59" s="136"/>
+      <c r="H59" s="120" t="s">
         <v>27</v>
       </c>
       <c r="I59" s="19">
@@ -5749,17 +5832,17 @@
         <v>93</v>
       </c>
       <c r="Y59" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="60" spans="2:25" ht="15" hidden="1" customHeight="1">
-      <c r="B60" s="187"/>
-      <c r="C60" s="190"/>
-      <c r="D60" s="193"/>
-      <c r="E60" s="222"/>
-      <c r="F60" s="231"/>
-      <c r="G60" s="222"/>
-      <c r="H60" s="121" t="s">
+      <c r="B60" s="148"/>
+      <c r="C60" s="158"/>
+      <c r="D60" s="161"/>
+      <c r="E60" s="137"/>
+      <c r="F60" s="134"/>
+      <c r="G60" s="137"/>
+      <c r="H60" s="120" t="s">
         <v>28</v>
       </c>
       <c r="I60" s="36">
@@ -5777,33 +5860,33 @@
       <c r="S60" s="22"/>
       <c r="T60" s="20"/>
       <c r="U60" s="22"/>
-      <c r="V60" s="104"/>
-      <c r="W60" s="104"/>
+      <c r="V60" s="103"/>
+      <c r="W60" s="103"/>
       <c r="X60" s="20"/>
     </row>
     <row r="61" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B61" s="186" t="s">
-        <v>74</v>
-      </c>
-      <c r="C61" s="214" t="s">
+      <c r="B61" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="D61" s="150" t="s">
+      <c r="C61" s="146" t="s">
+        <v>76</v>
+      </c>
+      <c r="D61" s="153" t="s">
         <v>39</v>
       </c>
-      <c r="E61" s="219">
+      <c r="E61" s="154">
         <f>L61+P61+T61+X61</f>
         <v>30.187825999999998</v>
       </c>
-      <c r="F61" s="233">
+      <c r="F61" s="139">
         <f>SUM(L62,P62,T62,X62)</f>
         <v>28</v>
       </c>
-      <c r="G61" s="228">
+      <c r="G61" s="131">
         <f>L63+P63+T63+X63</f>
-        <v>11.850283999999998</v>
-      </c>
-      <c r="H61" s="121" t="s">
+        <v>14.112583999999998</v>
+      </c>
+      <c r="H61" s="120" t="s">
         <v>26</v>
       </c>
       <c r="I61" s="70">
@@ -5859,123 +5942,125 @@
       </c>
     </row>
     <row r="62" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B62" s="187"/>
-      <c r="C62" s="214"/>
-      <c r="D62" s="150"/>
-      <c r="E62" s="219"/>
-      <c r="F62" s="233"/>
-      <c r="G62" s="228"/>
-      <c r="H62" s="121" t="s">
+      <c r="B62" s="148"/>
+      <c r="C62" s="146"/>
+      <c r="D62" s="153"/>
+      <c r="E62" s="154"/>
+      <c r="F62" s="139"/>
+      <c r="G62" s="131"/>
+      <c r="H62" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="I62" s="135" t="s">
-        <v>32</v>
-      </c>
-      <c r="J62" s="135"/>
-      <c r="K62" s="135"/>
+      <c r="I62" s="130" t="s">
+        <v>32</v>
+      </c>
+      <c r="J62" s="130"/>
+      <c r="K62" s="130"/>
       <c r="L62" s="71">
         <v>5</v>
       </c>
-      <c r="M62" s="135" t="s">
-        <v>32</v>
-      </c>
-      <c r="N62" s="135"/>
-      <c r="O62" s="135"/>
+      <c r="M62" s="130" t="s">
+        <v>32</v>
+      </c>
+      <c r="N62" s="130"/>
+      <c r="O62" s="130"/>
       <c r="P62" s="71">
         <v>7</v>
       </c>
-      <c r="Q62" s="135" t="s">
-        <v>32</v>
-      </c>
-      <c r="R62" s="135"/>
-      <c r="S62" s="135"/>
+      <c r="Q62" s="130" t="s">
+        <v>32</v>
+      </c>
+      <c r="R62" s="130"/>
+      <c r="S62" s="130"/>
       <c r="T62" s="71">
         <v>7</v>
       </c>
       <c r="U62" s="71" t="s">
         <v>32</v>
       </c>
-      <c r="V62" s="117"/>
-      <c r="W62" s="117"/>
+      <c r="V62" s="119"/>
+      <c r="W62" s="119"/>
       <c r="X62" s="71">
         <v>9</v>
       </c>
     </row>
     <row r="63" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B63" s="187"/>
-      <c r="C63" s="214"/>
-      <c r="D63" s="150"/>
-      <c r="E63" s="219"/>
-      <c r="F63" s="233"/>
-      <c r="G63" s="228"/>
-      <c r="H63" s="121" t="s">
+      <c r="B63" s="148"/>
+      <c r="C63" s="146"/>
+      <c r="D63" s="153"/>
+      <c r="E63" s="154"/>
+      <c r="F63" s="139"/>
+      <c r="G63" s="131"/>
+      <c r="H63" s="120" t="s">
         <v>28</v>
       </c>
-      <c r="I63" s="117">
+      <c r="I63" s="119">
         <v>1.333</v>
       </c>
-      <c r="J63" s="117">
+      <c r="J63" s="119">
         <v>1.4</v>
       </c>
-      <c r="K63" s="117">
+      <c r="K63" s="119">
         <v>2.5</v>
       </c>
       <c r="L63" s="91">
         <f>K63+J63+I63</f>
         <v>5.2329999999999997</v>
       </c>
-      <c r="M63" s="117">
+      <c r="M63" s="119">
         <v>1.5</v>
       </c>
-      <c r="N63" s="117">
+      <c r="N63" s="119">
         <v>3.2572839999999998</v>
       </c>
-      <c r="O63" s="117">
+      <c r="O63" s="119">
         <v>1.86</v>
       </c>
-      <c r="P63" s="114">
+      <c r="P63" s="113">
         <f>O63+N63+M63</f>
         <v>6.6172839999999997</v>
       </c>
-      <c r="Q63" s="117"/>
-      <c r="R63" s="117"/>
-      <c r="S63" s="117"/>
+      <c r="Q63" s="119">
+        <v>2.2623000000000002</v>
+      </c>
+      <c r="R63" s="119"/>
+      <c r="S63" s="119"/>
       <c r="T63" s="92">
         <f>S63+R63+Q63</f>
-        <v>0</v>
-      </c>
-      <c r="U63" s="117"/>
-      <c r="V63" s="117"/>
-      <c r="W63" s="117"/>
+        <v>2.2623000000000002</v>
+      </c>
+      <c r="U63" s="119"/>
+      <c r="V63" s="119"/>
+      <c r="W63" s="119"/>
       <c r="X63" s="92">
         <f>W63+V63+U63</f>
         <v>0</v>
       </c>
       <c r="Y63" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="64" spans="2:25" ht="15.6">
-      <c r="B64" s="187"/>
-      <c r="C64" s="210" t="s">
-        <v>77</v>
-      </c>
-      <c r="D64" s="211" t="s">
+      <c r="B64" s="148"/>
+      <c r="C64" s="140" t="s">
         <v>78</v>
       </c>
-      <c r="E64" s="212">
+      <c r="D64" s="141" t="s">
+        <v>79</v>
+      </c>
+      <c r="E64" s="142">
         <f>L64+P64+T64+X64</f>
         <v>-8.4644727175232077</v>
       </c>
-      <c r="F64" s="232">
+      <c r="F64" s="138">
         <f>SUM(L65,P65,T65,X65)</f>
         <v>-7.0189285867816498</v>
       </c>
-      <c r="G64" s="227">
-        <f>SUM(L66,P66,T66,X66)</f>
-        <v>-3.8762228984112506</v>
-      </c>
-      <c r="H64" s="118" t="s">
+      <c r="G64" s="129">
+        <f>SUM(L66,P66,T66,Q66,X66)</f>
+        <v>-5.8522190000397307</v>
+      </c>
+      <c r="H64" s="122" t="s">
         <v>26</v>
       </c>
       <c r="I64" s="72">
@@ -6032,13 +6117,13 @@
       </c>
     </row>
     <row r="65" spans="2:24" ht="15.6">
-      <c r="B65" s="187"/>
-      <c r="C65" s="210"/>
-      <c r="D65" s="211"/>
-      <c r="E65" s="212"/>
-      <c r="F65" s="232"/>
-      <c r="G65" s="227"/>
-      <c r="H65" s="118" t="s">
+      <c r="B65" s="148"/>
+      <c r="C65" s="140"/>
+      <c r="D65" s="141"/>
+      <c r="E65" s="142"/>
+      <c r="F65" s="138"/>
+      <c r="G65" s="129"/>
+      <c r="H65" s="122" t="s">
         <v>27</v>
       </c>
       <c r="I65" s="72">
@@ -6095,13 +6180,13 @@
       </c>
     </row>
     <row r="66" spans="2:24" ht="15.6">
-      <c r="B66" s="187"/>
-      <c r="C66" s="210"/>
-      <c r="D66" s="211"/>
-      <c r="E66" s="212"/>
-      <c r="F66" s="232"/>
-      <c r="G66" s="227"/>
-      <c r="H66" s="118" t="s">
+      <c r="B66" s="148"/>
+      <c r="C66" s="140"/>
+      <c r="D66" s="141"/>
+      <c r="E66" s="142"/>
+      <c r="F66" s="138"/>
+      <c r="G66" s="129"/>
+      <c r="H66" s="122" t="s">
         <v>28</v>
       </c>
       <c r="I66" s="82">
@@ -6130,42 +6215,44 @@
         <f>SUM(M66:O66)</f>
         <v>-1.7762228984112503</v>
       </c>
-      <c r="Q66" s="72"/>
+      <c r="Q66" s="82">
+        <v>-0.98799805081423986</v>
+      </c>
       <c r="R66" s="72"/>
       <c r="S66" s="72"/>
-      <c r="T66" s="112">
+      <c r="T66" s="111">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-0.98799805081423986</v>
       </c>
       <c r="U66" s="72"/>
       <c r="V66" s="72"/>
       <c r="W66" s="72"/>
-      <c r="X66" s="112">
+      <c r="X66" s="111">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
     <row r="67" spans="2:24" ht="15" customHeight="1">
-      <c r="B67" s="187"/>
-      <c r="C67" s="216" t="s">
+      <c r="B67" s="148"/>
+      <c r="C67" s="150" t="s">
+        <v>80</v>
+      </c>
+      <c r="D67" s="151" t="s">
         <v>79</v>
       </c>
-      <c r="D67" s="217" t="s">
-        <v>78</v>
-      </c>
-      <c r="E67" s="218">
+      <c r="E67" s="152">
         <f>L67+P67+T67+X67</f>
         <v>-20.34262829557931</v>
       </c>
-      <c r="F67" s="223">
+      <c r="F67" s="125">
         <f>SUM(L68,P68,T68,X68)</f>
         <v>-24.141371751369434</v>
       </c>
-      <c r="G67" s="226">
+      <c r="G67" s="128">
         <f>SUM(L69,P69,T69,X69)</f>
-        <v>-11.6</v>
-      </c>
-      <c r="H67" s="120" t="s">
+        <v>-14.40318635548517</v>
+      </c>
+      <c r="H67" s="123" t="s">
         <v>26</v>
       </c>
       <c r="I67" s="74">
@@ -6222,13 +6309,13 @@
       </c>
     </row>
     <row r="68" spans="2:24" ht="15" customHeight="1">
-      <c r="B68" s="187"/>
-      <c r="C68" s="216"/>
-      <c r="D68" s="217"/>
-      <c r="E68" s="218"/>
-      <c r="F68" s="224"/>
-      <c r="G68" s="226"/>
-      <c r="H68" s="120" t="s">
+      <c r="B68" s="148"/>
+      <c r="C68" s="150"/>
+      <c r="D68" s="151"/>
+      <c r="E68" s="152"/>
+      <c r="F68" s="126"/>
+      <c r="G68" s="128"/>
+      <c r="H68" s="123" t="s">
         <v>27</v>
       </c>
       <c r="I68" s="74">
@@ -6285,13 +6372,13 @@
       </c>
     </row>
     <row r="69" spans="2:24" ht="15" customHeight="1">
-      <c r="B69" s="215"/>
-      <c r="C69" s="216"/>
-      <c r="D69" s="217"/>
-      <c r="E69" s="218"/>
-      <c r="F69" s="225"/>
-      <c r="G69" s="226"/>
-      <c r="H69" s="120" t="s">
+      <c r="B69" s="149"/>
+      <c r="C69" s="150"/>
+      <c r="D69" s="151"/>
+      <c r="E69" s="152"/>
+      <c r="F69" s="127"/>
+      <c r="G69" s="128"/>
+      <c r="H69" s="123" t="s">
         <v>28</v>
       </c>
       <c r="I69" s="89">
@@ -6316,21 +6403,23 @@
       <c r="O69" s="89">
         <v>-1.4</v>
       </c>
-      <c r="P69" s="116">
+      <c r="P69" s="115">
         <f t="shared" si="9"/>
         <v>-6.6</v>
       </c>
-      <c r="Q69" s="74"/>
+      <c r="Q69" s="82">
+        <v>-2.8031863554851699</v>
+      </c>
       <c r="R69" s="74"/>
       <c r="S69" s="74"/>
-      <c r="T69" s="113">
+      <c r="T69" s="112">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-2.8031863554851699</v>
       </c>
       <c r="U69" s="74"/>
       <c r="V69" s="74"/>
       <c r="W69" s="74"/>
-      <c r="X69" s="113">
+      <c r="X69" s="112">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -6349,31 +6438,84 @@
     </row>
   </sheetData>
   <mergeCells count="127">
-    <mergeCell ref="F67:F69"/>
-    <mergeCell ref="G67:G69"/>
-    <mergeCell ref="G64:G66"/>
-    <mergeCell ref="M62:O62"/>
-    <mergeCell ref="Q62:S62"/>
-    <mergeCell ref="G61:G63"/>
-    <mergeCell ref="F58:F60"/>
-    <mergeCell ref="G58:G60"/>
-    <mergeCell ref="I62:K62"/>
-    <mergeCell ref="F64:F66"/>
-    <mergeCell ref="F61:F63"/>
-    <mergeCell ref="C64:C66"/>
-    <mergeCell ref="D64:D66"/>
-    <mergeCell ref="E64:E66"/>
-    <mergeCell ref="C55:C57"/>
-    <mergeCell ref="D55:D57"/>
-    <mergeCell ref="E55:E57"/>
-    <mergeCell ref="C61:C63"/>
-    <mergeCell ref="B61:B69"/>
-    <mergeCell ref="C67:C69"/>
-    <mergeCell ref="D67:D69"/>
-    <mergeCell ref="E67:E69"/>
-    <mergeCell ref="D61:D63"/>
-    <mergeCell ref="E61:E63"/>
-    <mergeCell ref="E58:E60"/>
+    <mergeCell ref="G19:G21"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="D19:D21"/>
+    <mergeCell ref="E19:E21"/>
+    <mergeCell ref="G49:G51"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="G55:G57"/>
+    <mergeCell ref="G22:G24"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="D37:D39"/>
+    <mergeCell ref="F19:F21"/>
+    <mergeCell ref="F22:F24"/>
+    <mergeCell ref="F31:F33"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="D43:D45"/>
+    <mergeCell ref="F28:F30"/>
+    <mergeCell ref="G28:G30"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="F46:F48"/>
+    <mergeCell ref="G46:G48"/>
+    <mergeCell ref="M56:O56"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="Q56:S56"/>
+    <mergeCell ref="U56:W56"/>
+    <mergeCell ref="M53:O53"/>
+    <mergeCell ref="Q53:S53"/>
+    <mergeCell ref="U53:W53"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="F34:F36"/>
+    <mergeCell ref="F52:F54"/>
+    <mergeCell ref="G52:G54"/>
+    <mergeCell ref="F40:F42"/>
+    <mergeCell ref="G40:G42"/>
+    <mergeCell ref="E43:E45"/>
+    <mergeCell ref="F43:F45"/>
+    <mergeCell ref="G43:G45"/>
+    <mergeCell ref="E37:E39"/>
+    <mergeCell ref="F37:F39"/>
+    <mergeCell ref="G37:G39"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="D22:D24"/>
+    <mergeCell ref="E22:E24"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="D28:D30"/>
+    <mergeCell ref="E28:E30"/>
+    <mergeCell ref="I2:X2"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="D49:D51"/>
+    <mergeCell ref="E49:E51"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="E31:E33"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="G4:G6"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="F10:F12"/>
+    <mergeCell ref="G10:G12"/>
+    <mergeCell ref="F7:F9"/>
+    <mergeCell ref="G31:G33"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="G7:G9"/>
+    <mergeCell ref="G34:G36"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="F13:F15"/>
     <mergeCell ref="G13:G15"/>
     <mergeCell ref="B58:B60"/>
     <mergeCell ref="C58:C60"/>
@@ -6398,84 +6540,31 @@
     <mergeCell ref="B4:B18"/>
     <mergeCell ref="C31:C33"/>
     <mergeCell ref="C10:C12"/>
-    <mergeCell ref="I2:X2"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="D49:D51"/>
-    <mergeCell ref="E49:E51"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="D31:D33"/>
-    <mergeCell ref="E31:E33"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="D16:D18"/>
-    <mergeCell ref="G4:G6"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="F10:F12"/>
-    <mergeCell ref="G10:G12"/>
-    <mergeCell ref="F7:F9"/>
-    <mergeCell ref="G31:G33"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="F16:F18"/>
-    <mergeCell ref="G7:G9"/>
-    <mergeCell ref="G34:G36"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="F13:F15"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="E10:E12"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="D22:D24"/>
-    <mergeCell ref="E22:E24"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="D28:D30"/>
-    <mergeCell ref="E28:E30"/>
-    <mergeCell ref="M56:O56"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="Q56:S56"/>
-    <mergeCell ref="U56:W56"/>
-    <mergeCell ref="M53:O53"/>
-    <mergeCell ref="Q53:S53"/>
-    <mergeCell ref="U53:W53"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="F34:F36"/>
-    <mergeCell ref="F52:F54"/>
-    <mergeCell ref="G52:G54"/>
-    <mergeCell ref="F40:F42"/>
-    <mergeCell ref="G40:G42"/>
-    <mergeCell ref="E43:E45"/>
-    <mergeCell ref="F43:F45"/>
-    <mergeCell ref="G43:G45"/>
-    <mergeCell ref="E37:E39"/>
-    <mergeCell ref="F37:F39"/>
-    <mergeCell ref="G37:G39"/>
-    <mergeCell ref="G19:G21"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="C19:C21"/>
-    <mergeCell ref="D19:D21"/>
-    <mergeCell ref="E19:E21"/>
-    <mergeCell ref="G49:G51"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="G55:G57"/>
-    <mergeCell ref="G22:G24"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="D37:D39"/>
-    <mergeCell ref="F19:F21"/>
-    <mergeCell ref="F22:F24"/>
-    <mergeCell ref="F31:F33"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="D43:D45"/>
-    <mergeCell ref="F28:F30"/>
-    <mergeCell ref="G28:G30"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="F46:F48"/>
-    <mergeCell ref="G46:G48"/>
+    <mergeCell ref="C64:C66"/>
+    <mergeCell ref="D64:D66"/>
+    <mergeCell ref="E64:E66"/>
+    <mergeCell ref="C55:C57"/>
+    <mergeCell ref="D55:D57"/>
+    <mergeCell ref="E55:E57"/>
+    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="B61:B69"/>
+    <mergeCell ref="C67:C69"/>
+    <mergeCell ref="D67:D69"/>
+    <mergeCell ref="E67:E69"/>
+    <mergeCell ref="D61:D63"/>
+    <mergeCell ref="E61:E63"/>
+    <mergeCell ref="E58:E60"/>
+    <mergeCell ref="F67:F69"/>
+    <mergeCell ref="G67:G69"/>
+    <mergeCell ref="G64:G66"/>
+    <mergeCell ref="M62:O62"/>
+    <mergeCell ref="Q62:S62"/>
+    <mergeCell ref="G61:G63"/>
+    <mergeCell ref="F58:F60"/>
+    <mergeCell ref="G58:G60"/>
+    <mergeCell ref="I62:K62"/>
+    <mergeCell ref="F64:F66"/>
+    <mergeCell ref="F61:F63"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6496,55 +6585,55 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="29.1">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="28.9">
       <c r="A3" s="31" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="41" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B4" s="41" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="29.1">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="28.9">
       <c r="A5" s="41" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B5" s="41" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="62" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B6" s="62" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="31" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.6">
       <c r="A8" s="64" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B8" s="64"/>
       <c r="C8" s="30"/>
@@ -6554,7 +6643,7 @@
     </row>
     <row r="9" spans="1:6" ht="15.6">
       <c r="A9" s="64" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B9" s="64"/>
       <c r="C9" s="30"/>
@@ -6562,24 +6651,24 @@
       <c r="E9" s="30"/>
       <c r="F9" s="30"/>
     </row>
-    <row r="10" spans="1:6" ht="77.45">
+    <row r="10" spans="1:6" ht="78">
       <c r="A10" s="42" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B10" s="42" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C10" s="30"/>
       <c r="D10" s="30"/>
       <c r="E10" s="30"/>
       <c r="F10" s="30"/>
     </row>
-    <row r="11" spans="1:6" ht="46.5">
+    <row r="11" spans="1:6" ht="46.9">
       <c r="A11" s="42" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B11" s="42" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C11" s="30"/>
       <c r="D11" s="30"/>
@@ -6588,25 +6677,25 @@
     </row>
     <row r="12" spans="1:6" ht="15.6">
       <c r="A12" s="62" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C12" s="30"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="62" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.6">
       <c r="A14" s="31" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C14" s="30"/>
       <c r="D14" s="30"/>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="31" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -6626,26 +6715,26 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="F1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="B2" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="B3" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:6" outlineLevel="1">
@@ -6653,35 +6742,35 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:6" outlineLevel="1">
       <c r="B5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:6" outlineLevel="1">
       <c r="B6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:6" outlineLevel="1">
       <c r="B7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -6808,10 +6897,10 @@
     </row>
     <row r="26" spans="1:4">
       <c r="B26" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D26" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -6901,15 +6990,15 @@
     </row>
     <row r="44" spans="1:3">
       <c r="B44" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C44" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Preview: Week of 2026-09-14 — built 2026-09-11T11:36:10Z
</commit_message>
<xml_diff>
--- a/data/2026 Bowler Chart - OFS Training.xlsx
+++ b/data/2026 Bowler Chart - OFS Training.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\212448292\AppData\Local\Box\Box Edit\Documents\yHKq1N8p9kanefDTz1B5ig==\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\212529239\AppData\Local\Box\Box Edit\Documents\Z0nl+M3vCk+t6PhhVzER4Q==\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{A0FF72AF-E087-4B8F-939D-96A71C71115B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{099FC471-C0B4-45E1-B458-985519A21C3B}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="13_ncr:1_{3E31836C-1E49-40FF-A81F-A1F905B5151F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{246048CA-BDDC-44E9-95CD-181E933AAAA5}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-48" windowWidth="23256" windowHeight="12456" tabRatio="601" xr2:uid="{8476BB21-6D10-4BB9-B6CE-FEFD481D0662}"/>
+    <workbookView xWindow="51480" yWindow="3120" windowWidth="29040" windowHeight="15720" tabRatio="601" xr2:uid="{8476BB21-6D10-4BB9-B6CE-FEFD481D0662}"/>
   </bookViews>
   <sheets>
     <sheet name="Bowler L1 Training" sheetId="16" r:id="rId1"/>
@@ -43,6 +43,7 @@
     <author>tc={06BE996C-F791-4A9F-AA6D-EE2A8EE2F4C3}</author>
     <author>Jen Wright</author>
     <author>tc={17407CA0-19D6-410B-BD94-9BBC65BFCC7C}</author>
+    <author>tc={37C346EB-164E-421B-B3A5-A71619208C83}</author>
     <author>tc={160740E7-DFEB-4450-B5C5-A17286B215D6}</author>
     <author>Philip Ganssmann</author>
     <author>tc={50577B9E-D913-49BB-B91E-A5BD3E934319}</author>
@@ -87,7 +88,15 @@
     I&amp;I FW 33 1.089</t>
       </text>
     </comment>
-    <comment ref="F13" authorId="3" shapeId="0" xr:uid="{160740E7-DFEB-4450-B5C5-A17286B215D6}">
+    <comment ref="R9" authorId="3" shapeId="0" xr:uid="{37C346EB-164E-421B-B3A5-A71619208C83}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    estimated I&amp;I rate for now. Rate will change by next week</t>
+      </text>
+    </comment>
+    <comment ref="F13" authorId="4" shapeId="0" xr:uid="{160740E7-DFEB-4450-B5C5-A17286B215D6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -95,7 +104,7 @@
     90% RA ATS closure rate all sites by YE</t>
       </text>
     </comment>
-    <comment ref="I24" authorId="4" shapeId="0" xr:uid="{295EE1B2-A25B-412E-A639-7B1259576743}">
+    <comment ref="I24" authorId="5" shapeId="0" xr:uid="{295EE1B2-A25B-412E-A639-7B1259576743}">
       <text>
         <r>
           <rPr>
@@ -110,7 +119,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J24" authorId="4" shapeId="0" xr:uid="{DC09360C-6AE1-46FC-ABAD-4D81C3945042}">
+    <comment ref="J24" authorId="5" shapeId="0" xr:uid="{DC09360C-6AE1-46FC-ABAD-4D81C3945042}">
       <text>
         <r>
           <rPr>
@@ -129,7 +138,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K24" authorId="4" shapeId="0" xr:uid="{64E9CAD9-580E-40D0-B2F1-25AC4998B65A}">
+    <comment ref="K24" authorId="5" shapeId="0" xr:uid="{64E9CAD9-580E-40D0-B2F1-25AC4998B65A}">
       <text>
         <r>
           <rPr>
@@ -146,7 +155,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N24" authorId="4" shapeId="0" xr:uid="{7B5163D0-287F-484F-B9B7-4BE35DBAC943}">
+    <comment ref="N24" authorId="5" shapeId="0" xr:uid="{7B5163D0-287F-484F-B9B7-4BE35DBAC943}">
       <text>
         <r>
           <rPr>
@@ -163,7 +172,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I27" authorId="4" shapeId="0" xr:uid="{90DAD1A6-212D-45E4-8528-2D901E1C0C5A}">
+    <comment ref="I27" authorId="5" shapeId="0" xr:uid="{90DAD1A6-212D-45E4-8528-2D901E1C0C5A}">
       <text>
         <r>
           <rPr>
@@ -178,7 +187,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J27" authorId="4" shapeId="0" xr:uid="{7392AAE5-E54D-4232-B7DC-129B156C6F62}">
+    <comment ref="J27" authorId="5" shapeId="0" xr:uid="{7392AAE5-E54D-4232-B7DC-129B156C6F62}">
       <text>
         <r>
           <rPr>
@@ -205,7 +214,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K27" authorId="4" shapeId="0" xr:uid="{76FCDDC0-41DD-4A57-9E0C-979F0DC1595C}">
+    <comment ref="K27" authorId="5" shapeId="0" xr:uid="{76FCDDC0-41DD-4A57-9E0C-979F0DC1595C}">
       <text>
         <r>
           <rPr>
@@ -232,7 +241,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L27" authorId="4" shapeId="0" xr:uid="{C1388240-DDDB-4DD1-B7FE-11B7EF9BDF13}">
+    <comment ref="L27" authorId="5" shapeId="0" xr:uid="{C1388240-DDDB-4DD1-B7FE-11B7EF9BDF13}">
       <text>
         <r>
           <rPr>
@@ -364,7 +373,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O42" authorId="5" shapeId="0" xr:uid="{50577B9E-D913-49BB-B91E-A5BD3E934319}">
+    <comment ref="O42" authorId="6" shapeId="0" xr:uid="{50577B9E-D913-49BB-B91E-A5BD3E934319}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -449,7 +458,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K51" authorId="6" shapeId="0" xr:uid="{4A61949D-D058-4614-9CBE-136784BCC6E7}">
+    <comment ref="K51" authorId="7" shapeId="0" xr:uid="{4A61949D-D058-4614-9CBE-136784BCC6E7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -459,7 +468,7 @@
 As tracking stabilizes and system issues are resolved, the data will more accurately reflect true performance and is expected to improve.</t>
       </text>
     </comment>
-    <comment ref="M51" authorId="7" shapeId="0" xr:uid="{40736F15-DF93-4810-BC49-A79E1FB56ED1}">
+    <comment ref="M51" authorId="8" shapeId="0" xr:uid="{40736F15-DF93-4810-BC49-A79E1FB56ED1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -467,7 +476,7 @@
     https://gevernova.box.com/s/17o8hpcpubfb6lm82c157gdcde9kcful</t>
       </text>
     </comment>
-    <comment ref="Q51" authorId="8" shapeId="0" xr:uid="{F644D89E-1836-4B19-B5E0-2664B9B5862D}">
+    <comment ref="Q51" authorId="9" shapeId="0" xr:uid="{F644D89E-1836-4B19-B5E0-2664B9B5862D}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -537,12 +546,42 @@
         </r>
       </text>
     </comment>
+    <comment ref="R66" authorId="1" shapeId="0" xr:uid="{9B4E6628-812D-4C80-9A15-B8DCCE20236A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Jen Wright:
+Holding to plan - don't have visibility to August actuals  yet</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R69" authorId="1" shapeId="0" xr:uid="{8CE9D396-21E5-463C-8F92-EFD21B3F62A3}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Jen Wright:
+Holding to plan - don't have visibility to August actuals  yet</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="117">
   <si>
     <t>Level 2</t>
   </si>
@@ -620,7 +659,7 @@
     <t>I&amp;I</t>
   </si>
   <si>
-    <t>Galley</t>
+    <t>Arnold</t>
   </si>
   <si>
     <t>PY</t>
@@ -665,7 +704,7 @@
     <t>Daxer</t>
   </si>
   <si>
-    <t>Jul: ENBW (2 courses)-customer mgmt w/ very positive feedback, participants complaints about Sim not site specific; Mill Creek: not recommended, because GT-Maint not needed (LTSA); GECOL: students expected cash or credit card - outside of OFS TRG scope</t>
+    <t>Aug: OE Controls courses @ HLC w/ low rating because of AC and internet issues in building 3</t>
   </si>
   <si>
     <t># Exams Migrated to Xyleme</t>
@@ -794,7 +833,7 @@
     <t>GP TrainingOrg Gross Margin</t>
   </si>
   <si>
-    <t>Kandic</t>
+    <t>Sureshbabu</t>
   </si>
   <si>
     <t>FC Training Org Gross Margin</t>
@@ -1315,7 +1354,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="235">
+  <cellXfs count="236">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
@@ -1455,9 +1494,6 @@
     <xf numFmtId="1" fontId="22" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="22" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" indent="3"/>
-    </xf>
     <xf numFmtId="37" fontId="22" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1648,27 +1684,321 @@
     <xf numFmtId="37" fontId="7" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="27" fillId="8" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="37" fontId="7" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="3"/>
     </xf>
+    <xf numFmtId="9" fontId="27" fillId="8" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" indent="3"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="21" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="22" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="21" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="29" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="14" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="168" fontId="22" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1684,9 +2014,6 @@
     <xf numFmtId="168" fontId="30" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="171" fontId="21" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1699,305 +2026,20 @@
     <xf numFmtId="167" fontId="3" fillId="3" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="3" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="168" fontId="22" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="21" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="29" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="37" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="37" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="22" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="22" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="21" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="10" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="2" fontId="7" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="3"/>
+    </xf>
+    <xf numFmtId="39" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2335,6 +2377,9 @@
   <threadedComment ref="Q9" dT="2026-08-12T12:52:46.71" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{CFF977E5-20AE-4211-A668-ADE79729D017}" parentId="{17407CA0-19D6-410B-BD94-9BBC65BFCC7C}">
     <text>I&amp;I FW 33 1.089</text>
   </threadedComment>
+  <threadedComment ref="R9" dT="2026-09-09T13:18:12.41" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{37C346EB-164E-421B-B3A5-A71619208C83}">
+    <text>estimated I&amp;I rate for now. Rate will change by next week</text>
+  </threadedComment>
   <threadedComment ref="F13" dT="2024-05-21T17:14:25.01" personId="{F0C1FE1F-CA66-453D-BCFC-7F99948C8DD5}" id="{160740E7-DFEB-4450-B5C5-A17286B215D6}">
     <text>90% RA ATS closure rate all sites by YE</text>
   </threadedComment>
@@ -2414,24 +2459,24 @@
       <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="181">
+      <c r="I2" s="171">
         <v>2026</v>
       </c>
-      <c r="J2" s="182"/>
-      <c r="K2" s="182"/>
-      <c r="L2" s="182"/>
-      <c r="M2" s="182"/>
-      <c r="N2" s="182"/>
-      <c r="O2" s="182"/>
-      <c r="P2" s="182"/>
-      <c r="Q2" s="182"/>
-      <c r="R2" s="182"/>
-      <c r="S2" s="182"/>
-      <c r="T2" s="182"/>
-      <c r="U2" s="182"/>
-      <c r="V2" s="182"/>
-      <c r="W2" s="182"/>
-      <c r="X2" s="183"/>
+      <c r="J2" s="172"/>
+      <c r="K2" s="172"/>
+      <c r="L2" s="172"/>
+      <c r="M2" s="172"/>
+      <c r="N2" s="172"/>
+      <c r="O2" s="172"/>
+      <c r="P2" s="172"/>
+      <c r="Q2" s="172"/>
+      <c r="R2" s="172"/>
+      <c r="S2" s="172"/>
+      <c r="T2" s="172"/>
+      <c r="U2" s="172"/>
+      <c r="V2" s="172"/>
+      <c r="W2" s="172"/>
+      <c r="X2" s="173"/>
     </row>
     <row r="3" spans="1:25" ht="31.15">
       <c r="A3" s="5"/>
@@ -2504,23 +2549,23 @@
       </c>
     </row>
     <row r="4" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B4" s="162" t="s">
+      <c r="B4" s="193" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="180" t="s">
+      <c r="C4" s="178" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="187" t="s">
+      <c r="D4" s="164" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="188">
+      <c r="E4" s="180">
         <f>SUM(L4,P4,T4,X4)</f>
         <v>0</v>
       </c>
-      <c r="F4" s="191">
-        <v>0</v>
-      </c>
-      <c r="G4" s="190">
+      <c r="F4" s="124">
+        <v>0</v>
+      </c>
+      <c r="G4" s="181">
         <f>SUM(L6,P6,T6,X6)</f>
         <v>1</v>
       </c>
@@ -2581,12 +2626,12 @@
       </c>
     </row>
     <row r="5" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B5" s="162"/>
-      <c r="C5" s="180"/>
-      <c r="D5" s="187"/>
-      <c r="E5" s="188"/>
-      <c r="F5" s="191"/>
-      <c r="G5" s="190"/>
+      <c r="B5" s="193"/>
+      <c r="C5" s="178"/>
+      <c r="D5" s="164"/>
+      <c r="E5" s="180"/>
+      <c r="F5" s="124"/>
+      <c r="G5" s="181"/>
       <c r="H5" s="11" t="s">
         <v>27</v>
       </c>
@@ -2644,45 +2689,47 @@
       </c>
     </row>
     <row r="6" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B6" s="162"/>
-      <c r="C6" s="180"/>
-      <c r="D6" s="187"/>
-      <c r="E6" s="188"/>
-      <c r="F6" s="191"/>
-      <c r="G6" s="190"/>
+      <c r="B6" s="193"/>
+      <c r="C6" s="178"/>
+      <c r="D6" s="164"/>
+      <c r="E6" s="180"/>
+      <c r="F6" s="124"/>
+      <c r="G6" s="181"/>
       <c r="H6" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="87">
-        <v>0</v>
-      </c>
-      <c r="J6" s="87">
-        <v>0</v>
-      </c>
-      <c r="K6" s="87">
-        <v>0</v>
-      </c>
-      <c r="L6" s="98">
+      <c r="I6" s="86">
+        <v>0</v>
+      </c>
+      <c r="J6" s="86">
+        <v>0</v>
+      </c>
+      <c r="K6" s="86">
+        <v>0</v>
+      </c>
+      <c r="L6" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M6" s="87">
-        <v>0</v>
-      </c>
-      <c r="N6" s="87">
-        <v>0</v>
-      </c>
-      <c r="O6" s="116">
-        <v>0</v>
-      </c>
-      <c r="P6" s="98">
+      <c r="M6" s="86">
+        <v>0</v>
+      </c>
+      <c r="N6" s="86">
+        <v>0</v>
+      </c>
+      <c r="O6" s="115">
+        <v>0</v>
+      </c>
+      <c r="P6" s="97">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q6" s="117">
+      <c r="Q6" s="116">
         <v>1</v>
       </c>
-      <c r="R6" s="14"/>
+      <c r="R6" s="86">
+        <v>0</v>
+      </c>
       <c r="S6" s="14"/>
       <c r="T6" s="13">
         <f t="shared" si="2"/>
@@ -2697,21 +2744,21 @@
       </c>
     </row>
     <row r="7" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B7" s="162"/>
-      <c r="C7" s="143" t="s">
+      <c r="B7" s="193"/>
+      <c r="C7" s="127" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="170" t="s">
+      <c r="D7" s="128" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="202">
-        <v>0</v>
-      </c>
-      <c r="F7" s="192">
-        <v>0</v>
-      </c>
-      <c r="G7" s="195">
-        <v>1.089</v>
+      <c r="E7" s="165">
+        <v>0</v>
+      </c>
+      <c r="F7" s="182">
+        <v>0</v>
+      </c>
+      <c r="G7" s="234">
+        <v>0.95</v>
       </c>
       <c r="H7" s="121" t="s">
         <v>26</v>
@@ -2766,12 +2813,12 @@
       </c>
     </row>
     <row r="8" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B8" s="162"/>
-      <c r="C8" s="143"/>
-      <c r="D8" s="170"/>
-      <c r="E8" s="203"/>
-      <c r="F8" s="192"/>
-      <c r="G8" s="195"/>
+      <c r="B8" s="193"/>
+      <c r="C8" s="127"/>
+      <c r="D8" s="128"/>
+      <c r="E8" s="166"/>
+      <c r="F8" s="182"/>
+      <c r="G8" s="234"/>
       <c r="H8" s="121" t="s">
         <v>27</v>
       </c>
@@ -2825,43 +2872,45 @@
       </c>
     </row>
     <row r="9" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B9" s="162"/>
-      <c r="C9" s="143"/>
-      <c r="D9" s="170"/>
-      <c r="E9" s="204"/>
-      <c r="F9" s="192"/>
-      <c r="G9" s="195"/>
+      <c r="B9" s="193"/>
+      <c r="C9" s="127"/>
+      <c r="D9" s="128"/>
+      <c r="E9" s="167"/>
+      <c r="F9" s="182"/>
+      <c r="G9" s="234"/>
       <c r="H9" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="I9" s="86">
-        <v>0</v>
-      </c>
-      <c r="J9" s="86">
-        <v>0</v>
-      </c>
-      <c r="K9" s="86">
-        <v>0</v>
-      </c>
-      <c r="L9" s="98">
-        <v>0</v>
-      </c>
-      <c r="M9" s="86">
-        <v>0</v>
-      </c>
-      <c r="N9" s="86">
-        <v>0</v>
-      </c>
-      <c r="O9" s="86">
-        <v>0</v>
-      </c>
-      <c r="P9" s="98">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="124">
+      <c r="I9" s="85">
+        <v>0</v>
+      </c>
+      <c r="J9" s="85">
+        <v>0</v>
+      </c>
+      <c r="K9" s="85">
+        <v>0</v>
+      </c>
+      <c r="L9" s="97">
+        <v>0</v>
+      </c>
+      <c r="M9" s="85">
+        <v>0</v>
+      </c>
+      <c r="N9" s="85">
+        <v>0</v>
+      </c>
+      <c r="O9" s="85">
+        <v>0</v>
+      </c>
+      <c r="P9" s="97">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="117">
         <v>1.089</v>
       </c>
-      <c r="R9" s="45"/>
+      <c r="R9" s="233">
+        <v>0.95</v>
+      </c>
       <c r="S9" s="45"/>
       <c r="T9" s="44"/>
       <c r="U9" s="45"/>
@@ -2870,22 +2919,22 @@
       <c r="X9" s="16"/>
     </row>
     <row r="10" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B10" s="162"/>
-      <c r="C10" s="180" t="s">
+      <c r="B10" s="193"/>
+      <c r="C10" s="178" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="187" t="s">
+      <c r="D10" s="164" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="201">
+      <c r="E10" s="135">
         <f>SUM(L10,P10,T10,X10)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="191">
+      <c r="F10" s="124">
         <f>SUM(L11,P11,T11,X11)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="188">
+      <c r="G10" s="180">
         <f>SUM(L12,P12,T12,X12)</f>
         <v>0</v>
       </c>
@@ -2946,12 +2995,12 @@
       </c>
     </row>
     <row r="11" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B11" s="162"/>
-      <c r="C11" s="180"/>
-      <c r="D11" s="187"/>
-      <c r="E11" s="201"/>
-      <c r="F11" s="191"/>
-      <c r="G11" s="188"/>
+      <c r="B11" s="193"/>
+      <c r="C11" s="178"/>
+      <c r="D11" s="164"/>
+      <c r="E11" s="135"/>
+      <c r="F11" s="124"/>
+      <c r="G11" s="180"/>
       <c r="H11" s="11" t="s">
         <v>27</v>
       </c>
@@ -3009,45 +3058,47 @@
       </c>
     </row>
     <row r="12" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B12" s="162"/>
-      <c r="C12" s="180"/>
-      <c r="D12" s="187"/>
-      <c r="E12" s="201"/>
-      <c r="F12" s="191"/>
-      <c r="G12" s="188"/>
+      <c r="B12" s="193"/>
+      <c r="C12" s="178"/>
+      <c r="D12" s="164"/>
+      <c r="E12" s="135"/>
+      <c r="F12" s="124"/>
+      <c r="G12" s="180"/>
       <c r="H12" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="I12" s="87">
-        <v>0</v>
-      </c>
-      <c r="J12" s="87">
-        <v>0</v>
-      </c>
-      <c r="K12" s="87">
-        <v>0</v>
-      </c>
-      <c r="L12" s="98">
+      <c r="I12" s="86">
+        <v>0</v>
+      </c>
+      <c r="J12" s="86">
+        <v>0</v>
+      </c>
+      <c r="K12" s="86">
+        <v>0</v>
+      </c>
+      <c r="L12" s="97">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="M12" s="87">
-        <v>0</v>
-      </c>
-      <c r="N12" s="87">
-        <v>0</v>
-      </c>
-      <c r="O12" s="87">
-        <v>0</v>
-      </c>
-      <c r="P12" s="98">
+      <c r="M12" s="86">
+        <v>0</v>
+      </c>
+      <c r="N12" s="86">
+        <v>0</v>
+      </c>
+      <c r="O12" s="86">
+        <v>0</v>
+      </c>
+      <c r="P12" s="97">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Q12" s="87">
-        <v>0</v>
-      </c>
-      <c r="R12" s="14"/>
+      <c r="Q12" s="86">
+        <v>0</v>
+      </c>
+      <c r="R12" s="86">
+        <v>0</v>
+      </c>
       <c r="S12" s="14"/>
       <c r="T12" s="13">
         <f t="shared" si="6"/>
@@ -3062,20 +3113,20 @@
       </c>
     </row>
     <row r="13" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B13" s="162"/>
-      <c r="C13" s="143" t="s">
+      <c r="B13" s="193"/>
+      <c r="C13" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="170" t="s">
+      <c r="D13" s="128" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="155">
+      <c r="E13" s="179">
         <v>1</v>
       </c>
-      <c r="F13" s="200">
-        <v>0.9</v>
-      </c>
-      <c r="G13" s="155">
+      <c r="F13" s="143">
+        <v>0.9</v>
+      </c>
+      <c r="G13" s="179">
         <v>0.9</v>
       </c>
       <c r="H13" s="121" t="s">
@@ -3131,12 +3182,12 @@
       </c>
     </row>
     <row r="14" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B14" s="162"/>
-      <c r="C14" s="143"/>
-      <c r="D14" s="170"/>
-      <c r="E14" s="155"/>
-      <c r="F14" s="200"/>
-      <c r="G14" s="155"/>
+      <c r="B14" s="193"/>
+      <c r="C14" s="127"/>
+      <c r="D14" s="128"/>
+      <c r="E14" s="179"/>
+      <c r="F14" s="143"/>
+      <c r="G14" s="179"/>
       <c r="H14" s="121" t="s">
         <v>27</v>
       </c>
@@ -3149,7 +3200,7 @@
       <c r="K14" s="38">
         <v>0.9</v>
       </c>
-      <c r="L14" s="93">
+      <c r="L14" s="92">
         <v>0.9</v>
       </c>
       <c r="M14" s="38">
@@ -3190,43 +3241,45 @@
       </c>
     </row>
     <row r="15" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B15" s="162"/>
-      <c r="C15" s="143"/>
-      <c r="D15" s="170"/>
-      <c r="E15" s="155"/>
-      <c r="F15" s="200"/>
-      <c r="G15" s="155"/>
+      <c r="B15" s="193"/>
+      <c r="C15" s="127"/>
+      <c r="D15" s="128"/>
+      <c r="E15" s="179"/>
+      <c r="F15" s="143"/>
+      <c r="G15" s="179"/>
       <c r="H15" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="I15" s="77">
-        <v>0.9</v>
-      </c>
-      <c r="J15" s="77" t="s">
-        <v>32</v>
-      </c>
-      <c r="K15" s="77" t="s">
+      <c r="I15" s="76">
+        <v>0.9</v>
+      </c>
+      <c r="J15" s="76" t="s">
+        <v>32</v>
+      </c>
+      <c r="K15" s="76" t="s">
         <v>33</v>
       </c>
-      <c r="L15" s="88">
-        <v>0.9</v>
-      </c>
-      <c r="M15" s="77">
-        <v>0.9</v>
-      </c>
-      <c r="N15" s="77">
-        <v>0.9</v>
-      </c>
-      <c r="O15" s="77" t="s">
-        <v>32</v>
-      </c>
-      <c r="P15" s="88">
-        <v>0.9</v>
-      </c>
-      <c r="Q15" s="77" t="s">
-        <v>32</v>
-      </c>
-      <c r="R15" s="47"/>
+      <c r="L15" s="87">
+        <v>0.9</v>
+      </c>
+      <c r="M15" s="76">
+        <v>0.9</v>
+      </c>
+      <c r="N15" s="76">
+        <v>0.9</v>
+      </c>
+      <c r="O15" s="76" t="s">
+        <v>32</v>
+      </c>
+      <c r="P15" s="87">
+        <v>0.9</v>
+      </c>
+      <c r="Q15" s="76" t="s">
+        <v>32</v>
+      </c>
+      <c r="R15" s="76" t="s">
+        <v>32</v>
+      </c>
       <c r="S15" s="47"/>
       <c r="T15" s="48"/>
       <c r="U15" s="47"/>
@@ -3235,23 +3288,23 @@
       <c r="X15" s="16"/>
     </row>
     <row r="16" spans="1:25" ht="18.75" customHeight="1">
-      <c r="B16" s="162"/>
-      <c r="C16" s="205" t="s">
+      <c r="B16" s="193"/>
+      <c r="C16" s="125" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="189" t="s">
+      <c r="D16" s="169" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="191" t="s">
+      <c r="E16" s="124" t="s">
         <v>35</v>
       </c>
-      <c r="F16" s="193">
-        <v>0.9</v>
-      </c>
-      <c r="G16" s="198">
+      <c r="F16" s="155">
+        <v>0.9</v>
+      </c>
+      <c r="G16" s="152">
         <v>0.95</v>
       </c>
-      <c r="H16" s="120" t="s">
+      <c r="H16" s="123" t="s">
         <v>26</v>
       </c>
       <c r="I16" s="19" t="s">
@@ -3302,18 +3355,18 @@
       <c r="X16" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="Y16" s="55" t="s">
+      <c r="Y16" s="54" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="17" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B17" s="162"/>
-      <c r="C17" s="163"/>
-      <c r="D17" s="189"/>
-      <c r="E17" s="191"/>
-      <c r="F17" s="193"/>
-      <c r="G17" s="198"/>
-      <c r="H17" s="120" t="s">
+      <c r="B17" s="193"/>
+      <c r="C17" s="126"/>
+      <c r="D17" s="169"/>
+      <c r="E17" s="124"/>
+      <c r="F17" s="155"/>
+      <c r="G17" s="152"/>
+      <c r="H17" s="123" t="s">
         <v>27</v>
       </c>
       <c r="I17" s="21">
@@ -3366,247 +3419,251 @@
       </c>
     </row>
     <row r="18" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B18" s="162"/>
-      <c r="C18" s="163"/>
-      <c r="D18" s="189"/>
-      <c r="E18" s="191"/>
-      <c r="F18" s="194"/>
-      <c r="G18" s="199"/>
-      <c r="H18" s="120" t="s">
+      <c r="B18" s="193"/>
+      <c r="C18" s="126"/>
+      <c r="D18" s="169"/>
+      <c r="E18" s="124"/>
+      <c r="F18" s="183"/>
+      <c r="G18" s="153"/>
+      <c r="H18" s="123" t="s">
         <v>28</v>
       </c>
-      <c r="I18" s="85">
+      <c r="I18" s="84">
         <v>0.92300000000000004</v>
       </c>
-      <c r="J18" s="77">
-        <v>0.9</v>
-      </c>
-      <c r="K18" s="85">
+      <c r="J18" s="76">
+        <v>0.9</v>
+      </c>
+      <c r="K18" s="84">
         <v>0.92300000000000004</v>
       </c>
-      <c r="L18" s="94">
+      <c r="L18" s="93">
         <v>0.92</v>
       </c>
-      <c r="M18" s="118">
+      <c r="M18" s="84">
         <v>1</v>
       </c>
-      <c r="N18" s="118">
+      <c r="N18" s="84">
         <v>1</v>
       </c>
-      <c r="O18" s="104">
+      <c r="O18" s="103">
         <v>84.6</v>
       </c>
-      <c r="P18" s="94">
+      <c r="P18" s="93">
         <v>0.95</v>
       </c>
-      <c r="Q18" s="118">
+      <c r="Q18" s="84">
         <v>1</v>
       </c>
-      <c r="R18" s="53"/>
+      <c r="R18" s="118">
+        <v>1</v>
+      </c>
       <c r="S18" s="52"/>
       <c r="T18" s="43"/>
       <c r="U18" s="52"/>
-      <c r="V18" s="54"/>
-      <c r="W18" s="54"/>
+      <c r="V18" s="53"/>
+      <c r="W18" s="53"/>
       <c r="X18" s="43"/>
     </row>
     <row r="19" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B19" s="162" t="s">
+      <c r="B19" s="193" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="143" t="s">
+      <c r="C19" s="127" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="170" t="s">
+      <c r="D19" s="128" t="s">
         <v>39</v>
       </c>
-      <c r="E19" s="218">
+      <c r="E19" s="129">
         <v>83</v>
       </c>
-      <c r="F19" s="228">
+      <c r="F19" s="141">
         <v>83</v>
       </c>
-      <c r="G19" s="218">
-        <v>83.8</v>
+      <c r="G19" s="129">
+        <v>83.2</v>
       </c>
       <c r="H19" s="121" t="s">
         <v>26</v>
       </c>
-      <c r="I19" s="56">
+      <c r="I19" s="55">
         <v>80.3</v>
       </c>
-      <c r="J19" s="56">
+      <c r="J19" s="55">
         <v>89.2</v>
       </c>
-      <c r="K19" s="56">
+      <c r="K19" s="55">
         <v>81</v>
       </c>
-      <c r="L19" s="57">
+      <c r="L19" s="56">
         <v>83</v>
       </c>
-      <c r="M19" s="56">
+      <c r="M19" s="55">
         <v>88.6</v>
       </c>
-      <c r="N19" s="56">
+      <c r="N19" s="55">
         <v>86</v>
       </c>
-      <c r="O19" s="56">
+      <c r="O19" s="55">
         <v>82.7</v>
       </c>
-      <c r="P19" s="57">
+      <c r="P19" s="56">
         <v>86.3</v>
       </c>
-      <c r="Q19" s="56">
+      <c r="Q19" s="55">
         <v>82</v>
       </c>
-      <c r="R19" s="56">
+      <c r="R19" s="55">
         <v>79.400000000000006</v>
       </c>
-      <c r="S19" s="56">
+      <c r="S19" s="55">
         <v>83.2</v>
       </c>
-      <c r="T19" s="57">
+      <c r="T19" s="56">
         <v>81.599999999999994</v>
       </c>
-      <c r="U19" s="56">
+      <c r="U19" s="55">
         <v>79.099999999999994</v>
       </c>
-      <c r="V19" s="56">
+      <c r="V19" s="55">
         <v>83.6</v>
       </c>
-      <c r="W19" s="56">
+      <c r="W19" s="55">
         <v>72.8</v>
       </c>
-      <c r="X19" s="57">
+      <c r="X19" s="56">
         <v>80.099999999999994</v>
       </c>
     </row>
     <row r="20" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B20" s="162"/>
-      <c r="C20" s="143"/>
-      <c r="D20" s="170"/>
-      <c r="E20" s="219"/>
-      <c r="F20" s="229"/>
-      <c r="G20" s="219"/>
+      <c r="B20" s="193"/>
+      <c r="C20" s="127"/>
+      <c r="D20" s="128"/>
+      <c r="E20" s="130"/>
+      <c r="F20" s="142"/>
+      <c r="G20" s="130"/>
       <c r="H20" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I20" s="56">
+      <c r="I20" s="55">
         <v>83</v>
       </c>
-      <c r="J20" s="56">
+      <c r="J20" s="55">
         <v>83</v>
       </c>
-      <c r="K20" s="56">
+      <c r="K20" s="55">
         <v>83</v>
       </c>
-      <c r="L20" s="57">
+      <c r="L20" s="56">
         <v>83</v>
       </c>
-      <c r="M20" s="56">
+      <c r="M20" s="55">
         <v>83</v>
       </c>
-      <c r="N20" s="56">
+      <c r="N20" s="55">
         <v>83</v>
       </c>
-      <c r="O20" s="56">
+      <c r="O20" s="55">
         <v>83</v>
       </c>
-      <c r="P20" s="57">
+      <c r="P20" s="56">
         <v>83</v>
       </c>
-      <c r="Q20" s="56">
+      <c r="Q20" s="55">
         <v>83</v>
       </c>
-      <c r="R20" s="56">
+      <c r="R20" s="55">
         <v>83</v>
       </c>
-      <c r="S20" s="56">
+      <c r="S20" s="55">
         <v>83</v>
       </c>
-      <c r="T20" s="57">
+      <c r="T20" s="56">
         <v>83</v>
       </c>
-      <c r="U20" s="56">
+      <c r="U20" s="55">
         <v>83</v>
       </c>
-      <c r="V20" s="56">
+      <c r="V20" s="55">
         <v>83</v>
       </c>
-      <c r="W20" s="56">
+      <c r="W20" s="55">
         <v>83</v>
       </c>
-      <c r="X20" s="57">
+      <c r="X20" s="56">
         <v>83</v>
       </c>
     </row>
     <row r="21" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B21" s="162"/>
-      <c r="C21" s="143"/>
-      <c r="D21" s="170"/>
-      <c r="E21" s="219"/>
-      <c r="F21" s="229"/>
-      <c r="G21" s="219"/>
+      <c r="B21" s="193"/>
+      <c r="C21" s="127"/>
+      <c r="D21" s="128"/>
+      <c r="E21" s="130"/>
+      <c r="F21" s="142"/>
+      <c r="G21" s="130"/>
       <c r="H21" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="I21" s="76">
+      <c r="I21" s="75">
         <v>79</v>
       </c>
-      <c r="J21" s="84">
+      <c r="J21" s="83">
         <v>84</v>
       </c>
-      <c r="K21" s="84">
+      <c r="K21" s="83">
         <v>87</v>
       </c>
-      <c r="L21" s="90">
+      <c r="L21" s="89">
         <v>85</v>
       </c>
-      <c r="M21" s="76">
+      <c r="M21" s="75">
         <v>79</v>
       </c>
-      <c r="N21" s="105">
+      <c r="N21" s="104">
         <v>91</v>
       </c>
-      <c r="O21" s="76">
-        <v>78</v>
-      </c>
-      <c r="P21" s="90">
+      <c r="O21" s="75">
+        <v>75.8</v>
+      </c>
+      <c r="P21" s="89">
         <v>84.4</v>
       </c>
-      <c r="Q21" s="76">
-        <v>82.5</v>
-      </c>
-      <c r="R21" s="58"/>
-      <c r="S21" s="58"/>
-      <c r="T21" s="58"/>
-      <c r="U21" s="58"/>
-      <c r="V21" s="58"/>
-      <c r="W21" s="58"/>
+      <c r="Q21" s="104">
+        <v>84.7</v>
+      </c>
+      <c r="R21" s="75">
+        <v>82.9</v>
+      </c>
+      <c r="S21" s="57"/>
+      <c r="T21" s="57"/>
+      <c r="U21" s="57"/>
+      <c r="V21" s="57"/>
+      <c r="W21" s="57"/>
       <c r="X21" s="44"/>
       <c r="Y21" s="7" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="22" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B22" s="162"/>
-      <c r="C22" s="205" t="s">
+      <c r="B22" s="193"/>
+      <c r="C22" s="125" t="s">
         <v>41</v>
       </c>
-      <c r="D22" s="206" t="s">
+      <c r="D22" s="168" t="s">
         <v>42</v>
       </c>
-      <c r="E22" s="207" t="s">
+      <c r="E22" s="170" t="s">
         <v>35</v>
       </c>
-      <c r="F22" s="191">
+      <c r="F22" s="124">
         <v>55</v>
       </c>
-      <c r="G22" s="201">
+      <c r="G22" s="135">
         <f>SUM(L24,P24,T24,X24)</f>
-        <v>76</v>
-      </c>
-      <c r="H22" s="120" t="s">
+        <v>78</v>
+      </c>
+      <c r="H22" s="123" t="s">
         <v>26</v>
       </c>
       <c r="I22" s="24" t="s">
@@ -3657,18 +3714,18 @@
       <c r="X22" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="Y22" s="55" t="s">
+      <c r="Y22" s="54" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="23" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B23" s="162"/>
-      <c r="C23" s="163"/>
-      <c r="D23" s="189"/>
-      <c r="E23" s="207"/>
-      <c r="F23" s="191"/>
-      <c r="G23" s="201"/>
-      <c r="H23" s="120" t="s">
+      <c r="B23" s="193"/>
+      <c r="C23" s="126"/>
+      <c r="D23" s="169"/>
+      <c r="E23" s="170"/>
+      <c r="F23" s="124"/>
+      <c r="G23" s="135"/>
+      <c r="H23" s="123" t="s">
         <v>27</v>
       </c>
       <c r="I23" s="12">
@@ -3721,74 +3778,76 @@
       </c>
     </row>
     <row r="24" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B24" s="162"/>
-      <c r="C24" s="163"/>
-      <c r="D24" s="189"/>
-      <c r="E24" s="207"/>
-      <c r="F24" s="191"/>
-      <c r="G24" s="201"/>
-      <c r="H24" s="120" t="s">
+      <c r="B24" s="193"/>
+      <c r="C24" s="126"/>
+      <c r="D24" s="169"/>
+      <c r="E24" s="170"/>
+      <c r="F24" s="124"/>
+      <c r="G24" s="135"/>
+      <c r="H24" s="123" t="s">
         <v>28</v>
       </c>
-      <c r="I24" s="86">
+      <c r="I24" s="85">
         <v>2</v>
       </c>
-      <c r="J24" s="84">
+      <c r="J24" s="83">
         <v>5</v>
       </c>
-      <c r="K24" s="80">
+      <c r="K24" s="79">
         <v>3</v>
       </c>
-      <c r="L24" s="99">
+      <c r="L24" s="98">
         <v>10</v>
       </c>
-      <c r="M24" s="84">
+      <c r="M24" s="83">
         <v>24</v>
       </c>
-      <c r="N24" s="80">
+      <c r="N24" s="79">
         <v>3</v>
       </c>
-      <c r="O24" s="84">
+      <c r="O24" s="83">
         <v>19</v>
       </c>
-      <c r="P24" s="99">
+      <c r="P24" s="98">
         <f>SUM(M24:O24)</f>
         <v>46</v>
       </c>
-      <c r="Q24" s="84">
+      <c r="Q24" s="83">
         <v>20</v>
       </c>
-      <c r="R24" s="19"/>
-      <c r="S24" s="69"/>
-      <c r="T24" s="79">
+      <c r="R24" s="79">
+        <v>2</v>
+      </c>
+      <c r="S24" s="68"/>
+      <c r="T24" s="78">
         <f>SUM(Q24:S24)</f>
-        <v>20</v>
-      </c>
-      <c r="U24" s="69"/>
-      <c r="V24" s="69"/>
+        <v>22</v>
+      </c>
+      <c r="U24" s="68"/>
+      <c r="V24" s="68"/>
       <c r="W24" s="19"/>
-      <c r="X24" s="79">
+      <c r="X24" s="78">
         <f>SUM(U24:W24)</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B25" s="162"/>
-      <c r="C25" s="168" t="s">
+      <c r="B25" s="193"/>
+      <c r="C25" s="198" t="s">
         <v>43</v>
       </c>
-      <c r="D25" s="169" t="s">
+      <c r="D25" s="199" t="s">
         <v>42</v>
       </c>
-      <c r="E25" s="171" t="s">
+      <c r="E25" s="200" t="s">
         <v>35</v>
       </c>
-      <c r="F25" s="172">
+      <c r="F25" s="201">
         <v>120</v>
       </c>
-      <c r="G25" s="173">
+      <c r="G25" s="202">
         <f>SUM(L27,P27,T27,X27)</f>
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="H25" s="121" t="s">
         <v>26</v>
@@ -3841,17 +3900,17 @@
       <c r="X25" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="Y25" s="55" t="s">
+      <c r="Y25" s="54" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="26" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B26" s="162"/>
-      <c r="C26" s="143"/>
-      <c r="D26" s="170"/>
-      <c r="E26" s="171"/>
-      <c r="F26" s="172"/>
-      <c r="G26" s="174"/>
+      <c r="B26" s="193"/>
+      <c r="C26" s="127"/>
+      <c r="D26" s="128"/>
+      <c r="E26" s="200"/>
+      <c r="F26" s="201"/>
+      <c r="G26" s="203"/>
       <c r="H26" s="121" t="s">
         <v>27</v>
       </c>
@@ -3908,77 +3967,81 @@
       </c>
     </row>
     <row r="27" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B27" s="162"/>
-      <c r="C27" s="143"/>
-      <c r="D27" s="170"/>
-      <c r="E27" s="171"/>
-      <c r="F27" s="172"/>
-      <c r="G27" s="174"/>
+      <c r="B27" s="193"/>
+      <c r="C27" s="127"/>
+      <c r="D27" s="128"/>
+      <c r="E27" s="200"/>
+      <c r="F27" s="201"/>
+      <c r="G27" s="203"/>
       <c r="H27" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="I27" s="80">
-        <v>0</v>
-      </c>
-      <c r="J27" s="80">
-        <v>0</v>
-      </c>
-      <c r="K27" s="80">
+      <c r="I27" s="79">
+        <v>0</v>
+      </c>
+      <c r="J27" s="79">
+        <v>0</v>
+      </c>
+      <c r="K27" s="79">
         <v>3</v>
       </c>
-      <c r="L27" s="100">
+      <c r="L27" s="99">
         <f>SUM(I27:K27)</f>
         <v>3</v>
       </c>
-      <c r="M27" s="80">
+      <c r="M27" s="79">
         <v>4</v>
       </c>
-      <c r="N27" s="80">
+      <c r="N27" s="79">
         <v>4</v>
       </c>
-      <c r="O27" s="84">
+      <c r="O27" s="83">
         <v>23</v>
       </c>
-      <c r="P27" s="99">
+      <c r="P27" s="98">
         <f>SUM(M27:O27)</f>
         <v>31</v>
       </c>
-      <c r="Q27" s="80">
+      <c r="Q27" s="79">
         <v>4</v>
       </c>
-      <c r="R27" s="102"/>
-      <c r="S27" s="102"/>
-      <c r="T27" s="57">
+      <c r="R27" s="79">
+        <v>3</v>
+      </c>
+      <c r="S27" s="79">
+        <v>5</v>
+      </c>
+      <c r="T27" s="56">
         <f>SUM(Q27:S27)</f>
-        <v>4</v>
-      </c>
-      <c r="U27" s="102"/>
-      <c r="V27" s="102"/>
-      <c r="W27" s="102"/>
-      <c r="X27" s="57">
+        <v>12</v>
+      </c>
+      <c r="U27" s="101"/>
+      <c r="V27" s="101"/>
+      <c r="W27" s="101"/>
+      <c r="X27" s="56">
         <f>SUM(U27:W27)</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B28" s="162"/>
-      <c r="C28" s="205" t="s">
+      <c r="B28" s="193"/>
+      <c r="C28" s="125" t="s">
         <v>45</v>
       </c>
-      <c r="D28" s="206" t="s">
+      <c r="D28" s="168" t="s">
         <v>42</v>
       </c>
-      <c r="E28" s="207" t="s">
+      <c r="E28" s="170" t="s">
         <v>35</v>
       </c>
-      <c r="F28" s="209">
+      <c r="F28" s="146">
         <v>0.82</v>
       </c>
-      <c r="G28" s="232">
-        <f>O30</f>
-        <v>0.73</v>
-      </c>
-      <c r="H28" s="120" t="s">
+      <c r="G28" s="147">
+        <f>R30</f>
+        <v>0.85</v>
+      </c>
+      <c r="H28" s="123" t="s">
         <v>26</v>
       </c>
       <c r="I28" s="24" t="s">
@@ -4029,18 +4092,18 @@
       <c r="X28" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="Y28" s="55" t="s">
+      <c r="Y28" s="54" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="29" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B29" s="162"/>
-      <c r="C29" s="163"/>
-      <c r="D29" s="189"/>
-      <c r="E29" s="207"/>
-      <c r="F29" s="209"/>
-      <c r="G29" s="232"/>
-      <c r="H29" s="120" t="s">
+      <c r="B29" s="193"/>
+      <c r="C29" s="126"/>
+      <c r="D29" s="169"/>
+      <c r="E29" s="170"/>
+      <c r="F29" s="146"/>
+      <c r="G29" s="147"/>
+      <c r="H29" s="123" t="s">
         <v>27</v>
       </c>
       <c r="I29" s="24">
@@ -4096,73 +4159,75 @@
       </c>
     </row>
     <row r="30" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B30" s="162"/>
-      <c r="C30" s="163"/>
-      <c r="D30" s="189"/>
-      <c r="E30" s="207"/>
-      <c r="F30" s="209"/>
-      <c r="G30" s="232"/>
-      <c r="H30" s="120" t="s">
+      <c r="B30" s="193"/>
+      <c r="C30" s="126"/>
+      <c r="D30" s="169"/>
+      <c r="E30" s="170"/>
+      <c r="F30" s="146"/>
+      <c r="G30" s="147"/>
+      <c r="H30" s="123" t="s">
         <v>28</v>
       </c>
-      <c r="I30" s="78">
+      <c r="I30" s="77">
         <v>0.72</v>
       </c>
-      <c r="J30" s="77">
+      <c r="J30" s="76">
         <v>0.76</v>
       </c>
-      <c r="K30" s="77">
+      <c r="K30" s="76">
         <v>0.8</v>
       </c>
-      <c r="L30" s="88">
+      <c r="L30" s="87">
         <f>AVERAGE(I30:K30)</f>
         <v>0.76000000000000012</v>
       </c>
-      <c r="M30" s="78">
+      <c r="M30" s="77">
         <v>0.75</v>
       </c>
-      <c r="N30" s="77">
+      <c r="N30" s="76">
         <v>0.84</v>
       </c>
-      <c r="O30" s="78">
+      <c r="O30" s="77">
         <v>0.73</v>
       </c>
-      <c r="P30" s="95">
+      <c r="P30" s="94">
         <f>AVERAGE(M30:O30)</f>
         <v>0.77333333333333332</v>
       </c>
-      <c r="Q30" s="77">
+      <c r="Q30" s="76">
         <v>0.82</v>
       </c>
-      <c r="R30" s="19"/>
-      <c r="S30" s="65"/>
-      <c r="T30" s="66">
+      <c r="R30" s="76">
+        <v>0.85</v>
+      </c>
+      <c r="S30" s="64"/>
+      <c r="T30" s="65">
         <f>AVERAGE(Q30:S30)</f>
-        <v>0.82</v>
-      </c>
-      <c r="U30" s="65"/>
-      <c r="V30" s="65"/>
+        <v>0.83499999999999996</v>
+      </c>
+      <c r="U30" s="64"/>
+      <c r="V30" s="64"/>
       <c r="W30" s="19"/>
-      <c r="X30" s="66" t="e">
+      <c r="X30" s="65" t="e">
         <f>AVERAGE(U30:W30)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="31" spans="2:25" ht="19.5" customHeight="1">
-      <c r="B31" s="162"/>
-      <c r="C31" s="143" t="s">
+      <c r="B31" s="193"/>
+      <c r="C31" s="127" t="s">
         <v>47</v>
       </c>
-      <c r="D31" s="170" t="s">
+      <c r="D31" s="128" t="s">
         <v>48</v>
       </c>
-      <c r="E31" s="155">
+      <c r="E31" s="179">
         <v>0.82</v>
       </c>
-      <c r="F31" s="200">
+      <c r="F31" s="143">
         <v>0.7</v>
       </c>
-      <c r="G31" s="155">
+      <c r="G31" s="179">
         <v>0.83</v>
       </c>
       <c r="H31" s="121" t="s">
@@ -4218,12 +4283,12 @@
       </c>
     </row>
     <row r="32" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B32" s="162"/>
-      <c r="C32" s="143"/>
-      <c r="D32" s="170"/>
-      <c r="E32" s="155"/>
-      <c r="F32" s="200"/>
-      <c r="G32" s="155"/>
+      <c r="B32" s="193"/>
+      <c r="C32" s="127"/>
+      <c r="D32" s="128"/>
+      <c r="E32" s="179"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="179"/>
       <c r="H32" s="121" t="s">
         <v>27</v>
       </c>
@@ -4280,12 +4345,12 @@
       </c>
     </row>
     <row r="33" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B33" s="162"/>
-      <c r="C33" s="143"/>
-      <c r="D33" s="170"/>
-      <c r="E33" s="155"/>
-      <c r="F33" s="200"/>
-      <c r="G33" s="155"/>
+      <c r="B33" s="193"/>
+      <c r="C33" s="127"/>
+      <c r="D33" s="128"/>
+      <c r="E33" s="179"/>
+      <c r="F33" s="143"/>
+      <c r="G33" s="179"/>
       <c r="H33" s="121" t="s">
         <v>28</v>
       </c>
@@ -4295,10 +4360,10 @@
       <c r="J33" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="K33" s="77">
+      <c r="K33" s="76">
         <v>0.83</v>
       </c>
-      <c r="L33" s="88">
+      <c r="L33" s="87">
         <v>0.83</v>
       </c>
       <c r="M33" s="15" t="s">
@@ -4307,43 +4372,45 @@
       <c r="N33" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="O33" s="77">
+      <c r="O33" s="76">
         <v>0.81</v>
       </c>
-      <c r="P33" s="88">
+      <c r="P33" s="87">
         <v>0.81</v>
       </c>
       <c r="Q33" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="R33" s="15"/>
+      <c r="R33" s="15" t="s">
+        <v>50</v>
+      </c>
       <c r="S33" s="49"/>
-      <c r="T33" s="63"/>
+      <c r="T33" s="62"/>
       <c r="U33" s="49"/>
       <c r="V33" s="49"/>
       <c r="W33" s="15"/>
       <c r="X33" s="33"/>
     </row>
     <row r="34" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B34" s="147" t="s">
+      <c r="B34" s="185" t="s">
         <v>51</v>
       </c>
-      <c r="C34" s="163" t="s">
+      <c r="C34" s="126" t="s">
         <v>52</v>
       </c>
-      <c r="D34" s="153" t="s">
+      <c r="D34" s="148" t="s">
         <v>53</v>
       </c>
-      <c r="E34" s="198">
+      <c r="E34" s="152">
         <v>0.77</v>
       </c>
-      <c r="F34" s="209">
+      <c r="F34" s="146">
         <v>0.85</v>
       </c>
-      <c r="G34" s="196">
+      <c r="G34" s="156">
         <v>0.79</v>
       </c>
-      <c r="H34" s="120" t="s">
+      <c r="H34" s="123" t="s">
         <v>26</v>
       </c>
       <c r="I34" s="21">
@@ -4396,13 +4463,13 @@
       </c>
     </row>
     <row r="35" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B35" s="148"/>
-      <c r="C35" s="163"/>
-      <c r="D35" s="153"/>
-      <c r="E35" s="198"/>
-      <c r="F35" s="209"/>
-      <c r="G35" s="196"/>
-      <c r="H35" s="120" t="s">
+      <c r="B35" s="186"/>
+      <c r="C35" s="126"/>
+      <c r="D35" s="148"/>
+      <c r="E35" s="152"/>
+      <c r="F35" s="146"/>
+      <c r="G35" s="156"/>
+      <c r="H35" s="123" t="s">
         <v>27</v>
       </c>
       <c r="I35" s="21">
@@ -4455,129 +4522,131 @@
       </c>
     </row>
     <row r="36" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B36" s="148"/>
-      <c r="C36" s="164"/>
-      <c r="D36" s="159"/>
-      <c r="E36" s="199"/>
-      <c r="F36" s="209"/>
-      <c r="G36" s="197"/>
-      <c r="H36" s="120" t="s">
+      <c r="B36" s="186"/>
+      <c r="C36" s="194"/>
+      <c r="D36" s="190"/>
+      <c r="E36" s="153"/>
+      <c r="F36" s="146"/>
+      <c r="G36" s="184"/>
+      <c r="H36" s="123" t="s">
         <v>28</v>
       </c>
-      <c r="I36" s="77">
+      <c r="I36" s="76">
         <v>0.78</v>
       </c>
-      <c r="J36" s="83">
+      <c r="J36" s="82">
         <v>0.77</v>
       </c>
-      <c r="K36" s="77">
+      <c r="K36" s="76">
         <v>0.79</v>
       </c>
-      <c r="L36" s="88">
+      <c r="L36" s="87">
         <v>0.79</v>
       </c>
-      <c r="M36" s="77">
+      <c r="M36" s="76">
         <v>0.8</v>
       </c>
-      <c r="N36" s="78">
+      <c r="N36" s="77">
         <v>0.8</v>
       </c>
-      <c r="O36" s="83">
+      <c r="O36" s="82">
         <v>0.79600000000000004</v>
       </c>
-      <c r="P36" s="95">
+      <c r="P36" s="94">
         <v>0.8</v>
       </c>
-      <c r="Q36" s="78">
+      <c r="Q36" s="77">
         <v>0.79</v>
       </c>
-      <c r="R36" s="50"/>
+      <c r="R36" s="82">
+        <v>0.8</v>
+      </c>
       <c r="S36" s="50"/>
-      <c r="T36" s="67"/>
+      <c r="T36" s="66"/>
       <c r="U36" s="50"/>
       <c r="V36" s="50"/>
       <c r="W36" s="50"/>
-      <c r="X36" s="67"/>
+      <c r="X36" s="66"/>
     </row>
     <row r="37" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B37" s="148"/>
-      <c r="C37" s="223" t="s">
+      <c r="B37" s="186"/>
+      <c r="C37" s="136" t="s">
         <v>54</v>
       </c>
-      <c r="D37" s="226" t="s">
+      <c r="D37" s="139" t="s">
         <v>55</v>
       </c>
-      <c r="E37" s="213" t="s">
+      <c r="E37" s="159" t="s">
         <v>35</v>
       </c>
-      <c r="F37" s="214">
-        <v>0.9</v>
-      </c>
-      <c r="G37" s="217">
+      <c r="F37" s="160">
+        <v>0.9</v>
+      </c>
+      <c r="G37" s="163">
         <v>0.6</v>
       </c>
       <c r="H37" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="I37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="J37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="K37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="L37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="M37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="N37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="O37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="P37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="R37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="S37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="T37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="U37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="V37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="W37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="X37" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="Y37" s="55" t="s">
+      <c r="I37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="J37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="K37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="L37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="M37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="N37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="O37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="P37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="R37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="S37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="T37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="U37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="V37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="W37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="X37" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y37" s="54" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="38" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B38" s="148"/>
-      <c r="C38" s="224"/>
-      <c r="D38" s="227"/>
-      <c r="E38" s="213"/>
-      <c r="F38" s="214"/>
-      <c r="G38" s="217"/>
+      <c r="B38" s="186"/>
+      <c r="C38" s="137"/>
+      <c r="D38" s="140"/>
+      <c r="E38" s="159"/>
+      <c r="F38" s="160"/>
+      <c r="G38" s="163"/>
       <c r="H38" s="39" t="s">
         <v>27</v>
       </c>
@@ -4631,130 +4700,132 @@
       </c>
     </row>
     <row r="39" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B39" s="148"/>
-      <c r="C39" s="225"/>
-      <c r="D39" s="227"/>
-      <c r="E39" s="213"/>
-      <c r="F39" s="215"/>
-      <c r="G39" s="217"/>
+      <c r="B39" s="186"/>
+      <c r="C39" s="138"/>
+      <c r="D39" s="140"/>
+      <c r="E39" s="159"/>
+      <c r="F39" s="161"/>
+      <c r="G39" s="163"/>
       <c r="H39" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="I39" s="78">
+      <c r="I39" s="77">
         <v>0.44</v>
       </c>
-      <c r="J39" s="78">
+      <c r="J39" s="77">
         <v>0.44</v>
       </c>
-      <c r="K39" s="77">
+      <c r="K39" s="76">
         <v>0.91</v>
       </c>
-      <c r="L39" s="95">
+      <c r="L39" s="94">
         <v>0.6</v>
       </c>
-      <c r="M39" s="78">
-        <v>0</v>
-      </c>
-      <c r="N39" s="78">
+      <c r="M39" s="77">
+        <v>0</v>
+      </c>
+      <c r="N39" s="77">
         <v>0.6</v>
       </c>
-      <c r="O39" s="78">
+      <c r="O39" s="77">
         <v>0.55000000000000004</v>
       </c>
-      <c r="P39" s="95">
+      <c r="P39" s="94">
         <v>0.4</v>
       </c>
-      <c r="Q39" s="78">
+      <c r="Q39" s="77">
         <v>0.2</v>
       </c>
-      <c r="R39" s="60"/>
-      <c r="S39" s="60"/>
-      <c r="T39" s="60"/>
-      <c r="U39" s="60"/>
-      <c r="V39" s="60"/>
-      <c r="W39" s="60"/>
+      <c r="R39" s="82">
+        <v>0.7</v>
+      </c>
+      <c r="S39" s="59"/>
+      <c r="T39" s="59"/>
+      <c r="U39" s="59"/>
+      <c r="V39" s="59"/>
+      <c r="W39" s="59"/>
       <c r="X39" s="18"/>
     </row>
     <row r="40" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B40" s="148"/>
-      <c r="C40" s="175" t="s">
+      <c r="B40" s="186"/>
+      <c r="C40" s="204" t="s">
         <v>56</v>
       </c>
-      <c r="D40" s="178" t="s">
+      <c r="D40" s="207" t="s">
         <v>55</v>
       </c>
-      <c r="E40" s="179" t="s">
+      <c r="E40" s="208" t="s">
         <v>35</v>
       </c>
-      <c r="F40" s="209">
-        <v>0.9</v>
-      </c>
-      <c r="G40" s="211">
+      <c r="F40" s="146">
+        <v>0.9</v>
+      </c>
+      <c r="G40" s="157">
         <v>0.85</v>
       </c>
-      <c r="H40" s="59" t="s">
+      <c r="H40" s="58" t="s">
         <v>26</v>
       </c>
-      <c r="I40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="J40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="K40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="L40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="M40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="N40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="O40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="P40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="R40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="S40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="T40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="U40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="V40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="W40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="X40" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="Y40" s="55" t="s">
+      <c r="I40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="J40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="K40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="L40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="M40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="N40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="O40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="P40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="R40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="S40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="T40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="U40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="V40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="W40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="X40" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y40" s="54" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="41" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B41" s="148"/>
-      <c r="C41" s="176"/>
-      <c r="D41" s="153"/>
-      <c r="E41" s="179"/>
-      <c r="F41" s="209"/>
-      <c r="G41" s="212"/>
-      <c r="H41" s="59" t="s">
+      <c r="B41" s="186"/>
+      <c r="C41" s="205"/>
+      <c r="D41" s="148"/>
+      <c r="E41" s="208"/>
+      <c r="F41" s="146"/>
+      <c r="G41" s="158"/>
+      <c r="H41" s="58" t="s">
         <v>27</v>
       </c>
       <c r="I41" s="21">
@@ -4807,43 +4878,45 @@
       </c>
     </row>
     <row r="42" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B42" s="148"/>
-      <c r="C42" s="177"/>
-      <c r="D42" s="153"/>
-      <c r="E42" s="179"/>
-      <c r="F42" s="209"/>
-      <c r="G42" s="212"/>
-      <c r="H42" s="59" t="s">
+      <c r="B42" s="186"/>
+      <c r="C42" s="206"/>
+      <c r="D42" s="148"/>
+      <c r="E42" s="208"/>
+      <c r="F42" s="146"/>
+      <c r="G42" s="158"/>
+      <c r="H42" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="I42" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="J42" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="K42" s="83">
+      <c r="I42" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="J42" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="K42" s="82">
         <v>0.85</v>
       </c>
-      <c r="L42" s="101">
+      <c r="L42" s="100">
         <v>0.85</v>
       </c>
-      <c r="M42" s="77">
+      <c r="M42" s="76">
         <v>1</v>
       </c>
-      <c r="N42" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="O42" s="83">
+      <c r="N42" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="O42" s="82">
         <v>0.15</v>
       </c>
-      <c r="P42" s="101">
+      <c r="P42" s="100">
         <v>0.57999999999999996</v>
       </c>
-      <c r="Q42" s="83">
+      <c r="Q42" s="82">
         <v>0.7</v>
       </c>
-      <c r="R42" s="51"/>
+      <c r="R42" s="76">
+        <v>1</v>
+      </c>
       <c r="S42" s="51"/>
       <c r="T42" s="51"/>
       <c r="U42" s="51"/>
@@ -4852,84 +4925,84 @@
       <c r="X42" s="13"/>
     </row>
     <row r="43" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B43" s="148"/>
-      <c r="C43" s="230" t="s">
+      <c r="B43" s="186"/>
+      <c r="C43" s="144" t="s">
         <v>57</v>
       </c>
-      <c r="D43" s="226" t="s">
+      <c r="D43" s="139" t="s">
         <v>55</v>
       </c>
-      <c r="E43" s="213" t="s">
+      <c r="E43" s="159" t="s">
         <v>35</v>
       </c>
-      <c r="F43" s="214">
+      <c r="F43" s="160">
         <v>1</v>
       </c>
-      <c r="G43" s="216">
+      <c r="G43" s="162">
         <v>0.93</v>
       </c>
       <c r="H43" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="I43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="J43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="K43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="L43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="M43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="N43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="O43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="P43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="R43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="S43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="T43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="U43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="V43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="W43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="X43" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="Y43" s="55" t="s">
+      <c r="I43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="J43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="K43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="L43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="M43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="N43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="O43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="P43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="R43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="S43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="T43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="U43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="V43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="W43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="X43" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y43" s="54" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="44" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B44" s="148"/>
-      <c r="C44" s="231"/>
-      <c r="D44" s="227"/>
-      <c r="E44" s="213"/>
-      <c r="F44" s="214"/>
-      <c r="G44" s="216"/>
+      <c r="B44" s="186"/>
+      <c r="C44" s="145"/>
+      <c r="D44" s="140"/>
+      <c r="E44" s="159"/>
+      <c r="F44" s="160"/>
+      <c r="G44" s="162"/>
       <c r="H44" s="39" t="s">
         <v>27</v>
       </c>
@@ -4986,175 +5059,177 @@
       </c>
     </row>
     <row r="45" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B45" s="148"/>
-      <c r="C45" s="231"/>
-      <c r="D45" s="227"/>
-      <c r="E45" s="213"/>
-      <c r="F45" s="215"/>
-      <c r="G45" s="216"/>
+      <c r="B45" s="186"/>
+      <c r="C45" s="145"/>
+      <c r="D45" s="140"/>
+      <c r="E45" s="159"/>
+      <c r="F45" s="161"/>
+      <c r="G45" s="162"/>
       <c r="H45" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="I45" s="81" t="s">
-        <v>32</v>
-      </c>
-      <c r="J45" s="81" t="s">
-        <v>32</v>
-      </c>
-      <c r="K45" s="83">
+      <c r="I45" s="80" t="s">
+        <v>32</v>
+      </c>
+      <c r="J45" s="80" t="s">
+        <v>32</v>
+      </c>
+      <c r="K45" s="82">
         <v>0.93</v>
       </c>
-      <c r="L45" s="101">
+      <c r="L45" s="100">
         <v>0.93</v>
       </c>
-      <c r="M45" s="77">
+      <c r="M45" s="76">
         <v>1</v>
       </c>
-      <c r="N45" s="81" t="s">
-        <v>32</v>
-      </c>
-      <c r="O45" s="83">
+      <c r="N45" s="80" t="s">
+        <v>32</v>
+      </c>
+      <c r="O45" s="82">
         <v>0.98</v>
       </c>
-      <c r="P45" s="101">
+      <c r="P45" s="100">
         <v>0.99</v>
       </c>
-      <c r="Q45" s="83">
+      <c r="Q45" s="82">
         <v>0.95</v>
       </c>
-      <c r="R45" s="60"/>
-      <c r="S45" s="60"/>
-      <c r="T45" s="60"/>
-      <c r="U45" s="60"/>
-      <c r="V45" s="60"/>
-      <c r="W45" s="60"/>
+      <c r="R45" s="76">
+        <v>1</v>
+      </c>
+      <c r="S45" s="59"/>
+      <c r="T45" s="59"/>
+      <c r="U45" s="59"/>
+      <c r="V45" s="59"/>
+      <c r="W45" s="59"/>
       <c r="X45" s="18"/>
     </row>
     <row r="46" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B46" s="148"/>
-      <c r="C46" s="163" t="s">
+      <c r="B46" s="186"/>
+      <c r="C46" s="126" t="s">
         <v>59</v>
       </c>
-      <c r="D46" s="153" t="s">
+      <c r="D46" s="148" t="s">
         <v>55</v>
       </c>
-      <c r="E46" s="233">
+      <c r="E46" s="149">
         <v>372</v>
       </c>
-      <c r="F46" s="234">
+      <c r="F46" s="150">
         <v>366</v>
       </c>
-      <c r="G46" s="201">
+      <c r="G46" s="135">
         <v>365</v>
       </c>
-      <c r="H46" s="120" t="s">
+      <c r="H46" s="123" t="s">
         <v>26</v>
       </c>
-      <c r="I46" s="106">
+      <c r="I46" s="105">
         <v>383</v>
       </c>
-      <c r="J46" s="106">
+      <c r="J46" s="105">
         <v>381</v>
       </c>
-      <c r="K46" s="106">
+      <c r="K46" s="105">
         <v>380</v>
       </c>
-      <c r="L46" s="107">
+      <c r="L46" s="106">
         <v>381</v>
       </c>
-      <c r="M46" s="106">
+      <c r="M46" s="105">
         <v>378</v>
       </c>
-      <c r="N46" s="106">
+      <c r="N46" s="105">
         <v>376</v>
       </c>
-      <c r="O46" s="106">
+      <c r="O46" s="105">
         <v>374</v>
       </c>
-      <c r="P46" s="107">
+      <c r="P46" s="106">
         <v>376</v>
       </c>
-      <c r="Q46" s="106">
+      <c r="Q46" s="105">
         <v>372</v>
       </c>
-      <c r="R46" s="106">
+      <c r="R46" s="105">
         <v>370</v>
       </c>
-      <c r="S46" s="106">
+      <c r="S46" s="105">
         <v>371</v>
       </c>
-      <c r="T46" s="107">
+      <c r="T46" s="106">
         <v>371</v>
       </c>
-      <c r="U46" s="106">
+      <c r="U46" s="105">
         <v>372</v>
       </c>
-      <c r="V46" s="106">
+      <c r="V46" s="105">
         <v>371</v>
       </c>
-      <c r="W46" s="106">
+      <c r="W46" s="105">
         <v>371</v>
       </c>
-      <c r="X46" s="107">
+      <c r="X46" s="106">
         <v>371</v>
       </c>
     </row>
     <row r="47" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B47" s="148"/>
-      <c r="C47" s="163"/>
-      <c r="D47" s="153"/>
-      <c r="E47" s="233"/>
-      <c r="F47" s="234"/>
-      <c r="G47" s="201"/>
-      <c r="H47" s="120" t="s">
+      <c r="B47" s="186"/>
+      <c r="C47" s="126"/>
+      <c r="D47" s="148"/>
+      <c r="E47" s="149"/>
+      <c r="F47" s="150"/>
+      <c r="G47" s="135"/>
+      <c r="H47" s="123" t="s">
         <v>27</v>
       </c>
-      <c r="I47" s="106">
+      <c r="I47" s="105">
         <v>366</v>
       </c>
-      <c r="J47" s="106">
+      <c r="J47" s="105">
         <v>366</v>
       </c>
-      <c r="K47" s="106">
+      <c r="K47" s="105">
         <v>366</v>
       </c>
-      <c r="L47" s="107">
+      <c r="L47" s="106">
         <v>366</v>
       </c>
-      <c r="M47" s="106">
+      <c r="M47" s="105">
         <v>366</v>
       </c>
-      <c r="N47" s="106">
+      <c r="N47" s="105">
         <v>366</v>
       </c>
-      <c r="O47" s="106">
+      <c r="O47" s="105">
         <v>366</v>
       </c>
-      <c r="P47" s="107">
+      <c r="P47" s="106">
         <v>366</v>
       </c>
-      <c r="Q47" s="106">
+      <c r="Q47" s="105">
         <v>366</v>
       </c>
-      <c r="R47" s="106">
+      <c r="R47" s="105">
         <v>366</v>
       </c>
-      <c r="S47" s="106">
+      <c r="S47" s="105">
         <v>366</v>
       </c>
-      <c r="T47" s="107">
+      <c r="T47" s="106">
         <v>366</v>
       </c>
-      <c r="U47" s="106">
+      <c r="U47" s="105">
         <v>366</v>
       </c>
-      <c r="V47" s="106">
+      <c r="V47" s="105">
         <v>366</v>
       </c>
-      <c r="W47" s="106">
+      <c r="W47" s="105">
         <v>366</v>
       </c>
-      <c r="X47" s="107">
+      <c r="X47" s="106">
         <v>366</v>
       </c>
       <c r="Y47" s="7" t="s">
@@ -5162,65 +5237,67 @@
       </c>
     </row>
     <row r="48" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B48" s="148"/>
-      <c r="C48" s="163"/>
-      <c r="D48" s="153"/>
-      <c r="E48" s="233"/>
-      <c r="F48" s="234"/>
-      <c r="G48" s="201"/>
-      <c r="H48" s="120" t="s">
+      <c r="B48" s="186"/>
+      <c r="C48" s="126"/>
+      <c r="D48" s="148"/>
+      <c r="E48" s="149"/>
+      <c r="F48" s="150"/>
+      <c r="G48" s="135"/>
+      <c r="H48" s="123" t="s">
         <v>28</v>
       </c>
-      <c r="I48" s="76">
+      <c r="I48" s="75">
         <v>379</v>
       </c>
-      <c r="J48" s="76">
+      <c r="J48" s="75">
         <v>373</v>
       </c>
-      <c r="K48" s="76">
+      <c r="K48" s="75">
         <v>380</v>
       </c>
-      <c r="L48" s="96">
+      <c r="L48" s="95">
         <v>377</v>
       </c>
-      <c r="M48" s="76">
+      <c r="M48" s="75">
         <v>377</v>
       </c>
-      <c r="N48" s="87">
+      <c r="N48" s="86">
         <v>365</v>
       </c>
-      <c r="O48" s="87">
+      <c r="O48" s="86">
         <v>365</v>
       </c>
-      <c r="P48" s="96">
+      <c r="P48" s="95">
         <v>369</v>
       </c>
-      <c r="Q48" s="87">
+      <c r="Q48" s="86">
         <v>363</v>
       </c>
-      <c r="R48" s="106"/>
-      <c r="S48" s="106"/>
-      <c r="T48" s="107"/>
-      <c r="U48" s="106"/>
-      <c r="V48" s="106"/>
-      <c r="W48" s="106"/>
-      <c r="X48" s="107"/>
+      <c r="R48" s="86">
+        <v>360</v>
+      </c>
+      <c r="S48" s="105"/>
+      <c r="T48" s="106"/>
+      <c r="U48" s="105"/>
+      <c r="V48" s="105"/>
+      <c r="W48" s="105"/>
+      <c r="X48" s="106"/>
     </row>
     <row r="49" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B49" s="148"/>
-      <c r="C49" s="184" t="s">
+      <c r="B49" s="186"/>
+      <c r="C49" s="174" t="s">
         <v>61</v>
       </c>
-      <c r="D49" s="185" t="s">
+      <c r="D49" s="175" t="s">
         <v>48</v>
       </c>
-      <c r="E49" s="186">
+      <c r="E49" s="177">
         <v>0.71</v>
       </c>
-      <c r="F49" s="166">
+      <c r="F49" s="196">
         <v>0.92</v>
       </c>
-      <c r="G49" s="220">
+      <c r="G49" s="131">
         <v>0.72</v>
       </c>
       <c r="H49" s="121" t="s">
@@ -5276,12 +5353,12 @@
       </c>
     </row>
     <row r="50" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B50" s="148"/>
-      <c r="C50" s="143"/>
-      <c r="D50" s="144"/>
-      <c r="E50" s="186"/>
-      <c r="F50" s="166"/>
-      <c r="G50" s="221"/>
+      <c r="B50" s="186"/>
+      <c r="C50" s="127"/>
+      <c r="D50" s="176"/>
+      <c r="E50" s="177"/>
+      <c r="F50" s="196"/>
+      <c r="G50" s="132"/>
       <c r="H50" s="121" t="s">
         <v>27</v>
       </c>
@@ -5335,43 +5412,45 @@
       </c>
     </row>
     <row r="51" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B51" s="148"/>
-      <c r="C51" s="143"/>
-      <c r="D51" s="144"/>
-      <c r="E51" s="186"/>
-      <c r="F51" s="166"/>
-      <c r="G51" s="221"/>
+      <c r="B51" s="186"/>
+      <c r="C51" s="127"/>
+      <c r="D51" s="176"/>
+      <c r="E51" s="177"/>
+      <c r="F51" s="196"/>
+      <c r="G51" s="132"/>
       <c r="H51" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="I51" s="78">
+      <c r="I51" s="77">
         <v>0.83</v>
       </c>
-      <c r="J51" s="78">
+      <c r="J51" s="77">
         <v>0.6</v>
       </c>
-      <c r="K51" s="78" t="s">
+      <c r="K51" s="77" t="s">
         <v>62</v>
       </c>
-      <c r="L51" s="95">
+      <c r="L51" s="94">
         <v>0.72</v>
       </c>
-      <c r="M51" s="78">
+      <c r="M51" s="77">
         <v>0.85</v>
       </c>
-      <c r="N51" s="78">
+      <c r="N51" s="77">
         <v>0.89</v>
       </c>
-      <c r="O51" s="78">
+      <c r="O51" s="77">
         <v>0.91</v>
       </c>
-      <c r="P51" s="95">
+      <c r="P51" s="94">
         <v>0.82</v>
       </c>
-      <c r="Q51" s="78">
+      <c r="Q51" s="77">
         <v>0.89</v>
       </c>
-      <c r="R51" s="49"/>
+      <c r="R51" s="77">
+        <v>0.89</v>
+      </c>
       <c r="S51" s="49"/>
       <c r="T51" s="48"/>
       <c r="U51" s="47"/>
@@ -5380,23 +5459,23 @@
       <c r="X51" s="27"/>
     </row>
     <row r="52" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B52" s="148"/>
-      <c r="C52" s="163" t="s">
+      <c r="B52" s="186"/>
+      <c r="C52" s="126" t="s">
         <v>63</v>
       </c>
-      <c r="D52" s="153" t="s">
+      <c r="D52" s="148" t="s">
         <v>48</v>
       </c>
-      <c r="E52" s="167" t="s">
+      <c r="E52" s="197" t="s">
         <v>35</v>
       </c>
-      <c r="F52" s="210" t="s">
+      <c r="F52" s="154" t="s">
         <v>64</v>
       </c>
-      <c r="G52" s="196">
+      <c r="G52" s="156">
         <v>0.28999999999999998</v>
       </c>
-      <c r="H52" s="120" t="s">
+      <c r="H52" s="123" t="s">
         <v>26</v>
       </c>
       <c r="I52" s="24" t="s">
@@ -5447,42 +5526,42 @@
       <c r="X52" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="Y52" s="55" t="s">
+      <c r="Y52" s="54" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="53" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B53" s="148"/>
-      <c r="C53" s="163"/>
-      <c r="D53" s="153"/>
-      <c r="E53" s="167"/>
-      <c r="F53" s="193"/>
-      <c r="G53" s="196"/>
-      <c r="H53" s="120" t="s">
+      <c r="B53" s="186"/>
+      <c r="C53" s="126"/>
+      <c r="D53" s="148"/>
+      <c r="E53" s="197"/>
+      <c r="F53" s="155"/>
+      <c r="G53" s="156"/>
+      <c r="H53" s="123" t="s">
         <v>27</v>
       </c>
-      <c r="I53" s="130"/>
-      <c r="J53" s="130"/>
-      <c r="K53" s="130"/>
-      <c r="L53" s="108" t="s">
+      <c r="I53" s="133"/>
+      <c r="J53" s="133"/>
+      <c r="K53" s="133"/>
+      <c r="L53" s="107" t="s">
         <v>64</v>
       </c>
-      <c r="M53" s="130"/>
-      <c r="N53" s="130"/>
-      <c r="O53" s="130"/>
-      <c r="P53" s="108" t="s">
+      <c r="M53" s="133"/>
+      <c r="N53" s="133"/>
+      <c r="O53" s="133"/>
+      <c r="P53" s="107" t="s">
         <v>64</v>
       </c>
-      <c r="Q53" s="130"/>
-      <c r="R53" s="130"/>
-      <c r="S53" s="130"/>
-      <c r="T53" s="108" t="s">
+      <c r="Q53" s="133"/>
+      <c r="R53" s="133"/>
+      <c r="S53" s="133"/>
+      <c r="T53" s="107" t="s">
         <v>64</v>
       </c>
-      <c r="U53" s="130"/>
-      <c r="V53" s="130"/>
-      <c r="W53" s="130"/>
-      <c r="X53" s="108" t="s">
+      <c r="U53" s="133"/>
+      <c r="V53" s="133"/>
+      <c r="W53" s="133"/>
+      <c r="X53" s="107" t="s">
         <v>64</v>
       </c>
       <c r="Y53" s="7" t="s">
@@ -5490,13 +5569,13 @@
       </c>
     </row>
     <row r="54" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B54" s="148"/>
-      <c r="C54" s="163"/>
-      <c r="D54" s="153"/>
-      <c r="E54" s="167"/>
-      <c r="F54" s="193"/>
-      <c r="G54" s="196"/>
-      <c r="H54" s="120" t="s">
+      <c r="B54" s="186"/>
+      <c r="C54" s="126"/>
+      <c r="D54" s="148"/>
+      <c r="E54" s="197"/>
+      <c r="F54" s="155"/>
+      <c r="G54" s="156"/>
+      <c r="H54" s="123" t="s">
         <v>28</v>
       </c>
       <c r="I54" s="24" t="s">
@@ -5508,7 +5587,7 @@
       <c r="K54" s="24">
         <v>0.28799999999999998</v>
       </c>
-      <c r="L54" s="95">
+      <c r="L54" s="94">
         <v>0.28999999999999998</v>
       </c>
       <c r="M54" s="24">
@@ -5520,13 +5599,15 @@
       <c r="O54" s="24">
         <v>0.13</v>
       </c>
-      <c r="P54" s="95">
+      <c r="P54" s="94">
         <v>0.16</v>
       </c>
       <c r="Q54" s="24">
         <v>0.214</v>
       </c>
-      <c r="R54" s="24"/>
+      <c r="R54" s="24">
+        <v>0.214</v>
+      </c>
       <c r="S54" s="24"/>
       <c r="T54" s="25"/>
       <c r="U54" s="24"/>
@@ -5535,23 +5616,23 @@
       <c r="X54" s="25"/>
     </row>
     <row r="55" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B55" s="148"/>
-      <c r="C55" s="143" t="s">
+      <c r="B55" s="186"/>
+      <c r="C55" s="127" t="s">
         <v>68</v>
       </c>
-      <c r="D55" s="144" t="s">
+      <c r="D55" s="176" t="s">
         <v>69</v>
       </c>
-      <c r="E55" s="145">
+      <c r="E55" s="212">
         <f>X55</f>
         <v>40</v>
       </c>
-      <c r="F55" s="165">
+      <c r="F55" s="195">
         <v>55</v>
       </c>
-      <c r="G55" s="222">
+      <c r="G55" s="134">
         <f>X57</f>
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H55" s="121" t="s">
         <v>26</v>
@@ -5606,119 +5687,121 @@
       </c>
     </row>
     <row r="56" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B56" s="148"/>
-      <c r="C56" s="143"/>
-      <c r="D56" s="144"/>
-      <c r="E56" s="145"/>
-      <c r="F56" s="165"/>
-      <c r="G56" s="222"/>
+      <c r="B56" s="186"/>
+      <c r="C56" s="127"/>
+      <c r="D56" s="176"/>
+      <c r="E56" s="212"/>
+      <c r="F56" s="195"/>
+      <c r="G56" s="134"/>
       <c r="H56" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I56" s="208" t="s">
-        <v>32</v>
-      </c>
-      <c r="J56" s="208"/>
-      <c r="K56" s="208"/>
+      <c r="I56" s="151" t="s">
+        <v>32</v>
+      </c>
+      <c r="J56" s="151"/>
+      <c r="K56" s="151"/>
       <c r="L56" s="18">
         <v>13</v>
       </c>
-      <c r="M56" s="208" t="s">
-        <v>32</v>
-      </c>
-      <c r="N56" s="208"/>
-      <c r="O56" s="208"/>
+      <c r="M56" s="151" t="s">
+        <v>32</v>
+      </c>
+      <c r="N56" s="151"/>
+      <c r="O56" s="151"/>
       <c r="P56" s="18">
         <v>27</v>
       </c>
-      <c r="Q56" s="208" t="s">
-        <v>32</v>
-      </c>
-      <c r="R56" s="208"/>
-      <c r="S56" s="208"/>
+      <c r="Q56" s="151" t="s">
+        <v>32</v>
+      </c>
+      <c r="R56" s="151"/>
+      <c r="S56" s="151"/>
       <c r="T56" s="18">
         <v>41</v>
       </c>
-      <c r="U56" s="208" t="s">
-        <v>32</v>
-      </c>
-      <c r="V56" s="208"/>
-      <c r="W56" s="208"/>
+      <c r="U56" s="151" t="s">
+        <v>32</v>
+      </c>
+      <c r="V56" s="151"/>
+      <c r="W56" s="151"/>
       <c r="X56" s="18">
         <v>55</v>
       </c>
     </row>
     <row r="57" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B57" s="148"/>
-      <c r="C57" s="143"/>
-      <c r="D57" s="144"/>
-      <c r="E57" s="145"/>
-      <c r="F57" s="165"/>
-      <c r="G57" s="222"/>
+      <c r="B57" s="186"/>
+      <c r="C57" s="127"/>
+      <c r="D57" s="176"/>
+      <c r="E57" s="212"/>
+      <c r="F57" s="195"/>
+      <c r="G57" s="134"/>
       <c r="H57" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="I57" s="109">
-        <v>0</v>
-      </c>
-      <c r="J57" s="109">
-        <v>0</v>
-      </c>
-      <c r="K57" s="109">
+      <c r="I57" s="108">
+        <v>0</v>
+      </c>
+      <c r="J57" s="108">
+        <v>0</v>
+      </c>
+      <c r="K57" s="108">
         <v>17</v>
       </c>
-      <c r="L57" s="90">
+      <c r="L57" s="89">
         <v>17</v>
       </c>
-      <c r="M57" s="109">
+      <c r="M57" s="108">
         <v>25</v>
       </c>
-      <c r="N57" s="109">
-        <v>0</v>
-      </c>
-      <c r="O57" s="109">
-        <v>0</v>
-      </c>
-      <c r="P57" s="114">
+      <c r="N57" s="108">
+        <v>0</v>
+      </c>
+      <c r="O57" s="108">
+        <v>0</v>
+      </c>
+      <c r="P57" s="113">
         <v>42</v>
       </c>
-      <c r="Q57" s="109">
+      <c r="Q57" s="108">
         <v>2</v>
       </c>
-      <c r="R57" s="109"/>
-      <c r="S57" s="109"/>
-      <c r="T57" s="110">
+      <c r="R57" s="108">
+        <v>3</v>
+      </c>
+      <c r="S57" s="108"/>
+      <c r="T57" s="109">
         <f>SUM(P57:S57)</f>
-        <v>44</v>
-      </c>
-      <c r="U57" s="109"/>
-      <c r="V57" s="109"/>
-      <c r="W57" s="109"/>
-      <c r="X57" s="110">
+        <v>47</v>
+      </c>
+      <c r="U57" s="108"/>
+      <c r="V57" s="108"/>
+      <c r="W57" s="108"/>
+      <c r="X57" s="109">
         <f>SUM(T57:W57)</f>
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="58" spans="2:25" ht="15" hidden="1" customHeight="1">
-      <c r="B58" s="147" t="s">
+      <c r="B58" s="185" t="s">
         <v>70</v>
       </c>
-      <c r="C58" s="156" t="s">
+      <c r="C58" s="187" t="s">
         <v>71</v>
       </c>
-      <c r="D58" s="159" t="s">
+      <c r="D58" s="190" t="s">
         <v>72</v>
       </c>
-      <c r="E58" s="135">
+      <c r="E58" s="219">
         <v>92.5</v>
       </c>
-      <c r="F58" s="132">
+      <c r="F58" s="228">
         <v>93</v>
       </c>
-      <c r="G58" s="135">
+      <c r="G58" s="219">
         <v>92.5</v>
       </c>
-      <c r="H58" s="120" t="s">
+      <c r="H58" s="123" t="s">
         <v>26</v>
       </c>
       <c r="I58" s="34">
@@ -5774,13 +5857,13 @@
       </c>
     </row>
     <row r="59" spans="2:25" ht="15" hidden="1" customHeight="1">
-      <c r="B59" s="148"/>
-      <c r="C59" s="157"/>
-      <c r="D59" s="160"/>
-      <c r="E59" s="136"/>
-      <c r="F59" s="133"/>
-      <c r="G59" s="136"/>
-      <c r="H59" s="120" t="s">
+      <c r="B59" s="186"/>
+      <c r="C59" s="188"/>
+      <c r="D59" s="191"/>
+      <c r="E59" s="220"/>
+      <c r="F59" s="229"/>
+      <c r="G59" s="220"/>
+      <c r="H59" s="123" t="s">
         <v>27</v>
       </c>
       <c r="I59" s="19">
@@ -5836,13 +5919,13 @@
       </c>
     </row>
     <row r="60" spans="2:25" ht="15" hidden="1" customHeight="1">
-      <c r="B60" s="148"/>
-      <c r="C60" s="158"/>
-      <c r="D60" s="161"/>
-      <c r="E60" s="137"/>
-      <c r="F60" s="134"/>
-      <c r="G60" s="137"/>
-      <c r="H60" s="120" t="s">
+      <c r="B60" s="186"/>
+      <c r="C60" s="189"/>
+      <c r="D60" s="192"/>
+      <c r="E60" s="221"/>
+      <c r="F60" s="230"/>
+      <c r="G60" s="221"/>
+      <c r="H60" s="123" t="s">
         <v>28</v>
       </c>
       <c r="I60" s="36">
@@ -5860,138 +5943,138 @@
       <c r="S60" s="22"/>
       <c r="T60" s="20"/>
       <c r="U60" s="22"/>
-      <c r="V60" s="103"/>
-      <c r="W60" s="103"/>
+      <c r="V60" s="102"/>
+      <c r="W60" s="102"/>
       <c r="X60" s="20"/>
     </row>
     <row r="61" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B61" s="147" t="s">
+      <c r="B61" s="185" t="s">
         <v>75</v>
       </c>
-      <c r="C61" s="146" t="s">
+      <c r="C61" s="213" t="s">
         <v>76</v>
       </c>
-      <c r="D61" s="153" t="s">
+      <c r="D61" s="148" t="s">
         <v>39</v>
       </c>
-      <c r="E61" s="154">
+      <c r="E61" s="218">
         <f>L61+P61+T61+X61</f>
         <v>30.187825999999998</v>
       </c>
-      <c r="F61" s="139">
+      <c r="F61" s="232">
         <f>SUM(L62,P62,T62,X62)</f>
         <v>28</v>
       </c>
-      <c r="G61" s="131">
+      <c r="G61" s="227">
         <f>L63+P63+T63+X63</f>
-        <v>14.112583999999998</v>
-      </c>
-      <c r="H61" s="120" t="s">
+        <v>16.622583999999996</v>
+      </c>
+      <c r="H61" s="123" t="s">
         <v>26</v>
       </c>
-      <c r="I61" s="70">
+      <c r="I61" s="69">
         <v>1.7</v>
       </c>
-      <c r="J61" s="70">
+      <c r="J61" s="69">
         <v>2.5150000000000001</v>
       </c>
-      <c r="K61" s="70">
+      <c r="K61" s="69">
         <v>2.2999999999999998</v>
       </c>
-      <c r="L61" s="71">
+      <c r="L61" s="70">
         <f>K61+J61+I61</f>
         <v>6.5149999999999997</v>
       </c>
-      <c r="M61" s="70">
+      <c r="M61" s="69">
         <v>2.8</v>
       </c>
-      <c r="N61" s="70">
+      <c r="N61" s="69">
         <v>2.2000000000000002</v>
       </c>
-      <c r="O61" s="70">
+      <c r="O61" s="69">
         <v>2.972826</v>
       </c>
-      <c r="P61" s="71">
+      <c r="P61" s="70">
         <f>O61+N61+M61</f>
         <v>7.9728260000000004</v>
       </c>
-      <c r="Q61" s="70">
+      <c r="Q61" s="69">
         <v>2</v>
       </c>
-      <c r="R61" s="70">
+      <c r="R61" s="69">
         <v>2.2999999999999998</v>
       </c>
-      <c r="S61" s="70">
+      <c r="S61" s="69">
         <v>2.7</v>
       </c>
-      <c r="T61" s="71">
+      <c r="T61" s="70">
         <f>S61+R61+Q61</f>
         <v>7</v>
       </c>
-      <c r="U61" s="70">
+      <c r="U61" s="69">
         <v>3.1</v>
       </c>
-      <c r="V61" s="70">
+      <c r="V61" s="69">
         <v>2.6</v>
       </c>
-      <c r="W61" s="70">
+      <c r="W61" s="69">
         <v>3.04</v>
       </c>
-      <c r="X61" s="71">
+      <c r="X61" s="70">
         <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="62" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B62" s="148"/>
-      <c r="C62" s="146"/>
-      <c r="D62" s="153"/>
-      <c r="E62" s="154"/>
-      <c r="F62" s="139"/>
-      <c r="G62" s="131"/>
-      <c r="H62" s="120" t="s">
+      <c r="B62" s="186"/>
+      <c r="C62" s="213"/>
+      <c r="D62" s="148"/>
+      <c r="E62" s="218"/>
+      <c r="F62" s="232"/>
+      <c r="G62" s="227"/>
+      <c r="H62" s="123" t="s">
         <v>27</v>
       </c>
-      <c r="I62" s="130" t="s">
-        <v>32</v>
-      </c>
-      <c r="J62" s="130"/>
-      <c r="K62" s="130"/>
-      <c r="L62" s="71">
+      <c r="I62" s="133" t="s">
+        <v>32</v>
+      </c>
+      <c r="J62" s="133"/>
+      <c r="K62" s="133"/>
+      <c r="L62" s="70">
         <v>5</v>
       </c>
-      <c r="M62" s="130" t="s">
-        <v>32</v>
-      </c>
-      <c r="N62" s="130"/>
-      <c r="O62" s="130"/>
-      <c r="P62" s="71">
+      <c r="M62" s="133" t="s">
+        <v>32</v>
+      </c>
+      <c r="N62" s="133"/>
+      <c r="O62" s="133"/>
+      <c r="P62" s="70">
         <v>7</v>
       </c>
-      <c r="Q62" s="130" t="s">
-        <v>32</v>
-      </c>
-      <c r="R62" s="130"/>
-      <c r="S62" s="130"/>
-      <c r="T62" s="71">
+      <c r="Q62" s="133" t="s">
+        <v>32</v>
+      </c>
+      <c r="R62" s="133"/>
+      <c r="S62" s="133"/>
+      <c r="T62" s="70">
         <v>7</v>
       </c>
-      <c r="U62" s="71" t="s">
+      <c r="U62" s="70" t="s">
         <v>32</v>
       </c>
       <c r="V62" s="119"/>
       <c r="W62" s="119"/>
-      <c r="X62" s="71">
+      <c r="X62" s="70">
         <v>9</v>
       </c>
     </row>
     <row r="63" spans="2:25" ht="18.75" customHeight="1">
-      <c r="B63" s="148"/>
-      <c r="C63" s="146"/>
-      <c r="D63" s="153"/>
-      <c r="E63" s="154"/>
-      <c r="F63" s="139"/>
-      <c r="G63" s="131"/>
-      <c r="H63" s="120" t="s">
+      <c r="B63" s="186"/>
+      <c r="C63" s="213"/>
+      <c r="D63" s="148"/>
+      <c r="E63" s="218"/>
+      <c r="F63" s="232"/>
+      <c r="G63" s="227"/>
+      <c r="H63" s="123" t="s">
         <v>28</v>
       </c>
       <c r="I63" s="119">
@@ -6003,7 +6086,7 @@
       <c r="K63" s="119">
         <v>2.5</v>
       </c>
-      <c r="L63" s="91">
+      <c r="L63" s="90">
         <f>K63+J63+I63</f>
         <v>5.2329999999999997</v>
       </c>
@@ -6016,23 +6099,25 @@
       <c r="O63" s="119">
         <v>1.86</v>
       </c>
-      <c r="P63" s="113">
+      <c r="P63" s="112">
         <f>O63+N63+M63</f>
         <v>6.6172839999999997</v>
       </c>
       <c r="Q63" s="119">
         <v>2.2623000000000002</v>
       </c>
-      <c r="R63" s="119"/>
+      <c r="R63" s="119">
+        <v>2.5099999999999998</v>
+      </c>
       <c r="S63" s="119"/>
-      <c r="T63" s="92">
+      <c r="T63" s="91">
         <f>S63+R63+Q63</f>
-        <v>2.2623000000000002</v>
+        <v>4.7722999999999995</v>
       </c>
       <c r="U63" s="119"/>
       <c r="V63" s="119"/>
       <c r="W63" s="119"/>
-      <c r="X63" s="92">
+      <c r="X63" s="91">
         <f>W63+V63+U63</f>
         <v>0</v>
       </c>
@@ -6040,386 +6125,390 @@
         <v>77</v>
       </c>
     </row>
-    <row r="64" spans="2:25" ht="15.6">
-      <c r="B64" s="148"/>
-      <c r="C64" s="140" t="s">
+    <row r="64" spans="2:25" ht="16.5">
+      <c r="B64" s="186"/>
+      <c r="C64" s="209" t="s">
         <v>78</v>
       </c>
-      <c r="D64" s="141" t="s">
+      <c r="D64" s="210" t="s">
         <v>79</v>
       </c>
-      <c r="E64" s="142">
+      <c r="E64" s="211">
         <f>L64+P64+T64+X64</f>
         <v>-8.4644727175232077</v>
       </c>
-      <c r="F64" s="138">
+      <c r="F64" s="231">
         <f>SUM(L65,P65,T65,X65)</f>
         <v>-7.0189285867816498</v>
       </c>
-      <c r="G64" s="129">
+      <c r="G64" s="226">
         <f>SUM(L66,P66,T66,Q66,X66)</f>
-        <v>-5.8522190000397307</v>
-      </c>
-      <c r="H64" s="122" t="s">
+        <v>-6.3300698065453469</v>
+      </c>
+      <c r="H64" s="120" t="s">
         <v>26</v>
       </c>
-      <c r="I64" s="72">
+      <c r="I64" s="71">
         <v>-0.5</v>
       </c>
-      <c r="J64" s="72">
+      <c r="J64" s="71">
         <v>-0.5</v>
       </c>
-      <c r="K64" s="72">
+      <c r="K64" s="71">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="L64" s="73">
+      <c r="L64" s="72">
         <f t="shared" ref="L64:L69" si="8">SUM(I64:K64)</f>
         <v>-2.1</v>
       </c>
-      <c r="M64" s="72">
+      <c r="M64" s="71">
         <v>-0.5</v>
       </c>
-      <c r="N64" s="72">
+      <c r="N64" s="71">
         <v>0.1</v>
       </c>
-      <c r="O64" s="72">
+      <c r="O64" s="71">
         <v>-1.5</v>
       </c>
-      <c r="P64" s="73">
+      <c r="P64" s="72">
         <f t="shared" ref="P64:P69" si="9">SUM(M64:O64)</f>
         <v>-1.9</v>
       </c>
-      <c r="Q64" s="72">
+      <c r="Q64" s="71">
         <v>-0.9</v>
       </c>
-      <c r="R64" s="72">
+      <c r="R64" s="71">
         <v>-0.83660522126404935</v>
       </c>
-      <c r="S64" s="72">
+      <c r="S64" s="71">
         <v>-0.41</v>
       </c>
-      <c r="T64" s="73">
+      <c r="T64" s="72">
         <f t="shared" ref="T64:T69" si="10">SUM(Q64:S64)</f>
         <v>-2.1466052212640494</v>
       </c>
-      <c r="U64" s="72">
+      <c r="U64" s="71">
         <v>-0.48</v>
       </c>
-      <c r="V64" s="72">
+      <c r="V64" s="71">
         <v>-0.34</v>
       </c>
-      <c r="W64" s="72">
+      <c r="W64" s="71">
         <v>-1.4978674962591589</v>
       </c>
-      <c r="X64" s="73">
+      <c r="X64" s="72">
         <f t="shared" ref="X64:X69" si="11">SUM(U64:W64)</f>
         <v>-2.3178674962591588</v>
       </c>
     </row>
     <row r="65" spans="2:24" ht="15.6">
-      <c r="B65" s="148"/>
-      <c r="C65" s="140"/>
-      <c r="D65" s="141"/>
-      <c r="E65" s="142"/>
-      <c r="F65" s="138"/>
-      <c r="G65" s="129"/>
-      <c r="H65" s="122" t="s">
+      <c r="B65" s="186"/>
+      <c r="C65" s="209"/>
+      <c r="D65" s="210"/>
+      <c r="E65" s="211"/>
+      <c r="F65" s="231"/>
+      <c r="G65" s="226"/>
+      <c r="H65" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="I65" s="72">
+      <c r="I65" s="71">
         <v>-0.6</v>
       </c>
-      <c r="J65" s="72">
+      <c r="J65" s="71">
         <v>-0.5</v>
       </c>
-      <c r="K65" s="72">
+      <c r="K65" s="71">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="L65" s="73">
+      <c r="L65" s="72">
         <f t="shared" si="8"/>
         <v>-2.2000000000000002</v>
       </c>
-      <c r="M65" s="72">
+      <c r="M65" s="71">
         <v>-0.8</v>
       </c>
-      <c r="N65" s="72">
+      <c r="N65" s="71">
         <v>-0.5</v>
       </c>
-      <c r="O65" s="72">
+      <c r="O65" s="71">
         <v>-0.7</v>
       </c>
-      <c r="P65" s="73">
+      <c r="P65" s="72">
         <f t="shared" si="9"/>
         <v>-2</v>
       </c>
-      <c r="Q65" s="72">
+      <c r="Q65" s="71">
         <v>-0.4710695833326044</v>
       </c>
-      <c r="R65" s="72">
+      <c r="R65" s="71">
         <v>-0.47785080650561662</v>
       </c>
-      <c r="S65" s="72">
+      <c r="S65" s="71">
         <v>-0.56812301870144577</v>
       </c>
-      <c r="T65" s="73">
+      <c r="T65" s="72">
         <f t="shared" si="10"/>
         <v>-1.5170434085396667</v>
       </c>
-      <c r="U65" s="72">
+      <c r="U65" s="71">
         <v>-0.32641448602076573</v>
       </c>
-      <c r="V65" s="72">
+      <c r="V65" s="71">
         <v>-0.37253694072630583</v>
       </c>
-      <c r="W65" s="72">
+      <c r="W65" s="71">
         <v>-0.60293375149491213</v>
       </c>
-      <c r="X65" s="73">
+      <c r="X65" s="72">
         <f t="shared" si="11"/>
         <v>-1.3018851782419838</v>
       </c>
     </row>
-    <row r="66" spans="2:24" ht="15.6">
-      <c r="B66" s="148"/>
-      <c r="C66" s="140"/>
-      <c r="D66" s="141"/>
-      <c r="E66" s="142"/>
-      <c r="F66" s="138"/>
-      <c r="G66" s="129"/>
-      <c r="H66" s="122" t="s">
+    <row r="66" spans="2:24" ht="16.5">
+      <c r="B66" s="186"/>
+      <c r="C66" s="209"/>
+      <c r="D66" s="210"/>
+      <c r="E66" s="211"/>
+      <c r="F66" s="231"/>
+      <c r="G66" s="226"/>
+      <c r="H66" s="120" t="s">
         <v>28</v>
       </c>
-      <c r="I66" s="82">
+      <c r="I66" s="81">
         <v>-0.8</v>
       </c>
-      <c r="J66" s="82">
+      <c r="J66" s="81">
         <v>-0.8</v>
       </c>
-      <c r="K66" s="89">
+      <c r="K66" s="88">
         <v>-0.5</v>
       </c>
-      <c r="L66" s="97">
+      <c r="L66" s="96">
         <f t="shared" si="8"/>
         <v>-2.1</v>
       </c>
-      <c r="M66" s="89">
+      <c r="M66" s="88">
         <v>-0.6</v>
       </c>
-      <c r="N66" s="82">
+      <c r="N66" s="81">
         <v>-0.9</v>
       </c>
-      <c r="O66" s="89">
+      <c r="O66" s="88">
         <v>-0.27622289841125025</v>
       </c>
-      <c r="P66" s="97">
+      <c r="P66" s="96">
         <f>SUM(M66:O66)</f>
         <v>-1.7762228984112503</v>
       </c>
-      <c r="Q66" s="82">
+      <c r="Q66" s="81">
         <v>-0.98799805081423986</v>
       </c>
-      <c r="R66" s="72"/>
-      <c r="S66" s="72"/>
-      <c r="T66" s="111">
+      <c r="R66" s="235">
+        <v>-0.47785080650561662</v>
+      </c>
+      <c r="S66" s="71"/>
+      <c r="T66" s="110">
         <f t="shared" si="10"/>
-        <v>-0.98799805081423986</v>
-      </c>
-      <c r="U66" s="72"/>
-      <c r="V66" s="72"/>
-      <c r="W66" s="72"/>
-      <c r="X66" s="111">
+        <v>-1.4658488573198565</v>
+      </c>
+      <c r="U66" s="71"/>
+      <c r="V66" s="71"/>
+      <c r="W66" s="71"/>
+      <c r="X66" s="110">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
     <row r="67" spans="2:24" ht="15" customHeight="1">
-      <c r="B67" s="148"/>
-      <c r="C67" s="150" t="s">
+      <c r="B67" s="186"/>
+      <c r="C67" s="215" t="s">
         <v>80</v>
       </c>
-      <c r="D67" s="151" t="s">
+      <c r="D67" s="216" t="s">
         <v>79</v>
       </c>
-      <c r="E67" s="152">
+      <c r="E67" s="217">
         <f>L67+P67+T67+X67</f>
         <v>-20.34262829557931</v>
       </c>
-      <c r="F67" s="125">
+      <c r="F67" s="222">
         <f>SUM(L68,P68,T68,X68)</f>
         <v>-24.141371751369434</v>
       </c>
-      <c r="G67" s="128">
+      <c r="G67" s="225">
         <f>SUM(L69,P69,T69,X69)</f>
-        <v>-14.40318635548517</v>
-      </c>
-      <c r="H67" s="123" t="s">
+        <v>-16.595412480713406</v>
+      </c>
+      <c r="H67" s="122" t="s">
         <v>26</v>
       </c>
-      <c r="I67" s="74">
+      <c r="I67" s="73">
         <v>-1.3</v>
       </c>
-      <c r="J67" s="74">
+      <c r="J67" s="73">
         <v>-1.8</v>
       </c>
-      <c r="K67" s="74">
+      <c r="K67" s="73">
         <v>-1.2</v>
       </c>
-      <c r="L67" s="75">
+      <c r="L67" s="74">
         <f t="shared" si="8"/>
         <v>-4.3</v>
       </c>
-      <c r="M67" s="74">
+      <c r="M67" s="73">
         <v>-1.6</v>
       </c>
-      <c r="N67" s="74">
+      <c r="N67" s="73">
         <v>-1.4</v>
       </c>
-      <c r="O67" s="74">
+      <c r="O67" s="73">
         <v>-1.5</v>
       </c>
-      <c r="P67" s="75">
+      <c r="P67" s="74">
         <f t="shared" si="9"/>
         <v>-4.5</v>
       </c>
-      <c r="Q67" s="74">
+      <c r="Q67" s="73">
         <v>-1.91</v>
       </c>
-      <c r="R67" s="74">
+      <c r="R67" s="73">
         <v>-2.3939222677777598</v>
       </c>
-      <c r="S67" s="74">
+      <c r="S67" s="73">
         <v>-2.1</v>
       </c>
-      <c r="T67" s="75">
+      <c r="T67" s="74">
         <f t="shared" si="10"/>
         <v>-6.4039222677777605</v>
       </c>
-      <c r="U67" s="74">
+      <c r="U67" s="73">
         <v>-1.71</v>
       </c>
-      <c r="V67" s="74">
+      <c r="V67" s="73">
         <v>-1.76033753077637</v>
       </c>
-      <c r="W67" s="74">
+      <c r="W67" s="73">
         <v>-1.66836849702518</v>
       </c>
-      <c r="X67" s="75">
+      <c r="X67" s="74">
         <f t="shared" si="11"/>
         <v>-5.1387060278015504</v>
       </c>
     </row>
     <row r="68" spans="2:24" ht="15" customHeight="1">
-      <c r="B68" s="148"/>
-      <c r="C68" s="150"/>
-      <c r="D68" s="151"/>
-      <c r="E68" s="152"/>
-      <c r="F68" s="126"/>
-      <c r="G68" s="128"/>
-      <c r="H68" s="123" t="s">
+      <c r="B68" s="186"/>
+      <c r="C68" s="215"/>
+      <c r="D68" s="216"/>
+      <c r="E68" s="217"/>
+      <c r="F68" s="223"/>
+      <c r="G68" s="225"/>
+      <c r="H68" s="122" t="s">
         <v>27</v>
       </c>
-      <c r="I68" s="74">
+      <c r="I68" s="73">
         <v>-2.1</v>
       </c>
-      <c r="J68" s="74">
+      <c r="J68" s="73">
         <v>-2.1</v>
       </c>
-      <c r="K68" s="74">
+      <c r="K68" s="73">
         <v>-2.1</v>
       </c>
-      <c r="L68" s="75">
+      <c r="L68" s="74">
         <f t="shared" si="8"/>
         <v>-6.3000000000000007</v>
       </c>
-      <c r="M68" s="74">
+      <c r="M68" s="73">
         <v>-1.7</v>
       </c>
-      <c r="N68" s="74">
+      <c r="N68" s="73">
         <v>-1.7</v>
       </c>
-      <c r="O68" s="74">
+      <c r="O68" s="73">
         <v>-1.7</v>
       </c>
-      <c r="P68" s="75">
+      <c r="P68" s="74">
         <f t="shared" si="9"/>
         <v>-5.0999999999999996</v>
       </c>
-      <c r="Q68" s="74">
+      <c r="Q68" s="73">
         <v>-2.1922261252282387</v>
       </c>
-      <c r="R68" s="74">
+      <c r="R68" s="73">
         <v>-2.1922261252282387</v>
       </c>
-      <c r="S68" s="74">
+      <c r="S68" s="73">
         <v>-2.1922261252282387</v>
       </c>
-      <c r="T68" s="75">
+      <c r="T68" s="74">
         <f t="shared" si="10"/>
         <v>-6.5766783756847165</v>
       </c>
-      <c r="U68" s="74">
+      <c r="U68" s="73">
         <v>-2.0548977918949052</v>
       </c>
-      <c r="V68" s="74">
+      <c r="V68" s="73">
         <v>-2.0548977918949052</v>
       </c>
-      <c r="W68" s="74">
+      <c r="W68" s="73">
         <v>-2.0548977918949052</v>
       </c>
-      <c r="X68" s="75">
+      <c r="X68" s="74">
         <f t="shared" si="11"/>
         <v>-6.1646933756847151</v>
       </c>
     </row>
     <row r="69" spans="2:24" ht="15" customHeight="1">
-      <c r="B69" s="149"/>
-      <c r="C69" s="150"/>
-      <c r="D69" s="151"/>
-      <c r="E69" s="152"/>
-      <c r="F69" s="127"/>
-      <c r="G69" s="128"/>
-      <c r="H69" s="123" t="s">
+      <c r="B69" s="214"/>
+      <c r="C69" s="215"/>
+      <c r="D69" s="216"/>
+      <c r="E69" s="217"/>
+      <c r="F69" s="224"/>
+      <c r="G69" s="225"/>
+      <c r="H69" s="122" t="s">
         <v>28</v>
       </c>
-      <c r="I69" s="89">
+      <c r="I69" s="88">
         <v>-0.9</v>
       </c>
-      <c r="J69" s="89">
+      <c r="J69" s="88">
         <v>-2</v>
       </c>
-      <c r="K69" s="89">
+      <c r="K69" s="88">
         <v>-2.1</v>
       </c>
-      <c r="L69" s="97">
+      <c r="L69" s="96">
         <f t="shared" si="8"/>
         <v>-5</v>
       </c>
-      <c r="M69" s="89">
+      <c r="M69" s="88">
         <v>-0.3</v>
       </c>
-      <c r="N69" s="82">
+      <c r="N69" s="81">
         <v>-4.9000000000000004</v>
       </c>
-      <c r="O69" s="89">
+      <c r="O69" s="88">
         <v>-1.4</v>
       </c>
-      <c r="P69" s="115">
+      <c r="P69" s="114">
         <f t="shared" si="9"/>
         <v>-6.6</v>
       </c>
-      <c r="Q69" s="82">
+      <c r="Q69" s="81">
         <v>-2.8031863554851699</v>
       </c>
-      <c r="R69" s="74"/>
-      <c r="S69" s="74"/>
-      <c r="T69" s="112">
+      <c r="R69" s="235">
+        <v>-2.1922261252282387</v>
+      </c>
+      <c r="S69" s="73"/>
+      <c r="T69" s="111">
         <f t="shared" si="10"/>
-        <v>-2.8031863554851699</v>
-      </c>
-      <c r="U69" s="74"/>
-      <c r="V69" s="74"/>
-      <c r="W69" s="74"/>
-      <c r="X69" s="112">
+        <v>-4.9954124807134086</v>
+      </c>
+      <c r="U69" s="73"/>
+      <c r="V69" s="73"/>
+      <c r="W69" s="73"/>
+      <c r="X69" s="111">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -6438,6 +6527,109 @@
     </row>
   </sheetData>
   <mergeCells count="127">
+    <mergeCell ref="F67:F69"/>
+    <mergeCell ref="G67:G69"/>
+    <mergeCell ref="G64:G66"/>
+    <mergeCell ref="M62:O62"/>
+    <mergeCell ref="Q62:S62"/>
+    <mergeCell ref="G61:G63"/>
+    <mergeCell ref="F58:F60"/>
+    <mergeCell ref="G58:G60"/>
+    <mergeCell ref="I62:K62"/>
+    <mergeCell ref="F64:F66"/>
+    <mergeCell ref="F61:F63"/>
+    <mergeCell ref="C64:C66"/>
+    <mergeCell ref="D64:D66"/>
+    <mergeCell ref="E64:E66"/>
+    <mergeCell ref="C55:C57"/>
+    <mergeCell ref="D55:D57"/>
+    <mergeCell ref="E55:E57"/>
+    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="B61:B69"/>
+    <mergeCell ref="C67:C69"/>
+    <mergeCell ref="D67:D69"/>
+    <mergeCell ref="E67:E69"/>
+    <mergeCell ref="D61:D63"/>
+    <mergeCell ref="E61:E63"/>
+    <mergeCell ref="E58:E60"/>
+    <mergeCell ref="G13:G15"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="C58:C60"/>
+    <mergeCell ref="D58:D60"/>
+    <mergeCell ref="B19:B33"/>
+    <mergeCell ref="C34:C36"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="B34:B57"/>
+    <mergeCell ref="F55:F57"/>
+    <mergeCell ref="F49:F51"/>
+    <mergeCell ref="C52:C54"/>
+    <mergeCell ref="D52:D54"/>
+    <mergeCell ref="E52:E54"/>
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="D25:D27"/>
+    <mergeCell ref="E25:E27"/>
+    <mergeCell ref="F25:F27"/>
+    <mergeCell ref="G25:G27"/>
+    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="D40:D42"/>
+    <mergeCell ref="E40:E42"/>
+    <mergeCell ref="B4:B18"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="I2:X2"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="D49:D51"/>
+    <mergeCell ref="E49:E51"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="E31:E33"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="G4:G6"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="F10:F12"/>
+    <mergeCell ref="G10:G12"/>
+    <mergeCell ref="F7:F9"/>
+    <mergeCell ref="G31:G33"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="G7:G9"/>
+    <mergeCell ref="G34:G36"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="F13:F15"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="D22:D24"/>
+    <mergeCell ref="E22:E24"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="D28:D30"/>
+    <mergeCell ref="E28:E30"/>
+    <mergeCell ref="M56:O56"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="Q56:S56"/>
+    <mergeCell ref="U56:W56"/>
+    <mergeCell ref="M53:O53"/>
+    <mergeCell ref="Q53:S53"/>
+    <mergeCell ref="U53:W53"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="F34:F36"/>
+    <mergeCell ref="F52:F54"/>
+    <mergeCell ref="G52:G54"/>
+    <mergeCell ref="F40:F42"/>
+    <mergeCell ref="G40:G42"/>
+    <mergeCell ref="E43:E45"/>
+    <mergeCell ref="F43:F45"/>
+    <mergeCell ref="G43:G45"/>
+    <mergeCell ref="E37:E39"/>
+    <mergeCell ref="F37:F39"/>
+    <mergeCell ref="G37:G39"/>
     <mergeCell ref="G19:G21"/>
     <mergeCell ref="E16:E18"/>
     <mergeCell ref="C16:C18"/>
@@ -6462,109 +6654,6 @@
     <mergeCell ref="E46:E48"/>
     <mergeCell ref="F46:F48"/>
     <mergeCell ref="G46:G48"/>
-    <mergeCell ref="M56:O56"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="Q56:S56"/>
-    <mergeCell ref="U56:W56"/>
-    <mergeCell ref="M53:O53"/>
-    <mergeCell ref="Q53:S53"/>
-    <mergeCell ref="U53:W53"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="F34:F36"/>
-    <mergeCell ref="F52:F54"/>
-    <mergeCell ref="G52:G54"/>
-    <mergeCell ref="F40:F42"/>
-    <mergeCell ref="G40:G42"/>
-    <mergeCell ref="E43:E45"/>
-    <mergeCell ref="F43:F45"/>
-    <mergeCell ref="G43:G45"/>
-    <mergeCell ref="E37:E39"/>
-    <mergeCell ref="F37:F39"/>
-    <mergeCell ref="G37:G39"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="E10:E12"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="D22:D24"/>
-    <mergeCell ref="E22:E24"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="D28:D30"/>
-    <mergeCell ref="E28:E30"/>
-    <mergeCell ref="I2:X2"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="D49:D51"/>
-    <mergeCell ref="E49:E51"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="D31:D33"/>
-    <mergeCell ref="E31:E33"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="D16:D18"/>
-    <mergeCell ref="G4:G6"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="F10:F12"/>
-    <mergeCell ref="G10:G12"/>
-    <mergeCell ref="F7:F9"/>
-    <mergeCell ref="G31:G33"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="F16:F18"/>
-    <mergeCell ref="G7:G9"/>
-    <mergeCell ref="G34:G36"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="F13:F15"/>
-    <mergeCell ref="G13:G15"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="C58:C60"/>
-    <mergeCell ref="D58:D60"/>
-    <mergeCell ref="B19:B33"/>
-    <mergeCell ref="C34:C36"/>
-    <mergeCell ref="D34:D36"/>
-    <mergeCell ref="B34:B57"/>
-    <mergeCell ref="F55:F57"/>
-    <mergeCell ref="F49:F51"/>
-    <mergeCell ref="C52:C54"/>
-    <mergeCell ref="D52:D54"/>
-    <mergeCell ref="E52:E54"/>
-    <mergeCell ref="C25:C27"/>
-    <mergeCell ref="D25:D27"/>
-    <mergeCell ref="E25:E27"/>
-    <mergeCell ref="F25:F27"/>
-    <mergeCell ref="G25:G27"/>
-    <mergeCell ref="C40:C42"/>
-    <mergeCell ref="D40:D42"/>
-    <mergeCell ref="E40:E42"/>
-    <mergeCell ref="B4:B18"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="C64:C66"/>
-    <mergeCell ref="D64:D66"/>
-    <mergeCell ref="E64:E66"/>
-    <mergeCell ref="C55:C57"/>
-    <mergeCell ref="D55:D57"/>
-    <mergeCell ref="E55:E57"/>
-    <mergeCell ref="C61:C63"/>
-    <mergeCell ref="B61:B69"/>
-    <mergeCell ref="C67:C69"/>
-    <mergeCell ref="D67:D69"/>
-    <mergeCell ref="E67:E69"/>
-    <mergeCell ref="D61:D63"/>
-    <mergeCell ref="E61:E63"/>
-    <mergeCell ref="E58:E60"/>
-    <mergeCell ref="F67:F69"/>
-    <mergeCell ref="G67:G69"/>
-    <mergeCell ref="G64:G66"/>
-    <mergeCell ref="M62:O62"/>
-    <mergeCell ref="Q62:S62"/>
-    <mergeCell ref="G61:G63"/>
-    <mergeCell ref="F58:F60"/>
-    <mergeCell ref="G58:G60"/>
-    <mergeCell ref="I62:K62"/>
-    <mergeCell ref="F64:F66"/>
-    <mergeCell ref="F61:F63"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6616,10 +6705,10 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="62" t="s">
+      <c r="A6" s="61" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="61" t="s">
         <v>90</v>
       </c>
     </row>
@@ -6632,20 +6721,20 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.6">
-      <c r="A8" s="64" t="s">
+      <c r="A8" s="63" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="64"/>
+      <c r="B8" s="63"/>
       <c r="C8" s="30"/>
       <c r="D8" s="30"/>
       <c r="E8" s="30"/>
       <c r="F8" s="30"/>
     </row>
     <row r="9" spans="1:6" ht="15.6">
-      <c r="A9" s="64" t="s">
+      <c r="A9" s="63" t="s">
         <v>94</v>
       </c>
-      <c r="B9" s="64"/>
+      <c r="B9" s="63"/>
       <c r="C9" s="30"/>
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
@@ -6676,13 +6765,13 @@
       <c r="F11" s="30"/>
     </row>
     <row r="12" spans="1:6" ht="15.6">
-      <c r="A12" s="62" t="s">
+      <c r="A12" s="61" t="s">
         <v>99</v>
       </c>
       <c r="C12" s="30"/>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="62" t="s">
+      <c r="A13" s="61" t="s">
         <v>100</v>
       </c>
     </row>

</xml_diff>